<commit_message>
feat(etf): split daily it/etf downloads; grow universe to 346 (extra_count=350)
Two changes:

1. Split the daily download into independent matrix legs (fail-fast: false),
   one per market. An etf download failure no longer blocks the it update (or
   vice versa) — each leg commits only its own market's Parquet files. The two
   legs run in parallel and push to the same branch, so the commit step
   rebase-retries on a rejected push (disjoint files => no conflict).

2. Raise DEFAULT_EXTRA_COUNT 250 -> 350, growing the active universe by ~100 to
   346 tickers (15 core + 331 extras; 19 known-dead pruned). Historical backfill
   for the new tickers is run separately via the cold-start workflow at the same
   2016-01-01 -> today range.
</commit_message>
<xml_diff>
--- a/data/ticker/etf/ticker_active.xlsx
+++ b/data/ticker/etf/ticker_active.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B247"/>
+  <dimension ref="A1:B347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3380,6 +3380,1206 @@
         </is>
       </c>
     </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Amundi Prime Europe UCITS ETF DR (C)</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>PRAE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Amundi Prime Europe UCITS ETF DR (D)</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>ETFEU.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Amundi Prime Eurozone UCITS ETF DR (C)</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>PRAZ.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Amundi Prime Eurozone UCITS ETF DR (D)</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>ETFEZ.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Amundi Prime Global UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>ETFGLO.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Amundi Prime Japan UCITS ETF DR (C)</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>PRAJ.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Amundi Prime Japan UCITS ETF DR (D)</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>ETFJAP.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Amundi Russell 1000 Growth UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>MWOT.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P 500 Buyback UCITS ETF EUR (C)</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>BYBE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P 500 Equal Weight ESG UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>WELE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P 500 Equal Weight ESG UCITS ETF EUR Hedged Acc</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>MWOQ.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P 500 Equal Weight UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>EQSU.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P 500 Screened UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>U500.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P 500 Screened UCITS ETF Acc EUR Hedged</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>S500H.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P 500 Swap UCITS ETF EUR Acc</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>500.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P 500 Swap UCITS ETF EUR Hedged Acc</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>500H.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P 500 Swap UCITS ETF USD Acc</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>500E.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P 500 Swap UCITS ETF USD Dist</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>500D.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Eurozone Dividend Aristocrat Screened UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>EUDIV.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Global Communication Services ESG UCITS ETF DR EUR (A)</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>TELW.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Global Consumer Discretionary ESG UCITS ETF DR EUR (A)</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>CODW.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Global Consumer Staples ESG UCITS ETF DR EUR (A)</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>COSW.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Global Energy Carbon Reduced UCITS ETF DR EUR (A)</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>NRGW.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Global Financials ESG UCITS ETF DR EUR (A)</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>GLFI.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Global Health Care ESG UCITS ETF DR EUR (A)</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>GLHL.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Global Industrials ESG UCITS ETF DR EUR (A)</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>INDW.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Global Information Technology ESG UCITS ETF DR EUR (A)</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>GLIT.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Global Materials ESG UCITS ETF DR EUR (A)</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>MATW.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Global Utilities ESG UCITS ETF DR EUR (A)</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>UTIW.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Amundi STOXX Europe 600 Banks UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>BNK.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Amundi STOXX Europe 600 Basic Materials UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>CHM.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Amundi STOXX Europe 600 Basic Resources UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>BRES.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Amundi STOXX Europe 600 Consumer Discretionary UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>TRV.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Amundi STOXX Europe 600 Consumer Staples UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>FOO.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Amundi STOXX Europe 600 Healthcare UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>HLT.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Amundi STOXX Europe 600 Telecommunications UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>TELE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Amundi STOXX Europe 600 Utilities UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>UTI.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Amundi ShortDAX Daily (-1x) Inverse UCITS ETF - Dist</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>AHYK.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Amundi ShortDAX Daily (-2x) Inverse UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>DSD.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Amundi Smart Overnight Return UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>CSH2.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Amundi Smart Overnight Return UCITS ETF CHF Hedged Acc</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>SMCH.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Amundi Smart Overnight Return UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>SMOR.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Amundi Smart Overnight Return UCITS ETF GBP Hedged Acc</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>LYSMG.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Amundi Smart Overnight Return UCITS ETF USD Hedged Acc</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>SMARTU.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Amundi Stoxx Europe 50 UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>C5E.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Amundi Stoxx Europe Select Dividend 30 UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>SEL.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Amundi US Curve steepening 2-10Y UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>STPU.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Amundi US Curve steepening 2-10Y UCITS ETF GBP Hedged Dist</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>STPH.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Amundi US Tech 100 Equal Weight UCITS ETF DR USD D</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>UTEC.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Amundi USD Corporate Bond Climate Paris Aligned UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>USIC.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Amundi USD Corporate Bond Climate Paris Aligned UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>USIG.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Amundi USD Corporate Bond Climate Paris Aligned UCITS ETF EUR Hedged Dist</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>USIH.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Amundi USD Fed Funds Rate UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>FEDF.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Amundi USD Fed Funds Rate UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>CBFEDF.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Amundi USD High Yield Corporate Bond ESG UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>USHYC.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Amundi USD High Yield Corporate Bond ESG UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>USHY.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Amundi USD High Yield Corporate Bond ESG UCITS ETF EUR HEDGED Dist</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>USYH.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Avantis America Equity UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>AVAE.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Avantis Emerging Markets Equity UCITS ETF USD Acc</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>AVEM.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Avantis Europe Equity UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>AVUE.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Avantis Global Equity UCITS ETF USD Acc</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>AVCG.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Avantis Global Small Cap Value UCITS ETF USD Acc</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>AVSG.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Avantis Pacific Equity UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>AVEP.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy Alpha Enhanced EUR Corporate Bond UCITS ETF (Acc)</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>QEIG.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy Alpha Enhanced Europe UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>QEUR.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy Alpha Enhanced Global High Yield UCITS ETF (Acc)</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>QGHY.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy Alpha Enhanced US UCITS ETF EUR Acc</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>QUSAE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy Alpha Enhanced US UCITS ETF USD Acc</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>QUSA.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy Alpha Enhanced USD Corporate Bond UCITS ETF (Acc)</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>QUIG.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy Alpha Enhanced World UCITS ETF EUR Acc</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>QGLOE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy Alpha Enhanced World UCITS ETF USD Acc</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>QGLO.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy Dividend Europe UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>EDEU.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ECPI Global ESG Blue Economy UCITS ETF EUR</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>BLUE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ECPI Global ESG Blue Economy UCITS ETF USD</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>BLUSD.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ECPI Global ESG Infrastructure UCITS ETF EUR Capitalisation</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>ENG.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ECPI Global ESG Infrastructure UCITS ETF USD Capitalisation</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>ENGUS.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced EMU UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>AEMUS.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2027 UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>ACE27.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2027 UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>ACD27.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2029 UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>ACE29.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2029 UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>ACD29.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2032 UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>ACE32.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2032 UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>ACD32.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond UCITS ETF Capitalisation</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>SEUCB.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>ACESD.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced EUR Government Bond UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>SEUGB.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced EUR Government Bond UCITS ETF Distribution</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>AGESD.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced Europe UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>AEUSE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced Japan UCITS ETF EUR Acc</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>AJASE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced Japan UCITS ETF EUR Hedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>AJASH.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced US UCITS ETF EUR Acc</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>AUSSE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced US UCITS ETF EUR Hedged Acc</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>AUSSH.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced US UCITS ETF USD Acc</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>AUSSD.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced World UCITS ETF EUR Acc</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>AWDSE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced World UCITS ETF EUR Hedged Acc</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>AWDSH.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy ESG Enhanced World UCITS ETF USD Acc</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>AWDS.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy EUR Corporate Bond SRI Fossil Free 7-10Y UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>SRIC7.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy EUR Corporate Bond SRI Fossil Free 7-10Y UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>SRID7.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy EUR Corporate Bond SRI Fossil Free Ultrashort Duration UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>SRIUC.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy EUR Corporate Bond SRI Fossil Free Ultrashort Duration UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>SRIUD.PA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(etf): prune 29 dead tickers from the 346-ticker run (active universe -> 317)
The extra_count=350 cold-start backfill downloaded 317/346 symbols over the
same 2016-01-04 -> 2026-07-10 range as the existing tickers (477,506 rows).
29 more justETF extras returned no Yahoo data (mostly crypto ETPs and thin
.PA/.SW listings); fold them into KNOWN_DEAD so the daily job skips them.

Regenerated seed is 317 tickers and matches the committed historical parquet
symbols exactly, so no re-backfill is needed.
</commit_message>
<xml_diff>
--- a/data/ticker/etf/ticker_active.xlsx
+++ b/data/ticker/etf/ticker_active.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B347"/>
+  <dimension ref="A1:B318"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -683,3898 +683,3550 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>21shares Aave ETP</t>
+          <t>21shares Bitcoin Cash ETP</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AAVE.AS</t>
+          <t>ABCH.AS</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>21shares Algorand ETP</t>
+          <t>21shares Bitcoin Core ETP</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ALGO.AS</t>
+          <t>CBTC.AS</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>21shares Avalanche Staking ETP</t>
+          <t>21shares Bitcoin ETP</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AVAX.AS</t>
+          <t>ABTC.AS</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>21shares Binance BNB ETP</t>
+          <t>21shares Bitcoin Ethereum Core ETP</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BNBA.AS</t>
+          <t>ABBA.SW</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>21shares Bitcoin Cash ETP</t>
+          <t>21shares Bitwise Select 10 ETP</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ABCH.AS</t>
+          <t>KEYS.SW</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>21shares Bitcoin Core ETP</t>
+          <t>21shares Cardano ETP</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CBTC.AS</t>
+          <t>AADA.AS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>21shares Bitcoin ETP</t>
+          <t>21shares Crypto Basket 10 Core ETP</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ABTC.AS</t>
+          <t>HODLX.AS</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>21shares Bitcoin Ethereum Core ETP</t>
+          <t>21shares Crypto Basket Equal Weight ETP</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ABBA.SW</t>
+          <t>HODLV.AS</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>21shares Bitcoin Gold ETP</t>
+          <t>21shares Dogecoin ETP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BOLD.AS</t>
+          <t>DOGE.SW</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>21shares Bitwise Select 10 ETP</t>
+          <t>21shares Ethena ETP</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>KEYS.SW</t>
+          <t>EENA.SW</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>21shares Cardano ETP</t>
+          <t>21shares Ethereum Staking ETP</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AADA.AS</t>
+          <t>AETH.AS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>21shares Chainlink ETP</t>
+          <t>21shares Hyperliquid ETP</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ALINK.AS</t>
+          <t>HYPE.SW</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>21shares Crypto Basket 10 Core ETP</t>
+          <t>21shares Jito Staked SOL ETP</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>HODLX.AS</t>
+          <t>JSOL.AS</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>21shares Crypto Basket Equal Weight ETP</t>
+          <t>21shares NEAR Protocol Staking ETP</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>HODLV.AS</t>
+          <t>NEAR.AS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>21shares Crypto Basket Index ETP</t>
+          <t>21shares Polkadot ETP</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>HODL.AS</t>
+          <t>ADOT.AS</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>21shares Crypto Mid-Cap Index ETP</t>
+          <t>21shares Solana Core Staking ETP</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ALTS.AS</t>
+          <t>CSOL.MI</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>21shares Dogecoin ETP</t>
+          <t>21shares Solana Staking ETP</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>DOGE.SW</t>
+          <t>ASOL.AS</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>21shares Ethena ETP</t>
+          <t>21shares Staking Basket Index ETP</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EENA.SW</t>
+          <t>STAKE.AS</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>21shares Ethereum Core Staking ETP</t>
+          <t>21shares Uniswap ETP</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ETHC.AS</t>
+          <t>AUNI.AS</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>21shares Ethereum Staking ETP</t>
+          <t>21shares XRP ETP</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>AETH.AS</t>
+          <t>AXRP.AS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>21shares Hyperliquid ETP</t>
+          <t>AMINA Bitcoin ETP</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>HYPE.SW</t>
+          <t>SBTCU.AS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>21shares Jito Staked SOL ETP</t>
+          <t>AMINA Ethereum ETP</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>JSOL.AS</t>
+          <t>SETH.AS</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>21shares NEAR Protocol Staking ETP</t>
+          <t>AMINA Polkadot ETP</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>NEAR.AS</t>
+          <t>SDOT.AS</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>21shares Polkadot ETP</t>
+          <t>ARK Artificial Intelligence &amp; Robotics UCITS ETF USD Accumulating</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ADOT.AS</t>
+          <t>ARKI.MI</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>21shares Solana Core Staking ETP</t>
+          <t>ARK Genomic Revolution UCITS ETF USD Accumulating</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CSOL.MI</t>
+          <t>ARKG.MI</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>21shares Solana Staking ETP</t>
+          <t>ARK Innovation UCITS ETF USD Accumulating</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ASOL.AS</t>
+          <t>ARKK.MI</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>21shares Staking Basket Index ETP</t>
+          <t>ARK Space &amp; Defence Innovation UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>STAKE.AS</t>
+          <t>ARKX.MI</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>21shares Stellar ETP</t>
+          <t>Amundi Australia S&amp;P/ASX 200 UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>AXLM.AS</t>
+          <t>AUST.MI</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>21shares Tezos Staking ETP</t>
+          <t>Amundi Bloomberg Equal-weight Commodity ex-Agriculture UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>AXTZ.AS</t>
+          <t>COMO.PA</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>21shares Toncoin Staking ETP</t>
+          <t>Amundi Bloomberg Equal-weight Commodity ex-Agriculture UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>GRAM.AS</t>
+          <t>COMH.MI</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>21shares Uniswap ETP</t>
+          <t>Amundi CAC 40 Daily (-1x) Inverse UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>AUNI.AS</t>
+          <t>SHC.PA</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>21shares XRP ETP</t>
+          <t>Amundi CAC 40 UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>AXRP.AS</t>
+          <t>CACC.PA</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>AMINA Bitcoin ETP</t>
+          <t>Amundi CAC 40 UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SBTCU.AS</t>
+          <t>CAC.PA</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>AMINA Ethereum ETP</t>
+          <t>Amundi Core DAX UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SETH.AS</t>
+          <t>CBDAX.SW</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>AMINA Polkadot ETP</t>
+          <t>Amundi Core EURO STOXX 50 UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>SDOT.AS</t>
+          <t>C50.PA</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ARK Artificial Intelligence &amp; Robotics UCITS ETF USD Accumulating</t>
+          <t>Amundi Core EURO STOXX 50 UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ARKI.MI</t>
+          <t>CD5.PA</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ARK Genomic Revolution UCITS ETF USD Accumulating</t>
+          <t>Amundi Core EURO STOXX 50 UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ARKG.MI</t>
+          <t>C50U.PA</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ARK Innovation UCITS ETF USD Accumulating</t>
+          <t>Amundi Core MSCI EMU UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ARKK.MI</t>
+          <t>MFEC.PA</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ARK Space &amp; Defence Innovation UCITS ETF USD (Acc)</t>
+          <t>Amundi Core MSCI EMU UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ARKX.MI</t>
+          <t>MFE.PA</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Amundi Australia S&amp;P/ASX 200 UCITS ETF Dist</t>
+          <t>Amundi Core MSCI Emerging Markets Swap UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>AUST.MI</t>
+          <t>LEMA.MI</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Amundi Bloomberg Equal-weight Commodity ex-Agriculture UCITS ETF Acc</t>
+          <t>Amundi Core MSCI Emerging Markets Swap UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>COMO.PA</t>
+          <t>E127.MI</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Amundi Bloomberg Equal-weight Commodity ex-Agriculture UCITS ETF EUR Hedged Acc</t>
+          <t>Amundi Core MSCI Emerging Markets UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>COMH.MI</t>
+          <t>AEME.AS</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Amundi CAC 40 Daily (-1x) Inverse UCITS ETF Acc</t>
+          <t>Amundi Core MSCI Europe UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SHC.PA</t>
+          <t>CEU2.AS</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Amundi CAC 40 UCITS ETF Acc</t>
+          <t>Amundi Core MSCI Japan UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>CACC.PA</t>
+          <t>LCJP.AS</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Amundi CAC 40 UCITS ETF Dist</t>
+          <t>Amundi Core MSCI Japan UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>CAC.PA</t>
+          <t>LJPN.AS</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Amundi Core DAX UCITS ETF Dist</t>
+          <t>Amundi Core MSCI USA UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>CBDAX.SW</t>
+          <t>WEBH.MI</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Amundi Core EURO STOXX 50 UCITS ETF EUR Acc</t>
+          <t>Amundi Core MSCI USA UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>C50.PA</t>
+          <t>ETFUSA.MI</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Amundi Core EURO STOXX 50 UCITS ETF EUR Dist</t>
+          <t>Amundi Core MSCI USA UCITS ETF UCITS ETF CHF Hedged Acc</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>CD5.PA</t>
+          <t>USCHF.SW</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Amundi Core EURO STOXX 50 UCITS ETF USD Acc</t>
+          <t>Amundi Core MSCI World UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>C50U.PA</t>
+          <t>WRDU.AS</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Amundi Core MSCI EMU UCITS ETF Acc</t>
+          <t>Amundi Core S&amp;P 500 Swap UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MFEC.PA</t>
+          <t>SP5C.PA</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Amundi Core MSCI EMU UCITS ETF Dist</t>
+          <t>Amundi Core S&amp;P 500 Swap UCITS ETF CHF Hedged Dist</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MFE.PA</t>
+          <t>LYSPH.SW</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Amundi Core MSCI Emerging Markets Swap UCITS ETF Acc</t>
+          <t>Amundi Core S&amp;P 500 Swap UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>LEMA.MI</t>
+          <t>SP5.PA</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Amundi Core MSCI Emerging Markets Swap UCITS ETF Dist</t>
+          <t>Amundi Core S&amp;P 500 Swap UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>E127.MI</t>
+          <t>SPHC.PA</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Amundi Core MSCI Emerging Markets UCITS ETF Acc</t>
+          <t>Amundi Core S&amp;P 500 Swap UCITS ETF EUR Hedged Dist</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>AEME.AS</t>
+          <t>SP5H.PA</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Amundi Core MSCI Europe UCITS ETF Acc</t>
+          <t>Amundi Core S&amp;P 500 Swap UCITS ETF USD Dist</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>CEU2.AS</t>
+          <t>LYSP5.SW</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Amundi Core MSCI Japan UCITS ETF Acc</t>
+          <t>Amundi Core Stoxx Europe 600 UCITS ETF USD Hedged Acc</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>LCJP.AS</t>
+          <t>MEUH.L</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Amundi Core MSCI Japan UCITS ETF Dist</t>
+          <t>Amundi Corporate Proceeds Bond UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>LJPN.AS</t>
+          <t>PLAN.PA</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Amundi Core MSCI USA UCITS ETF Acc</t>
+          <t>Amundi DAX II UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>WEBH.MI</t>
+          <t>DAX.PA</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Amundi Core MSCI USA UCITS ETF Dist</t>
+          <t>Amundi DAX II UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ETFUSA.MI</t>
+          <t>DAXD.SW</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Amundi Core MSCI USA UCITS ETF UCITS ETF CHF Hedged Acc</t>
+          <t>Amundi DIVDAX UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>USCHF.SW</t>
+          <t>CBDDAX.SW</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Amundi Core MSCI World UCITS ETF Acc</t>
+          <t>Amundi DJ Global Titans 50 UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>WRDU.AS</t>
+          <t>MGT.PA</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Amundi Core S&amp;P 500 Swap UCITS ETF Acc</t>
+          <t>Amundi Dow Jones Industrial Average UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SP5C.PA</t>
+          <t>DJE.PA</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Amundi Core S&amp;P 500 Swap UCITS ETF CHF Hedged Dist</t>
+          <t>Amundi ETF DAX UCITS ETF DR</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>LYSPH.SW</t>
+          <t>CG1.PA</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Amundi Core S&amp;P 500 Swap UCITS ETF EUR Dist</t>
+          <t>Amundi ETF JPX Nikkei 400 UCITS ETF Daily Hedged CHF</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SP5.PA</t>
+          <t>JPHC.PA</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Amundi Core S&amp;P 500 Swap UCITS ETF EUR Hedged Acc</t>
+          <t>Amundi ETF S&amp;P 500 Buyback UCITS ETF USD</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SPHC.PA</t>
+          <t>BYBU.PA</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Amundi Core S&amp;P 500 Swap UCITS ETF EUR Hedged Dist</t>
+          <t>Amundi EUR Corporate Bond 1-5Y ESG UCITS ETF DR</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SP5H.PA</t>
+          <t>EBBB.PA</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Amundi Core S&amp;P 500 Swap UCITS ETF USD Dist</t>
+          <t>Amundi EUR Corporate Bond 1-5Y ESG UCITS ETF USD Hedged Acc</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>LYSP5.SW</t>
+          <t>EBBU.PA</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Amundi Core Stoxx Europe 600 UCITS ETF USD Hedged Acc</t>
+          <t>Amundi EUR Corporate Bond Climate Paris Aligned UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MEUH.L</t>
+          <t>CRP.PA</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Amundi Corporate Proceeds Bond UCITS ETF Acc</t>
+          <t>Amundi EUR Corporate Bond ex-Financials ESG UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PLAN.PA</t>
+          <t>CNB.PA</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Amundi DAX II UCITS ETF Acc</t>
+          <t>Amundi EUR High Yield Corporate Bond ESG UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>DAX.PA</t>
+          <t>HYCC.PA</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Amundi DAX II UCITS ETF Dist</t>
+          <t>Amundi EUR High Yield Corporate Bond ESG UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>DAXD.SW</t>
+          <t>YIEL.PA</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Amundi DIVDAX UCITS ETF Dist</t>
+          <t>Amundi EUR Overnight Return UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>CBDDAX.SW</t>
+          <t>CSH.PA</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Amundi DJ Global Titans 50 UCITS ETF Dist</t>
+          <t>Amundi EUR Short Term High Yield Corporate Bond ESG UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>MGT.PA</t>
+          <t>HYS.MI</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Amundi DivDAX II UCITS ETF Dist</t>
+          <t>Amundi EURO STOXX 50 Daily (-1x) Inverse UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>0W76.L</t>
+          <t>BSX.PA</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Amundi Dow Jones Industrial Average UCITS ETF Dist</t>
+          <t>Amundi EURO STOXX 50 Daily (-2x) Inverse UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>DJE.PA</t>
+          <t>BXX.PA</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Amundi ETF DAX UCITS ETF DR</t>
+          <t>Amundi EURO STOXX 50 Daily (2x) Leveraged UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>CG1.PA</t>
+          <t>LVE.PA</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Amundi ETF JPX Nikkei 400 UCITS ETF Daily Hedged CHF</t>
+          <t>Amundi EURO STOXX 50 II UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>JPHC.PA</t>
+          <t>MSE.PA</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Amundi ETF S&amp;P 500 Buyback UCITS ETF USD</t>
+          <t>Amundi EURO STOXX 50 II UCITS ETF CHF Hedged Acc</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>BYBU.PA</t>
+          <t>MSEC.SW</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Amundi EUR Corporate Bond 1-5Y ESG UCITS ETF DR</t>
+          <t>Amundi EURO STOXX 50 II UCITS ETF GBP Hedged Acc</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>EBBB.PA</t>
+          <t>MSEG.SW</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Amundi EUR Corporate Bond 1-5Y ESG UCITS ETF USD Hedged Acc</t>
+          <t>Amundi EURO STOXX 50 II UCITS ETF USD Hedged Acc</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>EBBU.PA</t>
+          <t>MSEU.L</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Amundi EUR Corporate Bond Climate Paris Aligned UCITS ETF Acc</t>
+          <t>Amundi Euro Corporate 0-1Y ESG UCITS ETF DR (C)</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>CRP.PA</t>
+          <t>ECR1.PA</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Amundi EUR Corporate Bond ex-Financials ESG UCITS ETF Acc</t>
+          <t>Amundi Euro Government Bond 0-6 M UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>CNB.PA</t>
+          <t>C3M.PA</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Amundi EUR High Yield Corporate Bond ESG UCITS ETF Acc</t>
+          <t>Amundi Euro High Yield Bond ESG UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>HYCC.PA</t>
+          <t>HYBB.PA</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Amundi EUR High Yield Corporate Bond ESG UCITS ETF Dist</t>
+          <t>Amundi Euro High Yield Bond ESG UCITS ETF EUR (C)</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>YIEL.PA</t>
+          <t>AHYE.PA</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Amundi EUR Overnight Return UCITS ETF Acc</t>
+          <t>Amundi Euro Stoxx Banks UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>CSH.PA</t>
+          <t>BNKE.PA</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Amundi EUR Short Term High Yield Corporate Bond ESG UCITS ETF Dist</t>
+          <t>Amundi European Strategic Autonomy UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>HYS.MI</t>
+          <t>INDEP.PA</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Amundi EURO STOXX 50 Daily (-1x) Inverse UCITS ETF Acc</t>
+          <t>Amundi FTSE EPRA Europe Real Estate UCITS ETF (D)</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>BSX.PA</t>
+          <t>MEH.PA</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Amundi EURO STOXX 50 Daily (-2x) Inverse UCITS ETF Acc</t>
+          <t>Amundi FTSE EPRA Europe Real Estate UCITS ETF EUR (C)</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>BXX.PA</t>
+          <t>EPRE.PA</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Amundi EURO STOXX 50 Daily (2x) Leveraged UCITS ETF Acc</t>
+          <t>Amundi FTSE EPRA NAREIT Global II UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>LVE.PA</t>
+          <t>MWO.PA</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Amundi EURO STOXX 50 II UCITS ETF Acc</t>
+          <t>Amundi FTSE EPRA NAREIT Global UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>MSE.PA</t>
+          <t>EPRU.AS</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Amundi EURO STOXX 50 II UCITS ETF CHF Hedged Acc</t>
+          <t>Amundi FTSE Italia PMI PIR 2020 UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>MSEC.SW</t>
+          <t>ITAMID.MI</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Amundi EURO STOXX 50 II UCITS ETF GBP Hedged Acc</t>
+          <t>Amundi FTSE MIB Daily (-1x) Inverse UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>MSEG.SW</t>
+          <t>BERMIB.MI</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Amundi EURO STOXX 50 II UCITS ETF USD Hedged Acc</t>
+          <t>Amundi FTSE MIB Daily (-2x) Inverse UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>MSEU.L</t>
+          <t>XBRMIB.MI</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Amundi Euro Corporate 0-1Y ESG UCITS ETF DR (C)</t>
+          <t>Amundi FTSE MIB Daily (2x) Leveraged UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>ECR1.PA</t>
+          <t>LEVMIB.MI</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Amundi Euro Government Bond 0-6 M UCITS ETF Acc</t>
+          <t>Amundi FTSE MIB UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>C3M.PA</t>
+          <t>MIB.PA</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Amundi Euro High Yield Bond ESG UCITS ETF Dist</t>
+          <t>Amundi Floating Rate Euro Corporate ESG UCITS ETF EUR (C)</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>HYBB.PA</t>
+          <t>AFRN.PA</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Amundi Euro High Yield Bond ESG UCITS ETF EUR (C)</t>
+          <t>Amundi Floating Rate Euro Corporate ESG UCITS ETF GBP Hedged (C)</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>AHYE.PA</t>
+          <t>AFRHG.PA</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Amundi Euro Stoxx Banks UCITS ETF Acc</t>
+          <t>Amundi Floating Rate Euro Corporate ESG UCITS ETF USD Hedged (C)</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>BNKE.PA</t>
+          <t>AFRHU.PA</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Amundi European Strategic Autonomy UCITS ETF Acc</t>
+          <t>Amundi Floating Rate USD Corporate ESG UCITS ETF EUR Hedged (C)</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>INDEP.PA</t>
+          <t>AFLE.PA</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Amundi FTSE EPRA Europe Real Estate UCITS ETF (D)</t>
+          <t>Amundi Floating Rate USD Corporate ESG UCITS ETF USD (C)</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>MEH.PA</t>
+          <t>AFLT.PA</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Amundi FTSE EPRA Europe Real Estate UCITS ETF EUR (C)</t>
+          <t>Amundi German Bund Daily (-2x) Inverse UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>EPRE.PA</t>
+          <t>DSB.PA</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Amundi FTSE EPRA NAREIT Global II UCITS ETF Dist</t>
+          <t>Amundi Global Corporate SRI 1-5Y UCITS ETF DR (C)</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>MWO.PA</t>
+          <t>UBBB.PA</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Amundi FTSE EPRA NAREIT Global UCITS ETF Acc</t>
+          <t>Amundi Global High Yield Corporate Bond ESG UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>EPRU.AS</t>
+          <t>GHYEH.MI</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Amundi FTSE Italia PMI PIR 2020 UCITS ETF Acc</t>
+          <t>Amundi Global High Yield Corporate Bond ESG UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>ITAMID.MI</t>
+          <t>GHYE.MI</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Amundi FTSE MIB Daily (-1x) Inverse UCITS ETF Acc</t>
+          <t>Amundi IBEX 35 UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>BERMIB.MI</t>
+          <t>CS1.PA</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Amundi FTSE MIB Daily (-2x) Inverse UCITS ETF Acc</t>
+          <t>Amundi Index Euro Corporate SRI 0-3 Y UCITS ETF DR (C)</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>XBRMIB.MI</t>
+          <t>ECRP3.PA</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Amundi FTSE MIB Daily (2x) Leveraged UCITS ETF Dist</t>
+          <t>Amundi Index Euro Corporate SRI UCITS ETF 2 DR EUR (C)</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>LEVMIB.MI</t>
+          <t>CC4.PA</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Amundi FTSE MIB UCITS ETF Dist</t>
+          <t>Amundi Index Euro Corporate SRI UCITS ETF DR (C)</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>MIB.PA</t>
+          <t>ECRP.PA</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Amundi Floating Rate Euro Corporate ESG UCITS ETF EUR (C)</t>
+          <t>Amundi Index US Corporate SRI UCITS ETF DR (C)</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>AFRN.PA</t>
+          <t>UCRP.PA</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Amundi Floating Rate Euro Corporate ESG UCITS ETF GBP Hedged (C)</t>
+          <t>Amundi Italy BTP Daily (-2x) Inverse UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>AFRHG.PA</t>
+          <t>BTPS.PA</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Amundi Floating Rate Euro Corporate ESG UCITS ETF USD Hedged (C)</t>
+          <t>Amundi JPX Nikkei 400 UCITS ETF Daily Hedged EUR (C)</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>AFRHU.PA</t>
+          <t>JPHE.PA</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Amundi Floating Rate USD Corporate ESG UCITS ETF EUR Hedged (C)</t>
+          <t>Amundi JPX Nikkei 400 UCITS ETF Daily Hedged GBP</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>AFLE.PA</t>
+          <t>JPHG.PA</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Amundi Floating Rate USD Corporate ESG UCITS ETF USD (C)</t>
+          <t>Amundi JPX Nikkei 400 UCITS ETF Daily Hedged USD</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>AFLT.PA</t>
+          <t>JPHU.PA</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Amundi German Bund Daily (-2x) Inverse UCITS ETF Acc</t>
+          <t>Amundi JPX Nikkei 400 UCITS ETF EUR (C)</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>DSB.PA</t>
+          <t>JPNK.PA</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Amundi Global Corporate SRI 1-5Y UCITS ETF DR (C)</t>
+          <t>Amundi JPX Nikkei 400 UCITS ETF JPY</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>UBBB.PA</t>
+          <t>JPNY.PA</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Amundi Global High Yield Corporate Bond ESG UCITS ETF EUR Hedged Acc</t>
+          <t>Amundi Japan TOPIX II UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>GHYEH.MI</t>
+          <t>JPN.PA</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Amundi Global High Yield Corporate Bond ESG UCITS ETF USD Acc</t>
+          <t>Amundi Japan TOPIX II UCITS ETF EUR Hedged Dist</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>GHYE.MI</t>
+          <t>JPNH.PA</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Amundi IBEX 35 UCITS ETF Acc</t>
+          <t>Amundi Japan TOPIX II UCITS ETF JPY Dist</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>CS1.PA</t>
+          <t>LYJPN.SW</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Amundi Index Euro Corporate SRI 0-3 Y UCITS ETF DR (C)</t>
+          <t>Amundi Japan Topix UCITS ETF Daily Hedged CHF</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>ECRP3.PA</t>
+          <t>TPHC.PA</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Amundi Index Euro Corporate SRI UCITS ETF 2 DR EUR (C)</t>
+          <t>Amundi Japan Topix UCITS ETF Daily Hedged EUR (C)</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>CC4.PA</t>
+          <t>TPXH.PA</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Amundi Index Euro Corporate SRI UCITS ETF DR (C)</t>
+          <t>Amundi Japan Topix UCITS ETF Daily Hedged GBP</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>ECRP.PA</t>
+          <t>TPHG.PA</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Amundi Index US Corporate SRI UCITS ETF DR (C)</t>
+          <t>Amundi Japan Topix UCITS ETF Daily Hedged USD</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>UCRP.PA</t>
+          <t>TPHU.PA</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Amundi Italy BTP Daily (-2x) Inverse UCITS ETF Acc</t>
+          <t>Amundi Japan Topix UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>BTPS.PA</t>
+          <t>TPXE.PA</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Amundi JPX Nikkei 400 UCITS ETF Daily Hedged EUR (C)</t>
+          <t>Amundi Japan Topix UCITS ETF JPY</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>JPHE.PA</t>
+          <t>TPXY.PA</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Amundi JPX Nikkei 400 UCITS ETF Daily Hedged GBP</t>
+          <t>Amundi LevDax Daily (2x) leveraged UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>JPHG.PA</t>
+          <t>LVD.PA</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Amundi JPX Nikkei 400 UCITS ETF Daily Hedged USD</t>
+          <t>Amundi MDAX ESG II UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>JPHU.PA</t>
+          <t>CB1MDX.SW</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Amundi JPX Nikkei 400 UCITS ETF EUR (C)</t>
+          <t>Amundi MDAX ESG UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>JPNK.PA</t>
+          <t>CBMDAX.SW</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Amundi JPX Nikkei 400 UCITS ETF JPY</t>
+          <t>Amundi MDAX UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>JPNY.PA</t>
+          <t>MDX.PA</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Amundi Japan TOPIX II UCITS ETF EUR Dist</t>
+          <t>Amundi MSCI AC Asia Ex Japan UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>JPN.PA</t>
+          <t>APX.PA</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Amundi Japan TOPIX II UCITS ETF EUR Hedged Dist</t>
+          <t>Amundi MSCI AC Asia Pacific Ex Japan UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>JPNH.PA</t>
+          <t>AEJ.PA</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Amundi Japan TOPIX II UCITS ETF JPY Dist</t>
+          <t>Amundi MSCI ACWI SRI Climate Paris Aligned UCITS ETF DR - USD</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>LYJPN.SW</t>
+          <t>WELA.SW</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Amundi Japan Topix UCITS ETF Daily Hedged CHF</t>
+          <t>Amundi MSCI All Country World UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>TPHC.PA</t>
+          <t>ACWI.PA</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Amundi Japan Topix UCITS ETF Daily Hedged EUR (C)</t>
+          <t>Amundi MSCI EMU High Dividend UCITS ETF UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>TPXH.PA</t>
+          <t>CD8.PA</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Amundi Japan Topix UCITS ETF Daily Hedged GBP</t>
+          <t>Amundi MSCI Eastern Europe Ex Russia UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>TPHG.PA</t>
+          <t>CEC.PA</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Amundi Japan Topix UCITS ETF Daily Hedged USD</t>
+          <t>Amundi MSCI Emerging Ex China UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>TPHU.PA</t>
+          <t>EMXC.PA</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Amundi Japan Topix UCITS ETF EUR</t>
+          <t>Amundi MSCI Emerging Markets Asia UCITS ETF EUR (C)</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>TPXE.PA</t>
+          <t>AASI.PA</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Amundi Japan Topix UCITS ETF JPY</t>
+          <t>Amundi MSCI Emerging Markets Asia UCITS ETF USD</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>TPXY.PA</t>
+          <t>AASU.PA</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Amundi LevDax Daily (2x) leveraged UCITS ETF Acc</t>
+          <t>Amundi MSCI Emerging Markets Latin America UCITS ETF EUR (C)</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>LVD.PA</t>
+          <t>ALAT.PA</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Amundi MDAX ESG II UCITS ETF Dist</t>
+          <t>Amundi MSCI Emerging Markets Latin America UCITS ETF USD</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CB1MDX.SW</t>
+          <t>ALAU.PA</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Amundi MDAX ESG UCITS ETF Dist</t>
+          <t>Amundi MSCI Emerging Markets Swap II UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>CBMDAX.SW</t>
+          <t>LEM.PA</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Amundi MDAX UCITS ETF Dist</t>
+          <t>Amundi MSCI Emerging Markets Swap II UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>MDX.PA</t>
+          <t>LYLEM.SW</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Amundi MSCI AC Asia Ex Japan UCITS ETF Acc</t>
+          <t>Amundi MSCI Emerging Markets Swap UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>APX.PA</t>
+          <t>AEEM.PA</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Amundi MSCI AC Asia Pacific Ex Japan UCITS ETF Acc</t>
+          <t>Amundi MSCI Emerging Markets Swap UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>AEJ.PA</t>
+          <t>AUEM.PA</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Amundi MSCI ACWI SRI Climate Paris Aligned UCITS ETF DR - USD</t>
+          <t>Amundi MSCI Europe Growth UCITS ETF - EUR (C)</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>WELA.SW</t>
+          <t>CG9.PA</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Amundi MSCI All Country World UCITS ETF EUR Acc</t>
+          <t>Amundi MSCI Europe Growth UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>ACWI.PA</t>
+          <t>GWT.PA</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Amundi MSCI EMU High Dividend UCITS ETF UCITS ETF Acc</t>
+          <t>Amundi MSCI Europe High Dividend Factor UCITS ETF EUR (C)</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>CD8.PA</t>
+          <t>CD9.PA</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Amundi MSCI Eastern Europe Ex Russia UCITS ETF Acc</t>
+          <t>Amundi MSCI Europe Minimum Volatility Factor UCITS ETF EUR (C)</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>CEC.PA</t>
+          <t>MIVO.L</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Amundi MSCI Emerging Ex China UCITS ETF Acc</t>
+          <t>Amundi MSCI Europe Quality Factor UCITS ETF EUR (C)</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>EMXC.PA</t>
+          <t>QCEU.PA</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Amundi MSCI Emerging Markets Asia UCITS ETF EUR (C)</t>
+          <t>Amundi MSCI Europe UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>AASI.PA</t>
+          <t>MEU.PA</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Amundi MSCI Emerging Markets Asia UCITS ETF USD</t>
+          <t>Amundi MSCI Greece UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>AASU.PA</t>
+          <t>GRE.PA</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Amundi MSCI Emerging Markets Latin America UCITS ETF EUR (C)</t>
+          <t>Amundi MSCI India Swap II UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>ALAT.PA</t>
+          <t>CI2.PA</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Amundi MSCI Emerging Markets Latin America UCITS ETF USD</t>
+          <t>Amundi MSCI India Swap II UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>ALAU.PA</t>
+          <t>CI2U.PA</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Amundi MSCI Emerging Markets Swap II UCITS ETF EUR Acc</t>
+          <t>Amundi MSCI India Swap UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>LEM.PA</t>
+          <t>INR.PA</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Amundi MSCI Emerging Markets Swap II UCITS ETF USD Acc</t>
+          <t>Amundi MSCI India Swap UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>LYLEM.SW</t>
+          <t>LYINR.SW</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Amundi MSCI Emerging Markets Swap UCITS ETF EUR Acc</t>
+          <t>Amundi MSCI Indonesia UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>AEEM.PA</t>
+          <t>INDO.PA</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Amundi MSCI Emerging Markets Swap UCITS ETF USD Acc</t>
+          <t>Amundi MSCI Japan SRI Climate Paris Aligned UCITS ETF DR (C)</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>AUEM.PA</t>
+          <t>JPXY.AS</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Amundi MSCI Europe Growth UCITS ETF - EUR (C)</t>
+          <t>Amundi MSCI Japan SRI Climate Paris Aligned UCITS ETF DR - EUR Hedged (C)</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>CG9.PA</t>
+          <t>JPXH.PA</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Amundi MSCI Europe Growth UCITS ETF Dist</t>
+          <t>Amundi MSCI Japan SRI Climate Paris Aligned UCITS ETF DR - EUR Hedged (D)</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>GWT.PA</t>
+          <t>JPHD.PA</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Amundi MSCI Europe High Dividend Factor UCITS ETF EUR (C)</t>
+          <t>Amundi MSCI Japan SRI Climate Paris Aligned UCITS ETF DR - GBP Hedged (C)</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>CD9.PA</t>
+          <t>JPXX.L</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Amundi MSCI Europe Minimum Volatility Factor UCITS ETF EUR (C)</t>
+          <t>Amundi MSCI Japan SRI Climate Paris Aligned UCITS ETF DR - USD Hedged (C)</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>MIVO.L</t>
+          <t>JPXU.L</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Amundi MSCI Europe Quality Factor UCITS ETF EUR (C)</t>
+          <t>Amundi MSCI Korea UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>QCEU.PA</t>
+          <t>KRW.PA</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Amundi MSCI Europe UCITS ETF Acc</t>
+          <t>Amundi MSCI Nordic UCITS ETF EUR (C)</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>MEU.PA</t>
+          <t>CN1.PA</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Amundi MSCI Greece UCITS ETF Dist</t>
+          <t>Amundi MSCI Pacific Ex Japan UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>GRE.PA</t>
+          <t>PAXJ.SW</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Amundi MSCI India Swap II UCITS ETF EUR Acc</t>
+          <t>Amundi MSCI Robotics &amp; AI UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>CI2.PA</t>
+          <t>GOAI.AS</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Amundi MSCI India Swap II UCITS ETF USD Acc</t>
+          <t>Amundi MSCI Smart Cities UCITS ETF - Acc</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>CI2U.PA</t>
+          <t>SCITY.AS</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Amundi MSCI India Swap UCITS ETF EUR Acc</t>
+          <t>Amundi MSCI UK IMI SRI Climate Paris Aligned UCITS ETF - EUR (C)</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>INR.PA</t>
+          <t>C1U.PA</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Amundi MSCI India Swap UCITS ETF USD Acc</t>
+          <t>Amundi MSCI UK IMI SRI Climate Paris Aligned UCITS ETF - GBP (C)</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>LYINR.SW</t>
+          <t>FTSE.PA</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Amundi MSCI Indonesia UCITS ETF Acc</t>
+          <t>Amundi MSCI USA Daily (-1x) Inverse UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>INDO.PA</t>
+          <t>DSP5.PA</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Amundi MSCI Japan SRI Climate Paris Aligned UCITS ETF DR (C)</t>
+          <t>Amundi MSCI USA Daily (2x) Leveraged UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>JPXY.AS</t>
+          <t>CL2.PA</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Amundi MSCI Japan SRI Climate Paris Aligned UCITS ETF DR - EUR Hedged (C)</t>
+          <t>Amundi MSCI USA ESG Leaders Extra UCITS ETF DR - USD (D)</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>JPXH.PA</t>
+          <t>UESG.MI</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Amundi MSCI Japan SRI Climate Paris Aligned UCITS ETF DR - EUR Hedged (D)</t>
+          <t>Amundi MSCI USA ESG Leaders Extra UCITS ETF DR USD (A)</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>JPHD.PA</t>
+          <t>LUESG.SW</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Amundi MSCI Japan SRI Climate Paris Aligned UCITS ETF DR - GBP Hedged (C)</t>
+          <t>Amundi MSCI USA ESG Selection UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>JPXX.L</t>
+          <t>SADU.PA</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Amundi MSCI Japan SRI Climate Paris Aligned UCITS ETF DR - USD Hedged (C)</t>
+          <t>Amundi MSCI USA ESG Selection UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>JPXU.L</t>
+          <t>USAL.PA</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Amundi MSCI Korea UCITS ETF Acc</t>
+          <t>Amundi MSCI USA Ex Mega Cap UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>KRW.PA</t>
+          <t>XMGA.MI</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Amundi MSCI Nordic UCITS ETF EUR (C)</t>
+          <t>Amundi MSCI USA Mega Cap UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>CN1.PA</t>
+          <t>MEGA.L</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Amundi MSCI Pacific Ex Japan UCITS ETF Dist</t>
+          <t>Amundi MSCI USA Minimum Volatility Factor UCITS ETF DR</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>PAXJ.SW</t>
+          <t>MIVU.AS</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Amundi MSCI Robotics &amp; AI UCITS ETF Acc</t>
+          <t>Amundi MSCI USA SRI Climate Paris Aligned UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>GOAI.AS</t>
+          <t>USRI.AS</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Amundi MSCI Smart Cities UCITS ETF - Acc</t>
+          <t>Amundi MSCI USA SRI Climate Paris Aligned UCITS ETF Acc EUR Hedged</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>SCITY.AS</t>
+          <t>USRIH.MI</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Amundi MSCI UK IMI SRI Climate Paris Aligned UCITS ETF - EUR (C)</t>
+          <t>Amundi MSCI USA Screened UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>C1U.PA</t>
+          <t>USAS.PA</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Amundi MSCI UK IMI SRI Climate Paris Aligned UCITS ETF - GBP (C)</t>
+          <t>Amundi MSCI World (2x) Leveraged UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>FTSE.PA</t>
+          <t>LWLD.PA</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA Daily (-1x) Inverse UCITS ETF Acc</t>
+          <t>Amundi MSCI World ESG Selection UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>DSP5.PA</t>
+          <t>ESGWO.MI</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA Daily (2x) Leveraged UCITS ETF Acc</t>
+          <t>Amundi MSCI World ESG Selection UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>CL2.PA</t>
+          <t>MWOS.PA</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA ESG Leaders Extra UCITS ETF DR - USD (D)</t>
+          <t>Amundi MSCI World Ex EMU UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>UESG.MI</t>
+          <t>CM9.PA</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA ESG Leaders Extra UCITS ETF DR USD (A)</t>
+          <t>Amundi MSCI World Ex USA UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>LUESG.SW</t>
+          <t>WEXU.L</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA ESG Selection UCITS ETF Acc</t>
+          <t>Amundi MSCI World Financials UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>SADU.PA</t>
+          <t>FINSW.PA</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA ESG Selection UCITS ETF EUR Hedged Acc</t>
+          <t>Amundi MSCI World Financials UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>USAL.PA</t>
+          <t>LYFINW.SW</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA Ex Mega Cap UCITS ETF Acc</t>
+          <t>Amundi MSCI World Health Care UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>XMGA.MI</t>
+          <t>HLTW.PA</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA Mega Cap UCITS ETF Acc</t>
+          <t>Amundi MSCI World Health Care UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>MEGA.L</t>
+          <t>LYHLTW.SW</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA Minimum Volatility Factor UCITS ETF DR</t>
+          <t>Amundi MSCI World SRI Climate Paris Aligned UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>MIVU.AS</t>
+          <t>WSRI.AS</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA SRI Climate Paris Aligned UCITS ETF Acc</t>
+          <t>Amundi MSCI World SRI Climate Paris Aligned UCITS ETF Acc EUR Hedged</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>USRI.AS</t>
+          <t>WESE.PA</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA SRI Climate Paris Aligned UCITS ETF Acc EUR Hedged</t>
+          <t>Amundi MSCI World Screened UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>USRIH.MI</t>
+          <t>WLSC.PA</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA Screened UCITS ETF Acc</t>
+          <t>Amundi MSCI World Swap II UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>USAS.PA</t>
+          <t>WLDC.PA</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Amundi MSCI World (2x) Leveraged UCITS ETF Acc</t>
+          <t>Amundi MSCI World Swap II UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>LWLD.PA</t>
+          <t>WLD.PA</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Amundi MSCI World ESG Selection UCITS ETF Acc</t>
+          <t>Amundi MSCI World Swap II UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>ESGWO.MI</t>
+          <t>WLDHC.PA</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Amundi MSCI World ESG Selection UCITS ETF EUR Hedged Acc</t>
+          <t>Amundi MSCI World Swap II UCITS ETF EUR Hedged Dist</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>MWOS.PA</t>
+          <t>WLDH.PA</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Ex EMU UCITS ETF Acc</t>
+          <t>Amundi MSCI World Swap II UCITS ETF USD Hedged Dist</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>CM9.PA</t>
+          <t>WLDHU.SW</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Ex USA UCITS ETF Acc</t>
+          <t>Amundi MSCI World Swap UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>WEXU.L</t>
+          <t>CW8.PA</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Financials UCITS ETF EUR Acc</t>
+          <t>Amundi MSCI World Swap UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>FINSW.PA</t>
+          <t>EWLD.PA</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Financials UCITS ETF USD Acc</t>
+          <t>Amundi MSCI World Swap UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>LYFINW.SW</t>
+          <t>CW8U.PA</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Health Care UCITS ETF EUR Acc</t>
+          <t>Amundi MSCI World ex Europe UCITS ETF EUR (C)</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>HLTW.PA</t>
+          <t>CE8.PA</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Health Care UCITS ETF USD Acc</t>
+          <t>Amundi Multi-Asset Portfolio Defensive UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>LYHLTW.SW</t>
+          <t>CBVSD.SW</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Amundi MSCI World SRI Climate Paris Aligned UCITS ETF Acc</t>
+          <t>Amundi Multi-Asset Portfolio Offensive UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>WSRI.AS</t>
+          <t>CBVSO.SW</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Amundi MSCI World SRI Climate Paris Aligned UCITS ETF Acc EUR Hedged</t>
+          <t>Amundi Multi-Asset Portfolio UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>WESE.PA</t>
+          <t>CBVS.SW</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Screened UCITS ETF Acc</t>
+          <t>Amundi Nasdaq-100 Daily (2x) Leveraged UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>WLSC.PA</t>
+          <t>LQQ.PA</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Swap II UCITS ETF Acc</t>
+          <t>Amundi PEA MSCI USA ESG Selection UCITS ETF - EUR</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>WLDC.PA</t>
+          <t>CU2.PA</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Swap II UCITS ETF Dist</t>
+          <t>Amundi PEA MSCI USA ESG Selection UCITS ETF - USD</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>WLD.PA</t>
+          <t>CU2U.PA</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Swap II UCITS ETF EUR Hedged Acc</t>
+          <t>Amundi PEA Monde (MSCI World) UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>WLDHC.PA</t>
+          <t>DCAM.PA</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Swap II UCITS ETF EUR Hedged Dist</t>
+          <t>Amundi Pan Africa UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>WLDH.PA</t>
+          <t>LAFRI.MI</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Swap II UCITS ETF USD Hedged Dist</t>
+          <t>Amundi Physical Gold ETC (C)</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>WLDHU.SW</t>
+          <t>GOLD.AS</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Swap UCITS ETF EUR Acc</t>
+          <t>Amundi Prime All Country World UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>CW8.PA</t>
+          <t>WEBN.MI</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Swap UCITS ETF EUR Dist</t>
+          <t>Amundi Prime All Country World UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>EWLD.PA</t>
+          <t>WEBG.SW</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Amundi MSCI World Swap UCITS ETF USD Acc</t>
+          <t>Amundi Prime All Country World UCITS ETF GBP Hedged Dist</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>CW8U.PA</t>
+          <t>WEHG.L</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Amundi MSCI World ex Europe UCITS ETF EUR (C)</t>
+          <t>Amundi Prime Europe UCITS ETF DR (D)</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>CE8.PA</t>
+          <t>ETFEU.MI</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Amundi Multi-Asset Portfolio Defensive UCITS ETF Dist</t>
+          <t>Amundi Prime Eurozone UCITS ETF DR (D)</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>CBVSD.SW</t>
+          <t>ETFEZ.MI</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Amundi Multi-Asset Portfolio Offensive UCITS ETF Dist</t>
+          <t>Amundi Prime Global UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>CBVSO.SW</t>
+          <t>ETFGLO.MI</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Amundi Multi-Asset Portfolio UCITS ETF Dist</t>
+          <t>Amundi Prime Japan UCITS ETF DR (C)</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>CBVS.SW</t>
+          <t>PRAJ.PA</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Amundi Nasdaq-100 Daily (2x) Leveraged UCITS ETF Acc</t>
+          <t>Amundi Prime Japan UCITS ETF DR (D)</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>LQQ.PA</t>
+          <t>ETFJAP.MI</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Amundi PEA MSCI USA ESG Selection UCITS ETF - EUR</t>
+          <t>Amundi Russell 1000 Growth UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>CU2.PA</t>
+          <t>MWOT.L</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Amundi PEA MSCI USA ESG Selection UCITS ETF - USD</t>
+          <t>Amundi S&amp;P 500 Buyback UCITS ETF EUR (C)</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>CU2U.PA</t>
+          <t>BYBE.PA</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Amundi PEA Monde (MSCI World) UCITS ETF Acc</t>
+          <t>Amundi S&amp;P 500 Equal Weight ESG UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>DCAM.PA</t>
+          <t>WELE.MI</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Amundi Pan Africa UCITS ETF Acc</t>
+          <t>Amundi S&amp;P 500 Equal Weight ESG UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>LAFRI.MI</t>
+          <t>MWOQ.PA</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Amundi Physical Gold ETC (C)</t>
+          <t>Amundi S&amp;P 500 Equal Weight UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>GOLD.AS</t>
+          <t>EQSU.L</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Amundi Prime All Country World UCITS ETF Acc</t>
+          <t>Amundi S&amp;P 500 Screened UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>WEBN.MI</t>
+          <t>U500.AS</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Amundi Prime All Country World UCITS ETF Dist</t>
+          <t>Amundi S&amp;P 500 Screened UCITS ETF Acc EUR Hedged</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>WEBG.SW</t>
+          <t>S500H.PA</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Amundi Prime All Country World UCITS ETF GBP Hedged Dist</t>
+          <t>Amundi S&amp;P 500 Swap UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>WEHG.L</t>
+          <t>500.PA</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Amundi Prime Europe UCITS ETF DR (C)</t>
+          <t>Amundi S&amp;P 500 Swap UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>PRAE.PA</t>
+          <t>500H.PA</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Amundi Prime Europe UCITS ETF DR (D)</t>
+          <t>Amundi S&amp;P 500 Swap UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>ETFEU.MI</t>
+          <t>500E.AS</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Amundi Prime Eurozone UCITS ETF DR (C)</t>
+          <t>Amundi S&amp;P Eurozone Dividend Aristocrat Screened UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>PRAZ.PA</t>
+          <t>EUDIV.PA</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Amundi Prime Eurozone UCITS ETF DR (D)</t>
+          <t>Amundi S&amp;P Global Communication Services ESG UCITS ETF DR EUR (A)</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>ETFEZ.MI</t>
+          <t>TELW.PA</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Amundi Prime Global UCITS ETF Dist</t>
+          <t>Amundi S&amp;P Global Consumer Discretionary ESG UCITS ETF DR EUR (A)</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>ETFGLO.MI</t>
+          <t>CODW.PA</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Amundi Prime Japan UCITS ETF DR (C)</t>
+          <t>Amundi S&amp;P Global Consumer Staples ESG UCITS ETF DR EUR (A)</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>PRAJ.PA</t>
+          <t>COSW.PA</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>Amundi Prime Japan UCITS ETF DR (D)</t>
+          <t>Amundi S&amp;P Global Energy Carbon Reduced UCITS ETF DR EUR (A)</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>ETFJAP.MI</t>
+          <t>NRGW.PA</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Amundi Russell 1000 Growth UCITS ETF Acc</t>
+          <t>Amundi S&amp;P Global Financials ESG UCITS ETF DR EUR (A)</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>MWOT.L</t>
+          <t>GLFI.PA</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P 500 Buyback UCITS ETF EUR (C)</t>
+          <t>Amundi S&amp;P Global Health Care ESG UCITS ETF DR EUR (A)</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>BYBE.PA</t>
+          <t>GLHL.PA</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P 500 Equal Weight ESG UCITS ETF Acc</t>
+          <t>Amundi S&amp;P Global Industrials ESG UCITS ETF DR EUR (A)</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>WELE.MI</t>
+          <t>INDW.PA</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P 500 Equal Weight ESG UCITS ETF EUR Hedged Acc</t>
+          <t>Amundi S&amp;P Global Information Technology ESG UCITS ETF DR EUR (A)</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>MWOQ.PA</t>
+          <t>GLIT.PA</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P 500 Equal Weight UCITS ETF Acc</t>
+          <t>Amundi S&amp;P Global Materials ESG UCITS ETF DR EUR (A)</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>EQSU.L</t>
+          <t>MATW.PA</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P 500 Screened UCITS ETF Acc</t>
+          <t>Amundi S&amp;P Global Utilities ESG UCITS ETF DR EUR (A)</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>U500.AS</t>
+          <t>UTIW.MI</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P 500 Screened UCITS ETF Acc EUR Hedged</t>
+          <t>Amundi STOXX Europe 600 Banks UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>S500H.PA</t>
+          <t>BNK.PA</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P 500 Swap UCITS ETF EUR Acc</t>
+          <t>Amundi STOXX Europe 600 Basic Materials UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>500.PA</t>
+          <t>CHM.PA</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P 500 Swap UCITS ETF EUR Hedged Acc</t>
+          <t>Amundi STOXX Europe 600 Basic Resources UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>500H.PA</t>
+          <t>BRES.PA</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P 500 Swap UCITS ETF USD Acc</t>
+          <t>Amundi STOXX Europe 600 Consumer Discretionary UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>500E.AS</t>
+          <t>TRV.PA</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P 500 Swap UCITS ETF USD Dist</t>
+          <t>Amundi STOXX Europe 600 Consumer Staples UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>500D.PA</t>
+          <t>FOO.PA</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P Eurozone Dividend Aristocrat Screened UCITS ETF Dist</t>
+          <t>Amundi STOXX Europe 600 Healthcare UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>EUDIV.PA</t>
+          <t>HLT.PA</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P Global Communication Services ESG UCITS ETF DR EUR (A)</t>
+          <t>Amundi STOXX Europe 600 Telecommunications UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>TELW.PA</t>
+          <t>TELE.PA</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P Global Consumer Discretionary ESG UCITS ETF DR EUR (A)</t>
+          <t>Amundi STOXX Europe 600 Utilities UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>CODW.PA</t>
+          <t>UTI.PA</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P Global Consumer Staples ESG UCITS ETF DR EUR (A)</t>
+          <t>Amundi ShortDAX Daily (-2x) Inverse UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>COSW.PA</t>
+          <t>DSD.PA</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P Global Energy Carbon Reduced UCITS ETF DR EUR (A)</t>
+          <t>Amundi Smart Overnight Return UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>NRGW.PA</t>
+          <t>CSH2.PA</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P Global Financials ESG UCITS ETF DR EUR (A)</t>
+          <t>Amundi Smart Overnight Return UCITS ETF CHF Hedged Acc</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>GLFI.PA</t>
+          <t>SMCH.SW</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P Global Health Care ESG UCITS ETF DR EUR (A)</t>
+          <t>Amundi Smart Overnight Return UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>GLHL.PA</t>
+          <t>SMOR.SW</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P Global Industrials ESG UCITS ETF DR EUR (A)</t>
+          <t>Amundi Smart Overnight Return UCITS ETF GBP Hedged Acc</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>INDW.PA</t>
+          <t>LYSMG.SW</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P Global Information Technology ESG UCITS ETF DR EUR (A)</t>
+          <t>Amundi Smart Overnight Return UCITS ETF USD Hedged Acc</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>GLIT.PA</t>
+          <t>SMARTU.MI</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P Global Materials ESG UCITS ETF DR EUR (A)</t>
+          <t>Amundi Stoxx Europe 50 UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>MATW.PA</t>
+          <t>C5E.PA</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P Global Utilities ESG UCITS ETF DR EUR (A)</t>
+          <t>Amundi Stoxx Europe Select Dividend 30 UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>UTIW.MI</t>
+          <t>SEL.PA</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Amundi STOXX Europe 600 Banks UCITS ETF Acc</t>
+          <t>Amundi US Curve steepening 2-10Y UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>BNK.PA</t>
+          <t>STPU.PA</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Amundi STOXX Europe 600 Basic Materials UCITS ETF Acc</t>
+          <t>Amundi US Curve steepening 2-10Y UCITS ETF GBP Hedged Dist</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>CHM.PA</t>
+          <t>STPH.L</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Amundi STOXX Europe 600 Basic Resources UCITS ETF Acc</t>
+          <t>Amundi US Tech 100 Equal Weight UCITS ETF DR USD D</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>BRES.PA</t>
+          <t>UTEC.L</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Amundi STOXX Europe 600 Consumer Discretionary UCITS ETF Acc</t>
+          <t>Amundi USD Corporate Bond Climate Paris Aligned UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>TRV.PA</t>
+          <t>USIC.MI</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Amundi STOXX Europe 600 Consumer Staples UCITS ETF Acc</t>
+          <t>Amundi USD Corporate Bond Climate Paris Aligned UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>FOO.PA</t>
+          <t>USIG.MI</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Amundi STOXX Europe 600 Healthcare UCITS ETF Acc</t>
+          <t>Amundi USD Corporate Bond Climate Paris Aligned UCITS ETF EUR Hedged Dist</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>HLT.PA</t>
+          <t>USIH.PA</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Amundi STOXX Europe 600 Telecommunications UCITS ETF Acc</t>
+          <t>Amundi USD Fed Funds Rate UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>TELE.PA</t>
+          <t>FEDF.MI</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Amundi STOXX Europe 600 Utilities UCITS ETF Acc</t>
+          <t>Amundi USD Fed Funds Rate UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>UTI.PA</t>
+          <t>CBFEDF.SW</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Amundi ShortDAX Daily (-1x) Inverse UCITS ETF - Dist</t>
+          <t>Amundi USD High Yield Corporate Bond ESG UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>AHYK.PA</t>
+          <t>USHYC.MI</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Amundi ShortDAX Daily (-2x) Inverse UCITS ETF Acc</t>
+          <t>Amundi USD High Yield Corporate Bond ESG UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>DSD.PA</t>
+          <t>USHY.PA</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Amundi Smart Overnight Return UCITS ETF Acc</t>
+          <t>Amundi USD High Yield Corporate Bond ESG UCITS ETF EUR HEDGED Dist</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>CSH2.PA</t>
+          <t>USYH.MI</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Amundi Smart Overnight Return UCITS ETF CHF Hedged Acc</t>
+          <t>Avantis America Equity UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>SMCH.SW</t>
+          <t>AVAE.L</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Amundi Smart Overnight Return UCITS ETF Dist</t>
+          <t>Avantis Emerging Markets Equity UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>SMOR.SW</t>
+          <t>AVEM.L</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Amundi Smart Overnight Return UCITS ETF GBP Hedged Acc</t>
+          <t>Avantis Europe Equity UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>LYSMG.SW</t>
+          <t>AVUE.L</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Amundi Smart Overnight Return UCITS ETF USD Hedged Acc</t>
+          <t>Avantis Global Equity UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>SMARTU.MI</t>
+          <t>AVCG.L</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Amundi Stoxx Europe 50 UCITS ETF Acc</t>
+          <t>Avantis Global Small Cap Value UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>C5E.PA</t>
+          <t>AVSG.L</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>Amundi Stoxx Europe Select Dividend 30 UCITS ETF Dist</t>
+          <t>Avantis Pacific Equity UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>SEL.PA</t>
+          <t>AVEP.L</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Amundi US Curve steepening 2-10Y UCITS ETF Acc</t>
+          <t>BNP Paribas Easy Alpha Enhanced EUR Corporate Bond UCITS ETF (Acc)</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>STPU.PA</t>
+          <t>QEIG.PA</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Amundi US Curve steepening 2-10Y UCITS ETF GBP Hedged Dist</t>
+          <t>BNP Paribas Easy Alpha Enhanced Europe UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>STPH.L</t>
+          <t>QEUR.PA</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Amundi US Tech 100 Equal Weight UCITS ETF DR USD D</t>
+          <t>BNP Paribas Easy Alpha Enhanced US UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>UTEC.L</t>
+          <t>QUSAE.PA</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Amundi USD Corporate Bond Climate Paris Aligned UCITS ETF Acc</t>
+          <t>BNP Paribas Easy Alpha Enhanced World UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>USIC.MI</t>
+          <t>QGLOE.PA</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Amundi USD Corporate Bond Climate Paris Aligned UCITS ETF Dist</t>
+          <t>BNP Paribas Easy Dividend Europe UCITS ETF</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>USIG.MI</t>
+          <t>EDEU.PA</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>Amundi USD Corporate Bond Climate Paris Aligned UCITS ETF EUR Hedged Dist</t>
+          <t>BNP Paribas Easy ECPI Global ESG Blue Economy UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>USIH.PA</t>
+          <t>BLUE.PA</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Amundi USD Fed Funds Rate UCITS ETF Acc</t>
+          <t>BNP Paribas Easy ECPI Global ESG Blue Economy UCITS ETF USD</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>FEDF.MI</t>
+          <t>BLUSD.PA</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Amundi USD Fed Funds Rate UCITS ETF Dist</t>
+          <t>BNP Paribas Easy ECPI Global ESG Infrastructure UCITS ETF EUR Capitalisation</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>CBFEDF.SW</t>
+          <t>ENG.PA</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Amundi USD High Yield Corporate Bond ESG UCITS ETF Acc</t>
+          <t>BNP Paribas Easy ECPI Global ESG Infrastructure UCITS ETF USD Capitalisation</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>USHYC.MI</t>
+          <t>ENGUS.PA</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Amundi USD High Yield Corporate Bond ESG UCITS ETF Dist</t>
+          <t>BNP Paribas Easy ESG Enhanced EMU UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>USHY.PA</t>
+          <t>AEMUS.PA</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Amundi USD High Yield Corporate Bond ESG UCITS ETF EUR HEDGED Dist</t>
+          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2027 UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>USYH.MI</t>
+          <t>ACE27.MI</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Avantis America Equity UCITS ETF Acc</t>
+          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2029 UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>AVAE.L</t>
+          <t>ACE29.PA</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Avantis Emerging Markets Equity UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2032 UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>AVEM.L</t>
+          <t>ACE32.PA</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Avantis Europe Equity UCITS ETF Acc</t>
+          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond UCITS ETF Capitalisation</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>AVUE.L</t>
+          <t>SEUCB.MI</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Avantis Global Equity UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy ESG Enhanced EUR Government Bond UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>AVCG.L</t>
+          <t>SEUGB.MI</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Avantis Global Small Cap Value UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy ESG Enhanced Europe UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>AVSG.L</t>
+          <t>AEUSE.PA</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Avantis Pacific Equity UCITS ETF Acc</t>
+          <t>BNP Paribas Easy ESG Enhanced Japan UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>AVEP.L</t>
+          <t>AJASE.PA</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Alpha Enhanced EUR Corporate Bond UCITS ETF (Acc)</t>
+          <t>BNP Paribas Easy ESG Enhanced Japan UCITS ETF EUR Hedged (Acc)</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>QEIG.PA</t>
+          <t>AJASH.PA</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Alpha Enhanced Europe UCITS ETF Acc</t>
+          <t>BNP Paribas Easy ESG Enhanced US UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>QEUR.PA</t>
+          <t>AUSSE.PA</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Alpha Enhanced Global High Yield UCITS ETF (Acc)</t>
+          <t>BNP Paribas Easy ESG Enhanced US UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>QGHY.PA</t>
+          <t>AUSSH.PA</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Alpha Enhanced US UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy ESG Enhanced US UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>QUSAE.PA</t>
+          <t>AUSSD.PA</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Alpha Enhanced US UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy ESG Enhanced World UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>QUSA.PA</t>
+          <t>AWDSE.PA</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Alpha Enhanced USD Corporate Bond UCITS ETF (Acc)</t>
+          <t>BNP Paribas Easy ESG Enhanced World UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>QUIG.PA</t>
+          <t>AWDSH.PA</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Alpha Enhanced World UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy EUR Corporate Bond SRI Fossil Free Ultrashort Duration UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>QGLOE.PA</t>
+          <t>SRIUC.PA</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Alpha Enhanced World UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy EUR Corporate Bond SRI Fossil Free Ultrashort Duration UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
-        <is>
-          <t>QGLO.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy Dividend Europe UCITS ETF</t>
-        </is>
-      </c>
-      <c r="B319" t="inlineStr">
-        <is>
-          <t>EDEU.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ECPI Global ESG Blue Economy UCITS ETF EUR</t>
-        </is>
-      </c>
-      <c r="B320" t="inlineStr">
-        <is>
-          <t>BLUE.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ECPI Global ESG Blue Economy UCITS ETF USD</t>
-        </is>
-      </c>
-      <c r="B321" t="inlineStr">
-        <is>
-          <t>BLUSD.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ECPI Global ESG Infrastructure UCITS ETF EUR Capitalisation</t>
-        </is>
-      </c>
-      <c r="B322" t="inlineStr">
-        <is>
-          <t>ENG.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ECPI Global ESG Infrastructure UCITS ETF USD Capitalisation</t>
-        </is>
-      </c>
-      <c r="B323" t="inlineStr">
-        <is>
-          <t>ENGUS.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced EMU UCITS ETF Acc</t>
-        </is>
-      </c>
-      <c r="B324" t="inlineStr">
-        <is>
-          <t>AEMUS.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2027 UCITS ETF Acc</t>
-        </is>
-      </c>
-      <c r="B325" t="inlineStr">
-        <is>
-          <t>ACE27.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="326">
-      <c r="A326" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2027 UCITS ETF Dist</t>
-        </is>
-      </c>
-      <c r="B326" t="inlineStr">
-        <is>
-          <t>ACD27.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2029 UCITS ETF Acc</t>
-        </is>
-      </c>
-      <c r="B327" t="inlineStr">
-        <is>
-          <t>ACE29.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="328">
-      <c r="A328" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2029 UCITS ETF Dist</t>
-        </is>
-      </c>
-      <c r="B328" t="inlineStr">
-        <is>
-          <t>ACD29.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="329">
-      <c r="A329" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2032 UCITS ETF Acc</t>
-        </is>
-      </c>
-      <c r="B329" t="inlineStr">
-        <is>
-          <t>ACE32.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="330">
-      <c r="A330" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond December 2032 UCITS ETF Dist</t>
-        </is>
-      </c>
-      <c r="B330" t="inlineStr">
-        <is>
-          <t>ACD32.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="331">
-      <c r="A331" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond UCITS ETF Capitalisation</t>
-        </is>
-      </c>
-      <c r="B331" t="inlineStr">
-        <is>
-          <t>SEUCB.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced EUR Corporate Bond UCITS ETF Dist</t>
-        </is>
-      </c>
-      <c r="B332" t="inlineStr">
-        <is>
-          <t>ACESD.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="333">
-      <c r="A333" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced EUR Government Bond UCITS ETF Acc</t>
-        </is>
-      </c>
-      <c r="B333" t="inlineStr">
-        <is>
-          <t>SEUGB.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="334">
-      <c r="A334" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced EUR Government Bond UCITS ETF Distribution</t>
-        </is>
-      </c>
-      <c r="B334" t="inlineStr">
-        <is>
-          <t>AGESD.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="335">
-      <c r="A335" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced Europe UCITS ETF Acc</t>
-        </is>
-      </c>
-      <c r="B335" t="inlineStr">
-        <is>
-          <t>AEUSE.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="336">
-      <c r="A336" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced Japan UCITS ETF EUR Acc</t>
-        </is>
-      </c>
-      <c r="B336" t="inlineStr">
-        <is>
-          <t>AJASE.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="337">
-      <c r="A337" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced Japan UCITS ETF EUR Hedged (Acc)</t>
-        </is>
-      </c>
-      <c r="B337" t="inlineStr">
-        <is>
-          <t>AJASH.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="338">
-      <c r="A338" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced US UCITS ETF EUR Acc</t>
-        </is>
-      </c>
-      <c r="B338" t="inlineStr">
-        <is>
-          <t>AUSSE.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="339">
-      <c r="A339" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced US UCITS ETF EUR Hedged Acc</t>
-        </is>
-      </c>
-      <c r="B339" t="inlineStr">
-        <is>
-          <t>AUSSH.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced US UCITS ETF USD Acc</t>
-        </is>
-      </c>
-      <c r="B340" t="inlineStr">
-        <is>
-          <t>AUSSD.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="341">
-      <c r="A341" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced World UCITS ETF EUR Acc</t>
-        </is>
-      </c>
-      <c r="B341" t="inlineStr">
-        <is>
-          <t>AWDSE.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="342">
-      <c r="A342" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced World UCITS ETF EUR Hedged Acc</t>
-        </is>
-      </c>
-      <c r="B342" t="inlineStr">
-        <is>
-          <t>AWDSH.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced World UCITS ETF USD Acc</t>
-        </is>
-      </c>
-      <c r="B343" t="inlineStr">
-        <is>
-          <t>AWDS.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="344">
-      <c r="A344" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy EUR Corporate Bond SRI Fossil Free 7-10Y UCITS ETF Acc</t>
-        </is>
-      </c>
-      <c r="B344" t="inlineStr">
-        <is>
-          <t>SRIC7.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="345">
-      <c r="A345" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy EUR Corporate Bond SRI Fossil Free 7-10Y UCITS ETF Dist</t>
-        </is>
-      </c>
-      <c r="B345" t="inlineStr">
-        <is>
-          <t>SRID7.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="346">
-      <c r="A346" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy EUR Corporate Bond SRI Fossil Free Ultrashort Duration UCITS ETF Acc</t>
-        </is>
-      </c>
-      <c r="B346" t="inlineStr">
-        <is>
-          <t>SRIUC.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="347">
-      <c r="A347" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy EUR Corporate Bond SRI Fossil Free Ultrashort Duration UCITS ETF Dist</t>
-        </is>
-      </c>
-      <c r="B347" t="inlineStr">
         <is>
           <t>SRIUD.PA</t>
         </is>

</xml_diff>

<commit_message>
feat(etf): AUM-rank enrichment from profiles.jsonl (universe 317 -> ~395)
Add the justETF profiles export and use real AUM to enrich the active universe.

- data/ticker/etf/profiles.jsonl: justETF export (isin, name, category,
  fund_size_eur_mln, ...). No Yahoo ticker, so funds are mapped to tickers by
  exact name against data/ticker/etf/ticker.xlsx.
- etf_profiles.py: load_profiles + profiles_ticker_table — map name->ticker,
  rank by descending fund_size_eur_mln, dedupe (larger AUM wins), take top-N.
- etf_universe.build_active_universe_table gains an `aum_extras` union: the
  active seed is now core + justETF list-order extras + the top-100 funds by
  real AUM, deduped ("if not already there") and KNOWN_DEAD-pruned. Seed grows
  from 317 to ~395 (79 of the top-100 were not already present).

Note: the supplied profiles slice covers EUR 693-995 mln funds (mid-sized),
not the multi-billion giants already in the curated core.
</commit_message>
<xml_diff>
--- a/data/ticker/etf/ticker_active.xlsx
+++ b/data/ticker/etf/ticker_active.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B318"/>
+  <dimension ref="A1:B396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4232,6 +4232,942 @@
         </is>
       </c>
     </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>HSBC MSCI Emerging Markets UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>HEMA.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>iShares EUR Cash UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>YCSH.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI Nordic UCITS ETF 1D</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>XDN0.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>JPMorgan US Research Enhanced Index Equity Active UCITS ETF EUR Hedged (acc)</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>JUHE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>iShares iBonds Dec 2028 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>B28A.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Invesco S&amp;P 500 Equal Weight UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>SPEQ.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Xtrackers S&amp;P 500 Equal Weight Scored &amp; Screened UCITS ETF 2C - EUR Hedged</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>XEWE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>UBS Core MSCI World UCITS ETF hCHF acc</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>WORLD.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Schroder Global Equity Active UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>SAGE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>SXLE.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>iShares STOXX Europe 600 Utilities UCITS ETF (DE)</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>SX6PEX.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>iShares European Property Yield UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>IPRP.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Invesco CoinShares Global Blockchain UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>BCHN.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Global X Copper Miners UCITS ETF USD Accumulating</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>COPX.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>UBS S&amp;P 500 Scored &amp; Screened UCITS ETF hEUR acc</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>5ESGE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>iShares MSCI Korea UCITS ETF (Dist)</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>IKRA.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Minimum Volatility UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>XDEB.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>iShares STOXX Europe 600 UCITS ETF (DE) EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>IEXXF</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>JPMorgan Global Research Enhanced Index Equity (ESG) UCITS ETF EUR Hedged (acc)</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>JRGE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>UBS MSCI AC Asia ex Japan SF UCITS ETF USD acc</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>AJEUAS.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Invesco S&amp;P 500 Equal Weight Swap UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>RSPS.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>L&amp;G Battery Value-Chain UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>BATT.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>iShares MSCI Europe Quality Dividend Advanced UCITS ETF EUR (Dist)</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>QDVX.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>iShares MSCI Europe Health Care Sector UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>ESIH.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>HSBC Multi-Factor Worldwide Equity UCITS ETF USD</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>HWWA.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy MSCI World SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>EMWE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI Japan UCITS ETF 4C - EUR Hedged</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>XMK9.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>iShares EUR Floating Rate Bond Advanced UCITS ETF EUR (Dist)</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>EFRN.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>iShares iBonds Dec 2027 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>IB27.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>PIMCO Euro Short Maturity UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>PJSR.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI Emerging Markets Swap UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>XMEM.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Vanguard ESG Global All Cap UCITS ETF (USD) Accumulating</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>V3AA.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI Japan UCITS ETF JPY Unhedged</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>JPJY.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Utilities UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>XDWU.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI USA Communication Services UCITS ETF 1D</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>XUCM.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>iShares S&amp;P U.S. Banks UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>BNKS.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>EXCD.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>iShares Edge MSCI Europe Minimum Volatility UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>MVEU.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>iShares AI Infrastructure UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>AINF.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Vanguard LifeStrategy 60% Equity UCITS ETF Accumulating</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>V60A.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Consumer Staples UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>XDWS.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>iShares USD High Yield Corporate Bond ESG SRI UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>DHYE.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>iShares Russell 1000 Growth UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>R1GR.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI Europe Utilities UCITS ETF EUR</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>STU.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>iShares MSCI World Information Technology Sector Advanced UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>WITS.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy EURO STOXX 50 UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>ETBB.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>HSBC MSCI Pacific ex Japan UCITS ETF USD</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>HMXJ.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>UBS BBG Commodity CMCI SF UCITS ETF USD acc</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>BCCMA.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>iShares FTSE 250 UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>MIDD.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>UBS Core MSCI EMU UCITS ETF hCHF acc</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>EMUCHF.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>iShares MSCI USA Screened UCITS ETF EUR Hedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>SAUA.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>iShares iBonds Dec 2028 Term USD Corporate UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>D28A.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Financials UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>XDWF.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>State Street SPDR Bloomberg 1-3 Month T-Bill UCITS ETF USD Unhedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>TBIL.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>JPMorgan USD Ultra-Short Income UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>JPSA.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Invesco MDAX UCITS ETF A</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>MDAX.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>HSBC FTSE EPRA NAREIT Developed UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>HPRA.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>JPMorgan EUR Corporate Bond Research Enhanced Index (ESG) UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>JREB.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI USA Health Care UCITS ETF 1D</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>XUHC.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>VAPU.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>iShares MSCI Japan ESG Enhanced CTB UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>EEJD.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>iShares MSCI World ESG Enhanced CTB UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>EEWD.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>iShares Core MSCI EMU UCITS ETF USD Hedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>CEUU.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI World UCITS ETF EUR Hedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>SWRE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Xtrackers Swiss Large Cap UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>XSMC.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>UBS Core MSCI World UCITS ETF hEUR acc</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>WRDE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>UBS Core MSCI USA UCITS ETF EUR Hedged acc</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>USEUWH.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>UBS MSCI World Selection UCITS ETF USD acc</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>WDESG.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI UK ESG UCITS ETF 1D</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>XASX.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>iShares Edge MSCI Europe Quality Factor UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>IEQU.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>STN.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Xtrackers Portfolio UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>XQUI.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI Europe Financials UCITS ETF EUR</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>STZ.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>iShares S&amp;P 500 Consumer Discretionary Sector UCITS ETF (Acc)</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>IUCD.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>Vanguard FTSE 250 UCITS ETF (GBP) Accumulating</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>VMIG.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>BTEC.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>State Street SPDR S&amp;P 500 Quality Aristocrats UCITS ETF USD Unhedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>QUS5.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>iShares MSCI Poland UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>SPOL.SW</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(etf): prune 5 dead tickers from the AUM-enriched run (universe -> 390)
The 395-ticker AUM-enriched cold start downloaded 390/395 (99%) over the same
2016-01-04 -> 2026-07-10 range (592,979 rows). 5 symbols returned no Yahoo data
(BNKS.SW, D28A.AS, EEJD.AS, EEWD.AS, IEXXF); fold them into KNOWN_DEAD.

Regenerated seed is 390 tickers and matches the committed historical parquet
symbols exactly, so no re-backfill is needed.
</commit_message>
<xml_diff>
--- a/data/ticker/etf/ticker_active.xlsx
+++ b/data/ticker/etf/ticker_active.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B396"/>
+  <dimension ref="A1:B391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4439,730 +4439,670 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>iShares STOXX Europe 600 UCITS ETF (DE) EUR (Acc)</t>
+          <t>JPMorgan Global Research Enhanced Index Equity (ESG) UCITS ETF EUR Hedged (acc)</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>IEXXF</t>
+          <t>JRGE.MI</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>JPMorgan Global Research Enhanced Index Equity (ESG) UCITS ETF EUR Hedged (acc)</t>
+          <t>UBS MSCI AC Asia ex Japan SF UCITS ETF USD acc</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>JRGE.MI</t>
+          <t>AJEUAS.MI</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>UBS MSCI AC Asia ex Japan SF UCITS ETF USD acc</t>
+          <t>Invesco S&amp;P 500 Equal Weight Swap UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>AJEUAS.MI</t>
+          <t>RSPS.MI</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>Invesco S&amp;P 500 Equal Weight Swap UCITS ETF Acc</t>
+          <t>L&amp;G Battery Value-Chain UCITS ETF</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>RSPS.MI</t>
+          <t>BATT.AS</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>L&amp;G Battery Value-Chain UCITS ETF</t>
+          <t>iShares MSCI Europe Quality Dividend Advanced UCITS ETF EUR (Dist)</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>BATT.AS</t>
+          <t>QDVX.SW</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>iShares MSCI Europe Quality Dividend Advanced UCITS ETF EUR (Dist)</t>
+          <t>iShares MSCI Europe Health Care Sector UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>QDVX.SW</t>
+          <t>ESIH.L</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>iShares MSCI Europe Health Care Sector UCITS ETF EUR (Acc)</t>
+          <t>HSBC Multi-Factor Worldwide Equity UCITS ETF USD</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>ESIH.L</t>
+          <t>HWWA.L</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>HSBC Multi-Factor Worldwide Equity UCITS ETF USD</t>
+          <t>BNP Paribas Easy MSCI World SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>HWWA.L</t>
+          <t>EMWE.PA</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
+          <t>Xtrackers MSCI Japan UCITS ETF 4C - EUR Hedged</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>EMWE.PA</t>
+          <t>XMK9.MI</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Japan UCITS ETF 4C - EUR Hedged</t>
+          <t>iShares EUR Floating Rate Bond Advanced UCITS ETF EUR (Dist)</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>XMK9.MI</t>
+          <t>EFRN.SW</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>iShares EUR Floating Rate Bond Advanced UCITS ETF EUR (Dist)</t>
+          <t>iShares iBonds Dec 2027 Term EUR Corporate UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>EFRN.SW</t>
+          <t>IB27.PA</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2027 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+          <t>PIMCO Euro Short Maturity UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>IB27.PA</t>
+          <t>PJSR.MI</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>PIMCO Euro Short Maturity UCITS ETF Acc</t>
+          <t>Xtrackers MSCI Emerging Markets Swap UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>PJSR.MI</t>
+          <t>XMEM.MI</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Emerging Markets Swap UCITS ETF 1C</t>
+          <t>Vanguard ESG Global All Cap UCITS ETF (USD) Accumulating</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>XMEM.MI</t>
+          <t>V3AA.AS</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>Vanguard ESG Global All Cap UCITS ETF (USD) Accumulating</t>
+          <t>State Street SPDR MSCI Japan UCITS ETF JPY Unhedged</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>V3AA.AS</t>
+          <t>JPJY.PA</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Japan UCITS ETF JPY Unhedged</t>
+          <t>Xtrackers MSCI World Utilities UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>JPJY.PA</t>
+          <t>XDWU.MI</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Utilities UCITS ETF 1C</t>
+          <t>Xtrackers MSCI USA Communication Services UCITS ETF 1D</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>XDWU.MI</t>
+          <t>XUCM.L</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI USA Communication Services UCITS ETF 1D</t>
+          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>XUCM.L</t>
+          <t>EXCD.AS</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>iShares S&amp;P U.S. Banks UCITS ETF USD (Acc)</t>
+          <t>iShares Edge MSCI Europe Minimum Volatility UCITS ETF</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>BNKS.SW</t>
+          <t>MVEU.MI</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
+          <t>iShares AI Infrastructure UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>EXCD.AS</t>
+          <t>AINF.AS</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI Europe Minimum Volatility UCITS ETF</t>
+          <t>Vanguard LifeStrategy 60% Equity UCITS ETF Accumulating</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>MVEU.MI</t>
+          <t>V60A.AS</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>iShares AI Infrastructure UCITS ETF USD (Acc)</t>
+          <t>Xtrackers MSCI World Consumer Staples UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>AINF.AS</t>
+          <t>XDWS.MI</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>Vanguard LifeStrategy 60% Equity UCITS ETF Accumulating</t>
+          <t>iShares USD High Yield Corporate Bond ESG SRI UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>V60A.AS</t>
+          <t>DHYE.AS</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Consumer Staples UCITS ETF 1C</t>
+          <t>iShares Russell 1000 Growth UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>XDWS.MI</t>
+          <t>R1GR.AS</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>iShares USD High Yield Corporate Bond ESG SRI UCITS ETF USD (Acc)</t>
+          <t>State Street SPDR MSCI Europe Utilities UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>DHYE.AS</t>
+          <t>STU.PA</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>iShares Russell 1000 Growth UCITS ETF USD (Acc)</t>
+          <t>iShares MSCI World Information Technology Sector Advanced UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>R1GR.AS</t>
+          <t>WITS.AS</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Europe Utilities UCITS ETF EUR</t>
+          <t>BNP Paribas Easy EURO STOXX 50 UCITS ETF</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>STU.PA</t>
+          <t>ETBB.PA</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>iShares MSCI World Information Technology Sector Advanced UCITS ETF USD (Dist)</t>
+          <t>HSBC MSCI Pacific ex Japan UCITS ETF USD</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>WITS.AS</t>
+          <t>HMXJ.MI</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy EURO STOXX 50 UCITS ETF</t>
+          <t>UBS BBG Commodity CMCI SF UCITS ETF USD acc</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>ETBB.PA</t>
+          <t>BCCMA.SW</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>HSBC MSCI Pacific ex Japan UCITS ETF USD</t>
+          <t>iShares FTSE 250 UCITS ETF</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>HMXJ.MI</t>
+          <t>MIDD.SW</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>UBS BBG Commodity CMCI SF UCITS ETF USD acc</t>
+          <t>UBS Core MSCI EMU UCITS ETF hCHF acc</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>BCCMA.SW</t>
+          <t>EMUCHF.SW</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>iShares FTSE 250 UCITS ETF</t>
+          <t>iShares MSCI USA Screened UCITS ETF EUR Hedged (Acc)</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>MIDD.SW</t>
+          <t>SAUA.MI</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>UBS Core MSCI EMU UCITS ETF hCHF acc</t>
+          <t>Xtrackers MSCI World Financials UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>EMUCHF.SW</t>
+          <t>XDWF.MI</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>iShares MSCI USA Screened UCITS ETF EUR Hedged (Acc)</t>
+          <t>State Street SPDR Bloomberg 1-3 Month T-Bill UCITS ETF USD Unhedged (Acc)</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>SAUA.MI</t>
+          <t>TBIL.SW</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2028 Term USD Corporate UCITS ETF USD (Acc)</t>
+          <t>JPMorgan USD Ultra-Short Income UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>D28A.AS</t>
+          <t>JPSA.MI</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Financials UCITS ETF 1C</t>
+          <t>Invesco MDAX UCITS ETF A</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>XDWF.MI</t>
+          <t>MDAX.MI</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>State Street SPDR Bloomberg 1-3 Month T-Bill UCITS ETF USD Unhedged (Acc)</t>
+          <t>HSBC FTSE EPRA NAREIT Developed UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>TBIL.SW</t>
+          <t>HPRA.L</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>JPMorgan USD Ultra-Short Income UCITS ETF USD (Acc)</t>
+          <t>JPMorgan EUR Corporate Bond Research Enhanced Index (ESG) UCITS ETF</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>JPSA.MI</t>
+          <t>JREB.MI</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>Invesco MDAX UCITS ETF A</t>
+          <t>Xtrackers MSCI USA Health Care UCITS ETF 1D</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>MDAX.MI</t>
+          <t>XUHC.SW</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>HSBC FTSE EPRA NAREIT Developed UCITS ETF USD (Acc)</t>
+          <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>HPRA.L</t>
+          <t>VAPU.SW</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>JPMorgan EUR Corporate Bond Research Enhanced Index (ESG) UCITS ETF</t>
+          <t>iShares Core MSCI EMU UCITS ETF USD Hedged (Acc)</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>JREB.MI</t>
+          <t>CEUU.AS</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI USA Health Care UCITS ETF 1D</t>
+          <t>State Street SPDR MSCI World UCITS ETF EUR Hedged (Acc)</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>XUHC.SW</t>
+          <t>SWRE.MI</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
+          <t>Xtrackers Swiss Large Cap UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>VAPU.SW</t>
+          <t>XSMC.SW</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>iShares MSCI Japan ESG Enhanced CTB UCITS ETF USD (Dist)</t>
+          <t>UBS Core MSCI World UCITS ETF hEUR acc</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>EEJD.AS</t>
+          <t>WRDE.MI</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>iShares MSCI World ESG Enhanced CTB UCITS ETF USD (Dist)</t>
+          <t>UBS Core MSCI USA UCITS ETF EUR Hedged acc</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>EEWD.AS</t>
+          <t>USEUWH.MI</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>iShares Core MSCI EMU UCITS ETF USD Hedged (Acc)</t>
+          <t>UBS MSCI World Selection UCITS ETF USD acc</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>CEUU.AS</t>
+          <t>WDESG.MI</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI World UCITS ETF EUR Hedged (Acc)</t>
+          <t>Xtrackers MSCI UK ESG UCITS ETF 1D</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>SWRE.MI</t>
+          <t>XASX.L</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>Xtrackers Swiss Large Cap UCITS ETF 1C</t>
+          <t>iShares Edge MSCI Europe Quality Factor UCITS ETF</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>XSMC.SW</t>
+          <t>IEQU.MI</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>UBS Core MSCI World UCITS ETF hEUR acc</t>
+          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>WRDE.MI</t>
+          <t>STN.PA</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>UBS Core MSCI USA UCITS ETF EUR Hedged acc</t>
+          <t>Xtrackers Portfolio UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>USEUWH.MI</t>
+          <t>XQUI.MI</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>UBS MSCI World Selection UCITS ETF USD acc</t>
+          <t>State Street SPDR MSCI Europe Financials UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>WDESG.MI</t>
+          <t>STZ.PA</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI UK ESG UCITS ETF 1D</t>
+          <t>iShares S&amp;P 500 Consumer Discretionary Sector UCITS ETF (Acc)</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>XASX.L</t>
+          <t>IUCD.SW</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI Europe Quality Factor UCITS ETF</t>
+          <t>Vanguard FTSE 250 UCITS ETF (GBP) Accumulating</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>IEQU.MI</t>
+          <t>VMIG.MI</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
+          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>STN.PA</t>
+          <t>BTEC.SW</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>Xtrackers Portfolio UCITS ETF 1C</t>
+          <t>State Street SPDR S&amp;P 500 Quality Aristocrats UCITS ETF USD Unhedged (Acc)</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>XQUI.MI</t>
+          <t>QUS5.SW</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Europe Financials UCITS ETF EUR</t>
+          <t>iShares MSCI Poland UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
-        <is>
-          <t>STZ.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="392">
-      <c r="A392" t="inlineStr">
-        <is>
-          <t>iShares S&amp;P 500 Consumer Discretionary Sector UCITS ETF (Acc)</t>
-        </is>
-      </c>
-      <c r="B392" t="inlineStr">
-        <is>
-          <t>IUCD.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="393">
-      <c r="A393" t="inlineStr">
-        <is>
-          <t>Vanguard FTSE 250 UCITS ETF (GBP) Accumulating</t>
-        </is>
-      </c>
-      <c r="B393" t="inlineStr">
-        <is>
-          <t>VMIG.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="394">
-      <c r="A394" t="inlineStr">
-        <is>
-          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
-        </is>
-      </c>
-      <c r="B394" t="inlineStr">
-        <is>
-          <t>BTEC.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="395">
-      <c r="A395" t="inlineStr">
-        <is>
-          <t>State Street SPDR S&amp;P 500 Quality Aristocrats UCITS ETF USD Unhedged (Acc)</t>
-        </is>
-      </c>
-      <c r="B395" t="inlineStr">
-        <is>
-          <t>QUS5.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="396">
-      <c r="A396" t="inlineStr">
-        <is>
-          <t>iShares MSCI Poland UCITS ETF USD (Acc)</t>
-        </is>
-      </c>
-      <c r="B396" t="inlineStr">
         <is>
           <t>SPOL.SW</t>
         </is>

</xml_diff>

<commit_message>
feat(etf): add 100 more justETF sample ETFs (extra_count 350 -> 450)
Grow the active universe by ~100 list-order justETF extras. Seed regenerates
from 390 to 488 tickers (15 core + justETF extras + AUM top-100, deduped).
Historical backfill for the new tickers runs via the cold-start workflow at
the same 2016-01-01 -> today range.
</commit_message>
<xml_diff>
--- a/data/ticker/etf/ticker_active.xlsx
+++ b/data/ticker/etf/ticker_active.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B391"/>
+  <dimension ref="A1:B489"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4235,874 +4235,2050 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>HSBC MSCI Emerging Markets UCITS ETF USD (Acc)</t>
+          <t>BNP Paribas Easy EUR Corporate Bond SRI PAB 1-3Y UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>HEMA.PA</t>
+          <t>SRI3C.PA</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>iShares EUR Cash UCITS ETF EUR (Acc)</t>
+          <t>BNP Paribas Easy EUR Corporate Bond SRI PAB 1-3Y UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>YCSH.AS</t>
+          <t>SRIC3.PA</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Nordic UCITS ETF 1D</t>
+          <t>BNP Paribas Easy EUR Corporate Bond SRI PAB 3-5Y UCITS ETF</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>XDN0.SW</t>
+          <t>SRIC5.PA</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>JPMorgan US Research Enhanced Index Equity Active UCITS ETF EUR Hedged (acc)</t>
+          <t>BNP Paribas Easy EUR Corporate Bond SRI PAB 3-5Y UCITS ETF</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>JUHE.MI</t>
+          <t>SRIC6.PA</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2028 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+          <t>BNP Paribas Easy EUR Corporate Bond SRI PAB UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>B28A.PA</t>
+          <t>SRIC.PA</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>Invesco S&amp;P 500 Equal Weight UCITS ETF Acc</t>
+          <t>BNP Paribas Easy EUR Corporate Bond SRI PAB UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>SPEQ.MI</t>
+          <t>SRICD.PA</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>Xtrackers S&amp;P 500 Equal Weight Scored &amp; Screened UCITS ETF 2C - EUR Hedged</t>
+          <t>BNP Paribas Easy EUR High Yield SRI Fossil Free UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>XEWE.MI</t>
+          <t>HYSRI.PA</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>UBS Core MSCI World UCITS ETF hCHF acc</t>
+          <t>BNP Paribas Easy EUR High Yield SRI Fossil Free UCITS ETF Dis</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>WORLD.SW</t>
+          <t>HSRID.PA</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>Schroder Global Equity Active UCITS ETF</t>
+          <t>BNP Paribas Easy EUR Overnight UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>SAGE.MI</t>
+          <t>CASHE.PA</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
+          <t>BNP Paribas Easy EUR Overnight UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>SXLE.AS</t>
+          <t>CASHD.PA</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>iShares STOXX Europe 600 Utilities UCITS ETF (DE)</t>
+          <t>BNP Paribas Easy EURO STOXX 50 UCITS ETF</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>SX6PEX.SW</t>
+          <t>ETDD.PA</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>iShares European Property Yield UCITS ETF</t>
+          <t>BNP Paribas Easy EURO STOXX 50 UCITS ETF</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>IPRP.AS</t>
+          <t>ETBB.PA</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>Invesco CoinShares Global Blockchain UCITS ETF Acc</t>
+          <t>BNP Paribas Easy Energy &amp; Metals Enhanced Roll UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>BCHN.MI</t>
+          <t>GSCE.AS</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>Global X Copper Miners UCITS ETF USD Accumulating</t>
+          <t>BNP Paribas Easy Energy &amp; Metals Enhanced Roll UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>COPX.MI</t>
+          <t>EMEH.PA</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>UBS S&amp;P 500 Scored &amp; Screened UCITS ETF hEUR acc</t>
+          <t>BNP Paribas Easy Energy &amp; Metals Enhanced Roll UCITS ETF USD</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>5ESGE.MI</t>
+          <t>GSCU.PA</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>iShares MSCI Korea UCITS ETF (Dist)</t>
+          <t>BNP Paribas Easy FTSE EPRA Nareit Developed Europe Green CTB UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>IKRA.AS</t>
+          <t>GREAL.PA</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Minimum Volatility UCITS ETF 1C</t>
+          <t>BNP Paribas Easy FTSE EPRA Nareit Developed Europe Green CTB UCITS ETF QD Dist</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>XDEB.MI</t>
+          <t>GREAD.PA</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>JPMorgan Global Research Enhanced Index Equity (ESG) UCITS ETF EUR Hedged (acc)</t>
+          <t>BNP Paribas Easy FTSE EPRA Nareit Global Developed Green CTB UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>JRGE.MI</t>
+          <t>GRCTB.PA</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>UBS MSCI AC Asia ex Japan SF UCITS ETF USD acc</t>
+          <t>BNP Paribas Easy FTSE EPRA/NAREIT Eurozone Capped UCITS ETF</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>AJEUAS.MI</t>
+          <t>EEA.PA</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>Invesco S&amp;P 500 Equal Weight Swap UCITS ETF Acc</t>
+          <t>BNP Paribas Easy FTSE EPRA/NAREIT Eurozone Capped UCITS ETF QD</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>RSPS.MI</t>
+          <t>EEE.AS</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>L&amp;G Battery Value-Chain UCITS ETF</t>
+          <t>BNP Paribas Easy Growth Europe UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>BATT.AS</t>
+          <t>EGRO.PA</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>iShares MSCI Europe Quality Dividend Advanced UCITS ETF EUR (Dist)</t>
+          <t>BNP Paribas Easy II EUR Aggregate Bond Opportunities UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>QDVX.SW</t>
+          <t>AEAE.MI</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>iShares MSCI Europe Health Care Sector UCITS ETF EUR (Acc)</t>
+          <t>BNP Paribas Easy II EUR Aggregate Bond Opportunities UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>ESIH.L</t>
+          <t>AEJE.MI</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>HSBC Multi-Factor Worldwide Equity UCITS ETF USD</t>
+          <t>BNP Paribas Easy II EUR Credit PAB Opportunities UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>HWWA.L</t>
+          <t>AIPE.MI</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy II EUR Credit PAB Opportunities UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>EMWE.PA</t>
+          <t>AIDE.MI</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Japan UCITS ETF 4C - EUR Hedged</t>
+          <t>BNP Paribas Easy II Emerging Corp Bond PAB UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>XMK9.MI</t>
+          <t>AICU.MI</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>iShares EUR Floating Rate Bond Advanced UCITS ETF EUR (Dist)</t>
+          <t>BNP Paribas Easy II Emerging Corp Bond PAB UCITS ETF USD Dis</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>EFRN.SW</t>
+          <t>AQDU.MI</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2027 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+          <t>BNP Paribas Easy II Global High Yield Opportunities UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>IB27.PA</t>
+          <t>AGYU.MI</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>PIMCO Euro Short Maturity UCITS ETF Acc</t>
+          <t>BNP Paribas Easy II Global High Yield Opportunities UCITS ETF USD Dist</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>PJSR.MI</t>
+          <t>AIGU.MI</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Emerging Markets Swap UCITS ETF 1C</t>
+          <t>BNP Paribas Easy II Global Inflation-Linked Bond Opportunities UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>XMEM.MI</t>
+          <t>ACPI.MI</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>Vanguard ESG Global All Cap UCITS ETF (USD) Accumulating</t>
+          <t>BNP Paribas Easy II Global Inflation-Linked Bond Opportunities UCITS ETF USD Dist</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>V3AA.AS</t>
+          <t>AFDU.MI</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Japan UCITS ETF JPY Unhedged</t>
+          <t>BNP Paribas Easy II Short Duration Income Opportunities UCITS ETF EUR Hedged Dist</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>JPJY.PA</t>
+          <t>ASHE.MI</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Utilities UCITS ETF 1C</t>
+          <t>BNP Paribas Easy II Short Duration Income Opportunities UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>XDWU.MI</t>
+          <t>ASHU.MI</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI USA Communication Services UCITS ETF 1D</t>
+          <t>BNP Paribas Easy II Short Duration Income Opportunities UCITS ETF USD Dist</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>XUCM.L</t>
+          <t>ASLU.MI</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
+          <t>BNP Paribas Easy II US High Yield Opportunities UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>EXCD.AS</t>
+          <t>AHYU.MI</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI Europe Minimum Volatility UCITS ETF</t>
+          <t>BNP Paribas Easy II US High Yield Opportunities UCITS ETF USD Dist</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>MVEU.MI</t>
+          <t>AIHU.MI</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>iShares AI Infrastructure UCITS ETF USD (Acc)</t>
+          <t>BNP Paribas Easy II USD Credit PAB Opportunities UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>AINF.AS</t>
+          <t>AIPU.MI</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>Vanguard LifeStrategy 60% Equity UCITS ETF Accumulating</t>
+          <t>BNP Paribas Easy Low Volatility Europe UCITS ETF</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>V60A.AS</t>
+          <t>EVOE.PA</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Consumer Staples UCITS ETF 1C</t>
+          <t>BNP Paribas Easy Low Volatility Europe UCITS ETF</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>XDWS.MI</t>
+          <t>VLED.PA</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>iShares USD High Yield Corporate Bond ESG SRI UCITS ETF USD (Acc)</t>
+          <t>BNP Paribas Easy MSCI ACWI SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>DHYE.AS</t>
+          <t>PAACE.PA</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>iShares Russell 1000 Growth UCITS ETF USD (Acc)</t>
+          <t>BNP Paribas Easy MSCI ACWI SRI S-Series PAB 5% Capped UCITS ETF USD C</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>R1GR.AS</t>
+          <t>PAACU.PA</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Europe Utilities UCITS ETF EUR</t>
+          <t>BNP Paribas Easy MSCI ACWI UCITS ETF (Acc)</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>STU.PA</t>
+          <t>ALLC.PA</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>iShares MSCI World Information Technology Sector Advanced UCITS ETF USD (Dist)</t>
+          <t>BNP Paribas Easy MSCI ACWI UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>WITS.AS</t>
+          <t>ALLCE.PA</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy EURO STOXX 50 UCITS ETF</t>
+          <t>BNP Paribas Easy MSCI EMU UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>ETBB.PA</t>
+          <t>EUZON.PA</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>HSBC MSCI Pacific ex Japan UCITS ETF USD</t>
+          <t>BNP Paribas Easy MSCI Emerging UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>HMXJ.MI</t>
+          <t>BRIXU.PA</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>UBS BBG Commodity CMCI SF UCITS ETF USD acc</t>
+          <t>BNP Paribas Easy MSCI Emerging UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>BCCMA.SW</t>
+          <t>BRIX.PA</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>iShares FTSE 250 UCITS ETF</t>
+          <t>BNP Paribas Easy MSCI Emerging ex China UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>MIDD.SW</t>
+          <t>EMGXC.PA</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>UBS Core MSCI EMU UCITS ETF hCHF acc</t>
+          <t>BNP Paribas Easy MSCI Emerging ex China UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>EMUCHF.SW</t>
+          <t>EMEXC.PA</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>iShares MSCI USA Screened UCITS ETF EUR Hedged (Acc)</t>
+          <t>BNP Paribas Easy MSCI Europe UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>SAUA.MI</t>
+          <t>UEFA.PA</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Financials UCITS ETF 1C</t>
+          <t>BNP Paribas Easy MSCI Japan Min TE UCITS ETF</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>XDWF.MI</t>
+          <t>EJAP.PA</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>State Street SPDR Bloomberg 1-3 Month T-Bill UCITS ETF USD Unhedged (Acc)</t>
+          <t>BNP Paribas Easy MSCI Japan Min TE UCITS ETF EUR Hedged</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>TBIL.SW</t>
+          <t>EJAH.PA</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>JPMorgan USD Ultra-Short Income UCITS ETF USD (Acc)</t>
+          <t>BNP Paribas Easy MSCI Japan Min TE UCITS ETF USD</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>JPSA.MI</t>
+          <t>EJAPU.PA</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>Invesco MDAX UCITS ETF A</t>
+          <t>BNP Paribas Easy MSCI Japan SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>MDAX.MI</t>
+          <t>SRIJC.PA</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>HSBC FTSE EPRA NAREIT Developed UCITS ETF USD (Acc)</t>
+          <t>BNP Paribas Easy MSCI Japan SRI S-Series PAB 5% Capped UCITS ETF EUR Dis</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>HPRA.L</t>
+          <t>SRIJ.PA</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>JPMorgan EUR Corporate Bond Research Enhanced Index (ESG) UCITS ETF</t>
+          <t>BNP Paribas Easy MSCI Japan UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>JREB.MI</t>
+          <t>FUJI.PA</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI USA Health Care UCITS ETF 1D</t>
+          <t>BNP Paribas Easy MSCI USA Min TE UCITS ETF</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>XUHC.SW</t>
+          <t>ENAM.PA</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
+          <t>BNP Paribas Easy MSCI USA SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>VAPU.SW</t>
+          <t>EKLDC.PA</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>iShares Core MSCI EMU UCITS ETF USD Hedged (Acc)</t>
+          <t>BNP Paribas Easy MSCI USA SRI S-Series PAB 5% Capped UCITS ETF EUR Dis</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>CEUU.AS</t>
+          <t>EKUS.PA</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI World UCITS ETF EUR Hedged (Acc)</t>
+          <t>BNP Paribas Easy MSCI USA SRI S-Series PAB 5% Capped UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>SWRE.MI</t>
+          <t>EKLD.PA</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>Xtrackers Swiss Large Cap UCITS ETF 1C</t>
+          <t>BNP Paribas Easy MSCI USA UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>XSMC.SW</t>
+          <t>BIGUS.PA</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>UBS Core MSCI World UCITS ETF hEUR acc</t>
+          <t>BNP Paribas Easy MSCI USA UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>WRDE.MI</t>
+          <t>BGUS.PA</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>UBS Core MSCI USA UCITS ETF EUR Hedged acc</t>
+          <t>BNP Paribas Easy MSCI World Equal Weight Select UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>USEUWH.MI</t>
+          <t>WEWEU.PA</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>UBS MSCI World Selection UCITS ETF USD acc</t>
+          <t>BNP Paribas Easy MSCI World Equal Weight Select UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>WDESG.MI</t>
+          <t>WEWE.PA</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI UK ESG UCITS ETF 1D</t>
+          <t>BNP Paribas Easy MSCI World II UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>XASX.L</t>
+          <t>GLOBU.PA</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI Europe Quality Factor UCITS ETF</t>
+          <t>BNP Paribas Easy MSCI World II UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>IEQU.MI</t>
+          <t>GLOBD.PA</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
+          <t>BNP Paribas Easy MSCI World II UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>STN.PA</t>
+          <t>GLOEU.PA</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>Xtrackers Portfolio UCITS ETF 1C</t>
+          <t>BNP Paribas Easy MSCI World Min TE UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>XQUI.MI</t>
+          <t>WEMT2.PA</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Europe Financials UCITS ETF EUR</t>
+          <t>BNP Paribas Easy MSCI World Min TE UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>STZ.PA</t>
+          <t>WEMTH.PA</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>iShares S&amp;P 500 Consumer Discretionary Sector UCITS ETF (Acc)</t>
+          <t>BNP Paribas Easy MSCI World Min TE UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>IUCD.SW</t>
+          <t>WEMTE.PA</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>Vanguard FTSE 250 UCITS ETF (GBP) Accumulating</t>
+          <t>BNP Paribas Easy MSCI World SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>VMIG.MI</t>
+          <t>EMWE.PA</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
+          <t>BNP Paribas Easy MSCI World SRI S-Series PAB 5% Capped UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>BTEC.SW</t>
+          <t>EMWD.PA</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>State Street SPDR S&amp;P 500 Quality Aristocrats UCITS ETF USD Unhedged (Acc)</t>
+          <t>BNP Paribas Easy MSCI World SRI S-Series PAB 5% Capped UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>QUS5.SW</t>
+          <t>EWRD.PA</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
+          <t>BNP Paribas Easy MSCI World UCITS ETF EUR Acc</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>WETFE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy MSCI World UCITS ETF USD Acc</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>WETF.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy Quality Europe UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>EQUA.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy Quality Europe UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>QUED.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy S&amp;P 500 II UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>SPTRE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy S&amp;P 500 II UCITS ETF EUR Hedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>SPTRH.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy S&amp;P 500 II UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>SPTR.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy S&amp;P 500 II UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>EDEC.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy S&amp;P 500 Scored and Screened UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>SPEUS.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy S&amp;P 500 Scored and Screened UCITS ETF EUR Acc</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>SPEEU.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy S&amp;P 500 Scored and Screened UCITS ETF EUR Hedged Acc</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>SPEUH.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy S&amp;P 500 UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>ESDD.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy S&amp;P 500 UCITS ETF EUR</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>ESE.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy S&amp;P 500 UCITS ETF EUR Hedged</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>ESEH.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy S&amp;P 500 UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>ESD.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy STOXX Europe 600 UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>ETZ.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy STOXX Europe 600 UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>ETZD.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy USD Corporate Bond SRI Fossil Free UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>USCBC.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>BNP Paribas Easy USD Corporate Bond SRI Fossil Free UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>USCBD.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Bellevue Healthcare UCITS ETF USD Acc</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>CARE.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Bitwise Aptos Staking ETP</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>APTB.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Bitwise Celestia Staking ETP</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>TIAB.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Bitwise Core Bitcoin ETP</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>BTC2.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Bitwise Diaman Bitcoin &amp; Gold ETP</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>BTCG.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Bitwise Ethereum Staking ETP</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>ET32.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>Bitwise MSCI Digital Assets Select 20 ETP</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>DA20.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Bitwise Physical Bitcoin ETP</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>BTCE.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Bitwise Physical Ethereum ETP</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>ZETH.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>HSBC MSCI Emerging Markets UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>HEMA.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>iShares EUR Cash UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>YCSH.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI Nordic UCITS ETF 1D</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>XDN0.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>JPMorgan US Research Enhanced Index Equity Active UCITS ETF EUR Hedged (acc)</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>JUHE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>iShares iBonds Dec 2028 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>B28A.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>Invesco S&amp;P 500 Equal Weight UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>SPEQ.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Xtrackers S&amp;P 500 Equal Weight Scored &amp; Screened UCITS ETF 2C - EUR Hedged</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>XEWE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>UBS Core MSCI World UCITS ETF hCHF acc</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>WORLD.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>Schroder Global Equity Active UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>SAGE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>SXLE.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>iShares STOXX Europe 600 Utilities UCITS ETF (DE)</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>SX6PEX.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>iShares European Property Yield UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>IPRP.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Invesco CoinShares Global Blockchain UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>BCHN.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Global X Copper Miners UCITS ETF USD Accumulating</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>COPX.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>UBS S&amp;P 500 Scored &amp; Screened UCITS ETF hEUR acc</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>5ESGE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>iShares MSCI Korea UCITS ETF (Dist)</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>IKRA.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Minimum Volatility UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>XDEB.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>JPMorgan Global Research Enhanced Index Equity (ESG) UCITS ETF EUR Hedged (acc)</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>JRGE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>UBS MSCI AC Asia ex Japan SF UCITS ETF USD acc</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>AJEUAS.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>Invesco S&amp;P 500 Equal Weight Swap UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>RSPS.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>L&amp;G Battery Value-Chain UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>BATT.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>iShares MSCI Europe Quality Dividend Advanced UCITS ETF EUR (Dist)</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>QDVX.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>iShares MSCI Europe Health Care Sector UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>ESIH.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>HSBC Multi-Factor Worldwide Equity UCITS ETF USD</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>HWWA.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI Japan UCITS ETF 4C - EUR Hedged</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>XMK9.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>iShares EUR Floating Rate Bond Advanced UCITS ETF EUR (Dist)</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>EFRN.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>iShares iBonds Dec 2027 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>IB27.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>PIMCO Euro Short Maturity UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>PJSR.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI Emerging Markets Swap UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>XMEM.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>Vanguard ESG Global All Cap UCITS ETF (USD) Accumulating</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>V3AA.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI Japan UCITS ETF JPY Unhedged</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>JPJY.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Utilities UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>XDWU.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI USA Communication Services UCITS ETF 1D</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>XUCM.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>EXCD.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>iShares Edge MSCI Europe Minimum Volatility UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>MVEU.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>iShares AI Infrastructure UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>AINF.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Vanguard LifeStrategy 60% Equity UCITS ETF Accumulating</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>V60A.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Consumer Staples UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>XDWS.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>iShares USD High Yield Corporate Bond ESG SRI UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>DHYE.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>iShares Russell 1000 Growth UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>R1GR.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI Europe Utilities UCITS ETF EUR</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>STU.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>iShares MSCI World Information Technology Sector Advanced UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>WITS.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>HSBC MSCI Pacific ex Japan UCITS ETF USD</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>HMXJ.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>UBS BBG Commodity CMCI SF UCITS ETF USD acc</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>BCCMA.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>iShares FTSE 250 UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>MIDD.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>UBS Core MSCI EMU UCITS ETF hCHF acc</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>EMUCHF.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>iShares MSCI USA Screened UCITS ETF EUR Hedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>SAUA.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Financials UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>XDWF.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>State Street SPDR Bloomberg 1-3 Month T-Bill UCITS ETF USD Unhedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>TBIL.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>JPMorgan USD Ultra-Short Income UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>JPSA.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Invesco MDAX UCITS ETF A</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>MDAX.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>HSBC FTSE EPRA NAREIT Developed UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>HPRA.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>JPMorgan EUR Corporate Bond Research Enhanced Index (ESG) UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>JREB.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI USA Health Care UCITS ETF 1D</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>XUHC.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>VAPU.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>iShares Core MSCI EMU UCITS ETF USD Hedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>CEUU.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI World UCITS ETF EUR Hedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>SWRE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>Xtrackers Swiss Large Cap UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>XSMC.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>UBS Core MSCI World UCITS ETF hEUR acc</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>WRDE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>UBS Core MSCI USA UCITS ETF EUR Hedged acc</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>USEUWH.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>UBS MSCI World Selection UCITS ETF USD acc</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>WDESG.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI UK ESG UCITS ETF 1D</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>XASX.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>iShares Edge MSCI Europe Quality Factor UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>IEQU.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>STN.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Xtrackers Portfolio UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>XQUI.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI Europe Financials UCITS ETF EUR</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>STZ.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>iShares S&amp;P 500 Consumer Discretionary Sector UCITS ETF (Acc)</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>IUCD.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>Vanguard FTSE 250 UCITS ETF (GBP) Accumulating</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>VMIG.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>BTEC.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>State Street SPDR S&amp;P 500 Quality Aristocrats UCITS ETF USD Unhedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>QUS5.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
           <t>iShares MSCI Poland UCITS ETF USD (Acc)</t>
         </is>
       </c>
-      <c r="B391" t="inlineStr">
+      <c r="B489" t="inlineStr">
         <is>
           <t>SPOL.SW</t>
         </is>

</xml_diff>

<commit_message>
fix(etf): prune 17 dead tickers from the 488-ticker run (universe -> 471)
The extra_count=450 cold-start downloaded 471/488 (97%), 681,301 rows, range
2016-01-04 -> 2026-07-13. 17 symbols returned no Yahoo data (crypto ETPs and
thin .PA/.AS listings); fold them into KNOWN_DEAD.

Regenerated seed is 471 tickers and matches the committed historical parquet
symbols exactly, so no re-backfill is needed.
</commit_message>
<xml_diff>
--- a/data/ticker/etf/ticker_active.xlsx
+++ b/data/ticker/etf/ticker_active.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B489"/>
+  <dimension ref="A1:B472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4343,12 +4343,12 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy EUR Overnight UCITS ETF Dist</t>
+          <t>BNP Paribas Easy EURO STOXX 50 UCITS ETF</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>CASHD.PA</t>
+          <t>ETDD.PA</t>
         </is>
       </c>
     </row>
@@ -4360,19 +4360,19 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>ETDD.PA</t>
+          <t>ETBB.PA</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy EURO STOXX 50 UCITS ETF</t>
+          <t>BNP Paribas Easy Energy &amp; Metals Enhanced Roll UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>ETBB.PA</t>
+          <t>GSCE.AS</t>
         </is>
       </c>
     </row>
@@ -4384,1901 +4384,1697 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>GSCE.AS</t>
+          <t>EMEH.PA</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Energy &amp; Metals Enhanced Roll UCITS ETF EUR</t>
+          <t>BNP Paribas Easy Energy &amp; Metals Enhanced Roll UCITS ETF USD</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>EMEH.PA</t>
+          <t>GSCU.PA</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Energy &amp; Metals Enhanced Roll UCITS ETF USD</t>
+          <t>BNP Paribas Easy FTSE EPRA Nareit Developed Europe Green CTB UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>GSCU.PA</t>
+          <t>GREAL.PA</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy FTSE EPRA Nareit Developed Europe Green CTB UCITS ETF Acc</t>
+          <t>BNP Paribas Easy FTSE EPRA Nareit Developed Europe Green CTB UCITS ETF QD Dist</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>GREAL.PA</t>
+          <t>GREAD.PA</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy FTSE EPRA Nareit Developed Europe Green CTB UCITS ETF QD Dist</t>
+          <t>BNP Paribas Easy FTSE EPRA Nareit Global Developed Green CTB UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>GREAD.PA</t>
+          <t>GRCTB.PA</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy FTSE EPRA Nareit Global Developed Green CTB UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy FTSE EPRA/NAREIT Eurozone Capped UCITS ETF</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>GRCTB.PA</t>
+          <t>EEA.PA</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy FTSE EPRA/NAREIT Eurozone Capped UCITS ETF</t>
+          <t>BNP Paribas Easy Growth Europe UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>EEA.PA</t>
+          <t>EGRO.PA</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy FTSE EPRA/NAREIT Eurozone Capped UCITS ETF QD</t>
+          <t>BNP Paribas Easy II EUR Aggregate Bond Opportunities UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>EEE.AS</t>
+          <t>AEAE.MI</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Growth Europe UCITS ETF Acc</t>
+          <t>BNP Paribas Easy II EUR Aggregate Bond Opportunities UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>EGRO.PA</t>
+          <t>AEJE.MI</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II EUR Aggregate Bond Opportunities UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy II EUR Credit PAB Opportunities UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>AEAE.MI</t>
+          <t>AIPE.MI</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II EUR Aggregate Bond Opportunities UCITS ETF EUR Dist</t>
+          <t>BNP Paribas Easy II EUR Credit PAB Opportunities UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>AEJE.MI</t>
+          <t>AIDE.MI</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II EUR Credit PAB Opportunities UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy II Emerging Corp Bond PAB UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>AIPE.MI</t>
+          <t>AICU.MI</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II EUR Credit PAB Opportunities UCITS ETF EUR Dist</t>
+          <t>BNP Paribas Easy II Emerging Corp Bond PAB UCITS ETF USD Dis</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>AIDE.MI</t>
+          <t>AQDU.MI</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II Emerging Corp Bond PAB UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy II Global High Yield Opportunities UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>AICU.MI</t>
+          <t>AGYU.MI</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II Emerging Corp Bond PAB UCITS ETF USD Dis</t>
+          <t>BNP Paribas Easy II Global High Yield Opportunities UCITS ETF USD Dist</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>AQDU.MI</t>
+          <t>AIGU.MI</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II Global High Yield Opportunities UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy II Global Inflation-Linked Bond Opportunities UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>AGYU.MI</t>
+          <t>ACPI.MI</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II Global High Yield Opportunities UCITS ETF USD Dist</t>
+          <t>BNP Paribas Easy II Global Inflation-Linked Bond Opportunities UCITS ETF USD Dist</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>AIGU.MI</t>
+          <t>AFDU.MI</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II Global Inflation-Linked Bond Opportunities UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy II Short Duration Income Opportunities UCITS ETF EUR Hedged Dist</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>ACPI.MI</t>
+          <t>ASHE.MI</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II Global Inflation-Linked Bond Opportunities UCITS ETF USD Dist</t>
+          <t>BNP Paribas Easy II Short Duration Income Opportunities UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>AFDU.MI</t>
+          <t>ASHU.MI</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II Short Duration Income Opportunities UCITS ETF EUR Hedged Dist</t>
+          <t>BNP Paribas Easy II Short Duration Income Opportunities UCITS ETF USD Dist</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>ASHE.MI</t>
+          <t>ASLU.MI</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II Short Duration Income Opportunities UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy II US High Yield Opportunities UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>ASHU.MI</t>
+          <t>AHYU.MI</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II Short Duration Income Opportunities UCITS ETF USD Dist</t>
+          <t>BNP Paribas Easy II US High Yield Opportunities UCITS ETF USD Dist</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>ASLU.MI</t>
+          <t>AIHU.MI</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II US High Yield Opportunities UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy II USD Credit PAB Opportunities UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>AHYU.MI</t>
+          <t>AIPU.MI</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II US High Yield Opportunities UCITS ETF USD Dist</t>
+          <t>BNP Paribas Easy Low Volatility Europe UCITS ETF</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>AIHU.MI</t>
+          <t>EVOE.PA</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy II USD Credit PAB Opportunities UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy Low Volatility Europe UCITS ETF</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>AIPU.MI</t>
+          <t>VLED.PA</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Low Volatility Europe UCITS ETF</t>
+          <t>BNP Paribas Easy MSCI ACWI SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>EVOE.PA</t>
+          <t>PAACE.PA</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Low Volatility Europe UCITS ETF</t>
+          <t>BNP Paribas Easy MSCI ACWI SRI S-Series PAB 5% Capped UCITS ETF USD C</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>VLED.PA</t>
+          <t>PAACU.PA</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI ACWI SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy MSCI ACWI UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>PAACE.PA</t>
+          <t>ALLCE.PA</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI ACWI SRI S-Series PAB 5% Capped UCITS ETF USD C</t>
+          <t>BNP Paribas Easy MSCI EMU UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>PAACU.PA</t>
+          <t>EUZON.PA</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI ACWI UCITS ETF (Acc)</t>
+          <t>BNP Paribas Easy MSCI Emerging UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>ALLC.PA</t>
+          <t>BRIX.PA</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI ACWI UCITS ETF EUR (Acc)</t>
+          <t>BNP Paribas Easy MSCI Europe UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>ALLCE.PA</t>
+          <t>UEFA.PA</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI EMU UCITS ETF Acc</t>
+          <t>BNP Paribas Easy MSCI Japan Min TE UCITS ETF</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>EUZON.PA</t>
+          <t>EJAP.PA</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI Emerging UCITS ETF Acc</t>
+          <t>BNP Paribas Easy MSCI Japan Min TE UCITS ETF EUR Hedged</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>BRIXU.PA</t>
+          <t>EJAH.PA</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI Emerging UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy MSCI Japan Min TE UCITS ETF USD</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>BRIX.PA</t>
+          <t>EJAPU.PA</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI Emerging ex China UCITS ETF Acc</t>
+          <t>BNP Paribas Easy MSCI Japan SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>EMGXC.PA</t>
+          <t>SRIJC.PA</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI Emerging ex China UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy MSCI Japan SRI S-Series PAB 5% Capped UCITS ETF EUR Dis</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>EMEXC.PA</t>
+          <t>SRIJ.PA</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI Europe UCITS ETF Acc</t>
+          <t>BNP Paribas Easy MSCI Japan UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>UEFA.PA</t>
+          <t>FUJI.PA</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI Japan Min TE UCITS ETF</t>
+          <t>BNP Paribas Easy MSCI USA Min TE UCITS ETF</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>EJAP.PA</t>
+          <t>ENAM.PA</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI Japan Min TE UCITS ETF EUR Hedged</t>
+          <t>BNP Paribas Easy MSCI USA SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>EJAH.PA</t>
+          <t>EKLDC.PA</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI Japan Min TE UCITS ETF USD</t>
+          <t>BNP Paribas Easy MSCI USA SRI S-Series PAB 5% Capped UCITS ETF EUR Dis</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>EJAPU.PA</t>
+          <t>EKUS.PA</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI Japan SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy MSCI USA SRI S-Series PAB 5% Capped UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>SRIJC.PA</t>
+          <t>EKLD.PA</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI Japan SRI S-Series PAB 5% Capped UCITS ETF EUR Dis</t>
+          <t>BNP Paribas Easy MSCI USA UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>SRIJ.PA</t>
+          <t>BIGUS.PA</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI Japan UCITS ETF Acc</t>
+          <t>BNP Paribas Easy MSCI World Equal Weight Select UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>FUJI.PA</t>
+          <t>WEWEU.PA</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI USA Min TE UCITS ETF</t>
+          <t>BNP Paribas Easy MSCI World II UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>ENAM.PA</t>
+          <t>GLOEU.PA</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI USA SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy MSCI World Min TE UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>EKLDC.PA</t>
+          <t>WEMT2.PA</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI USA SRI S-Series PAB 5% Capped UCITS ETF EUR Dis</t>
+          <t>BNP Paribas Easy MSCI World Min TE UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>EKUS.PA</t>
+          <t>WEMTH.PA</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI USA SRI S-Series PAB 5% Capped UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy MSCI World Min TE UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>EKLD.PA</t>
+          <t>WEMTE.PA</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI USA UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy MSCI World SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>BIGUS.PA</t>
+          <t>EMWE.PA</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI USA UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy MSCI World SRI S-Series PAB 5% Capped UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>BGUS.PA</t>
+          <t>EMWD.PA</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World Equal Weight Select UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy MSCI World SRI S-Series PAB 5% Capped UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>WEWEU.PA</t>
+          <t>EWRD.PA</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World Equal Weight Select UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy MSCI World UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>WEWE.PA</t>
+          <t>WETFE.PA</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World II UCITS ETF Acc</t>
+          <t>BNP Paribas Easy Quality Europe UCITS ETF</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>GLOBU.PA</t>
+          <t>EQUA.PA</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World II UCITS ETF Dist</t>
+          <t>BNP Paribas Easy Quality Europe UCITS ETF</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>GLOBD.PA</t>
+          <t>QUED.PA</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World II UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy S&amp;P 500 II UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>GLOEU.PA</t>
+          <t>SPTRE.PA</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World Min TE UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy S&amp;P 500 II UCITS ETF EUR Hedged (Acc)</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>WEMT2.PA</t>
+          <t>SPTRH.PA</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World Min TE UCITS ETF EUR Hedged Acc</t>
+          <t>BNP Paribas Easy S&amp;P 500 Scored and Screened UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>WEMTH.PA</t>
+          <t>SPEUS.PA</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World Min TE UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy S&amp;P 500 Scored and Screened UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>WEMTE.PA</t>
+          <t>SPEEU.PA</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World SRI S-Series PAB 5% Capped UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy S&amp;P 500 Scored and Screened UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>EMWE.PA</t>
+          <t>SPEUH.PA</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World SRI S-Series PAB 5% Capped UCITS ETF EUR Dist</t>
+          <t>BNP Paribas Easy S&amp;P 500 UCITS ETF</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>EMWD.PA</t>
+          <t>ESDD.PA</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World SRI S-Series PAB 5% Capped UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy S&amp;P 500 UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>EWRD.PA</t>
+          <t>ESE.PA</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World UCITS ETF EUR Acc</t>
+          <t>BNP Paribas Easy S&amp;P 500 UCITS ETF EUR Hedged</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>WETFE.PA</t>
+          <t>ESEH.PA</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI World UCITS ETF USD Acc</t>
+          <t>BNP Paribas Easy S&amp;P 500 UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>WETF.PA</t>
+          <t>ESD.PA</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Quality Europe UCITS ETF</t>
+          <t>BNP Paribas Easy STOXX Europe 600 UCITS ETF</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>EQUA.PA</t>
+          <t>ETZ.PA</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Quality Europe UCITS ETF</t>
+          <t>BNP Paribas Easy STOXX Europe 600 UCITS ETF</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>QUED.PA</t>
+          <t>ETZD.PA</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy S&amp;P 500 II UCITS ETF EUR (Acc)</t>
+          <t>BNP Paribas Easy USD Corporate Bond SRI Fossil Free UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>SPTRE.PA</t>
+          <t>USCBC.PA</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy S&amp;P 500 II UCITS ETF EUR Hedged (Acc)</t>
+          <t>BNP Paribas Easy USD Corporate Bond SRI Fossil Free UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>SPTRH.PA</t>
+          <t>USCBD.PA</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy S&amp;P 500 II UCITS ETF USD (Acc)</t>
+          <t>Bellevue Healthcare UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>SPTR.PA</t>
+          <t>CARE.SW</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy S&amp;P 500 II UCITS ETF USD (Dist)</t>
+          <t>Bitwise Aptos Staking ETP</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>EDEC.PA</t>
+          <t>APTB.SW</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy S&amp;P 500 Scored and Screened UCITS ETF Acc</t>
+          <t>Bitwise Celestia Staking ETP</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>SPEUS.PA</t>
+          <t>TIAB.PA</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy S&amp;P 500 Scored and Screened UCITS ETF EUR Acc</t>
+          <t>Bitwise Core Bitcoin ETP</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>SPEEU.PA</t>
+          <t>BTC2.AS</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy S&amp;P 500 Scored and Screened UCITS ETF EUR Hedged Acc</t>
+          <t>Bitwise Ethereum Staking ETP</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>SPEUH.PA</t>
+          <t>ET32.PA</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy S&amp;P 500 UCITS ETF</t>
+          <t>HSBC MSCI Emerging Markets UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>ESDD.PA</t>
+          <t>HEMA.PA</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy S&amp;P 500 UCITS ETF EUR</t>
+          <t>iShares EUR Cash UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>ESE.PA</t>
+          <t>YCSH.AS</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy S&amp;P 500 UCITS ETF EUR Hedged</t>
+          <t>Xtrackers MSCI Nordic UCITS ETF 1D</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>ESEH.PA</t>
+          <t>XDN0.SW</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy S&amp;P 500 UCITS ETF USD (Acc)</t>
+          <t>JPMorgan US Research Enhanced Index Equity Active UCITS ETF EUR Hedged (acc)</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>ESD.PA</t>
+          <t>JUHE.MI</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy STOXX Europe 600 UCITS ETF</t>
+          <t>iShares iBonds Dec 2028 Term EUR Corporate UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>ETZ.PA</t>
+          <t>B28A.PA</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy STOXX Europe 600 UCITS ETF</t>
+          <t>Invesco S&amp;P 500 Equal Weight UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>ETZD.PA</t>
+          <t>SPEQ.MI</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy USD Corporate Bond SRI Fossil Free UCITS ETF Acc</t>
+          <t>Xtrackers S&amp;P 500 Equal Weight Scored &amp; Screened UCITS ETF 2C - EUR Hedged</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>USCBC.PA</t>
+          <t>XEWE.MI</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy USD Corporate Bond SRI Fossil Free UCITS ETF Dist</t>
+          <t>UBS Core MSCI World UCITS ETF hCHF acc</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>USCBD.PA</t>
+          <t>WORLD.SW</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>Bellevue Healthcare UCITS ETF USD Acc</t>
+          <t>Schroder Global Equity Active UCITS ETF</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>CARE.SW</t>
+          <t>SAGE.MI</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>Bitwise Aptos Staking ETP</t>
+          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>APTB.SW</t>
+          <t>SXLE.AS</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>Bitwise Celestia Staking ETP</t>
+          <t>iShares STOXX Europe 600 Utilities UCITS ETF (DE)</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>TIAB.PA</t>
+          <t>SX6PEX.SW</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>Bitwise Core Bitcoin ETP</t>
+          <t>iShares European Property Yield UCITS ETF</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>BTC2.AS</t>
+          <t>IPRP.AS</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>Bitwise Diaman Bitcoin &amp; Gold ETP</t>
+          <t>Invesco CoinShares Global Blockchain UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>BTCG.AS</t>
+          <t>BCHN.MI</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>Bitwise Ethereum Staking ETP</t>
+          <t>Global X Copper Miners UCITS ETF USD Accumulating</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>ET32.PA</t>
+          <t>COPX.MI</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>Bitwise MSCI Digital Assets Select 20 ETP</t>
+          <t>UBS S&amp;P 500 Scored &amp; Screened UCITS ETF hEUR acc</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>DA20.PA</t>
+          <t>5ESGE.MI</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>Bitwise Physical Bitcoin ETP</t>
+          <t>iShares MSCI Korea UCITS ETF (Dist)</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>BTCE.AS</t>
+          <t>IKRA.AS</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>Bitwise Physical Ethereum ETP</t>
+          <t>Xtrackers MSCI World Minimum Volatility UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>ZETH.AS</t>
+          <t>XDEB.MI</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>HSBC MSCI Emerging Markets UCITS ETF USD (Acc)</t>
+          <t>JPMorgan Global Research Enhanced Index Equity (ESG) UCITS ETF EUR Hedged (acc)</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>HEMA.PA</t>
+          <t>JRGE.MI</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>iShares EUR Cash UCITS ETF EUR (Acc)</t>
+          <t>UBS MSCI AC Asia ex Japan SF UCITS ETF USD acc</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>YCSH.AS</t>
+          <t>AJEUAS.MI</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Nordic UCITS ETF 1D</t>
+          <t>Invesco S&amp;P 500 Equal Weight Swap UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>XDN0.SW</t>
+          <t>RSPS.MI</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>JPMorgan US Research Enhanced Index Equity Active UCITS ETF EUR Hedged (acc)</t>
+          <t>L&amp;G Battery Value-Chain UCITS ETF</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>JUHE.MI</t>
+          <t>BATT.AS</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2028 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+          <t>iShares MSCI Europe Quality Dividend Advanced UCITS ETF EUR (Dist)</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>B28A.PA</t>
+          <t>QDVX.SW</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>Invesco S&amp;P 500 Equal Weight UCITS ETF Acc</t>
+          <t>iShares MSCI Europe Health Care Sector UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>SPEQ.MI</t>
+          <t>ESIH.L</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>Xtrackers S&amp;P 500 Equal Weight Scored &amp; Screened UCITS ETF 2C - EUR Hedged</t>
+          <t>HSBC Multi-Factor Worldwide Equity UCITS ETF USD</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>XEWE.MI</t>
+          <t>HWWA.L</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>UBS Core MSCI World UCITS ETF hCHF acc</t>
+          <t>Xtrackers MSCI Japan UCITS ETF 4C - EUR Hedged</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>WORLD.SW</t>
+          <t>XMK9.MI</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>Schroder Global Equity Active UCITS ETF</t>
+          <t>iShares EUR Floating Rate Bond Advanced UCITS ETF EUR (Dist)</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>SAGE.MI</t>
+          <t>EFRN.SW</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
+          <t>iShares iBonds Dec 2027 Term EUR Corporate UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>SXLE.AS</t>
+          <t>IB27.PA</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>iShares STOXX Europe 600 Utilities UCITS ETF (DE)</t>
+          <t>PIMCO Euro Short Maturity UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>SX6PEX.SW</t>
+          <t>PJSR.MI</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>iShares European Property Yield UCITS ETF</t>
+          <t>Xtrackers MSCI Emerging Markets Swap UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>IPRP.AS</t>
+          <t>XMEM.MI</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>Invesco CoinShares Global Blockchain UCITS ETF Acc</t>
+          <t>Vanguard ESG Global All Cap UCITS ETF (USD) Accumulating</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>BCHN.MI</t>
+          <t>V3AA.AS</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>Global X Copper Miners UCITS ETF USD Accumulating</t>
+          <t>State Street SPDR MSCI Japan UCITS ETF JPY Unhedged</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>COPX.MI</t>
+          <t>JPJY.PA</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>UBS S&amp;P 500 Scored &amp; Screened UCITS ETF hEUR acc</t>
+          <t>Xtrackers MSCI World Utilities UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>5ESGE.MI</t>
+          <t>XDWU.MI</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>iShares MSCI Korea UCITS ETF (Dist)</t>
+          <t>Xtrackers MSCI USA Communication Services UCITS ETF 1D</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>IKRA.AS</t>
+          <t>XUCM.L</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Minimum Volatility UCITS ETF 1C</t>
+          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>XDEB.MI</t>
+          <t>EXCD.AS</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>JPMorgan Global Research Enhanced Index Equity (ESG) UCITS ETF EUR Hedged (acc)</t>
+          <t>iShares Edge MSCI Europe Minimum Volatility UCITS ETF</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>JRGE.MI</t>
+          <t>MVEU.MI</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>UBS MSCI AC Asia ex Japan SF UCITS ETF USD acc</t>
+          <t>iShares AI Infrastructure UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>AJEUAS.MI</t>
+          <t>AINF.AS</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>Invesco S&amp;P 500 Equal Weight Swap UCITS ETF Acc</t>
+          <t>Vanguard LifeStrategy 60% Equity UCITS ETF Accumulating</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>RSPS.MI</t>
+          <t>V60A.AS</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>L&amp;G Battery Value-Chain UCITS ETF</t>
+          <t>Xtrackers MSCI World Consumer Staples UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>BATT.AS</t>
+          <t>XDWS.MI</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>iShares MSCI Europe Quality Dividend Advanced UCITS ETF EUR (Dist)</t>
+          <t>iShares USD High Yield Corporate Bond ESG SRI UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>QDVX.SW</t>
+          <t>DHYE.AS</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>iShares MSCI Europe Health Care Sector UCITS ETF EUR (Acc)</t>
+          <t>iShares Russell 1000 Growth UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>ESIH.L</t>
+          <t>R1GR.AS</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>HSBC Multi-Factor Worldwide Equity UCITS ETF USD</t>
+          <t>State Street SPDR MSCI Europe Utilities UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>HWWA.L</t>
+          <t>STU.PA</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Japan UCITS ETF 4C - EUR Hedged</t>
+          <t>iShares MSCI World Information Technology Sector Advanced UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>XMK9.MI</t>
+          <t>WITS.AS</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>iShares EUR Floating Rate Bond Advanced UCITS ETF EUR (Dist)</t>
+          <t>HSBC MSCI Pacific ex Japan UCITS ETF USD</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>EFRN.SW</t>
+          <t>HMXJ.MI</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2027 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+          <t>UBS BBG Commodity CMCI SF UCITS ETF USD acc</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>IB27.PA</t>
+          <t>BCCMA.SW</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>PIMCO Euro Short Maturity UCITS ETF Acc</t>
+          <t>iShares FTSE 250 UCITS ETF</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>PJSR.MI</t>
+          <t>MIDD.SW</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Emerging Markets Swap UCITS ETF 1C</t>
+          <t>UBS Core MSCI EMU UCITS ETF hCHF acc</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>XMEM.MI</t>
+          <t>EMUCHF.SW</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>Vanguard ESG Global All Cap UCITS ETF (USD) Accumulating</t>
+          <t>iShares MSCI USA Screened UCITS ETF EUR Hedged (Acc)</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>V3AA.AS</t>
+          <t>SAUA.MI</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Japan UCITS ETF JPY Unhedged</t>
+          <t>Xtrackers MSCI World Financials UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>JPJY.PA</t>
+          <t>XDWF.MI</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Utilities UCITS ETF 1C</t>
+          <t>State Street SPDR Bloomberg 1-3 Month T-Bill UCITS ETF USD Unhedged (Acc)</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>XDWU.MI</t>
+          <t>TBIL.SW</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI USA Communication Services UCITS ETF 1D</t>
+          <t>JPMorgan USD Ultra-Short Income UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>XUCM.L</t>
+          <t>JPSA.MI</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
+          <t>Invesco MDAX UCITS ETF A</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>EXCD.AS</t>
+          <t>MDAX.MI</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI Europe Minimum Volatility UCITS ETF</t>
+          <t>HSBC FTSE EPRA NAREIT Developed UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>MVEU.MI</t>
+          <t>HPRA.L</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>iShares AI Infrastructure UCITS ETF USD (Acc)</t>
+          <t>JPMorgan EUR Corporate Bond Research Enhanced Index (ESG) UCITS ETF</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>AINF.AS</t>
+          <t>JREB.MI</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>Vanguard LifeStrategy 60% Equity UCITS ETF Accumulating</t>
+          <t>Xtrackers MSCI USA Health Care UCITS ETF 1D</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>V60A.AS</t>
+          <t>XUHC.SW</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Consumer Staples UCITS ETF 1C</t>
+          <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
         </is>
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>XDWS.MI</t>
+          <t>VAPU.SW</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>iShares USD High Yield Corporate Bond ESG SRI UCITS ETF USD (Acc)</t>
+          <t>iShares Core MSCI EMU UCITS ETF USD Hedged (Acc)</t>
         </is>
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>DHYE.AS</t>
+          <t>CEUU.AS</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>iShares Russell 1000 Growth UCITS ETF USD (Acc)</t>
+          <t>State Street SPDR MSCI World UCITS ETF EUR Hedged (Acc)</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>R1GR.AS</t>
+          <t>SWRE.MI</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Europe Utilities UCITS ETF EUR</t>
+          <t>Xtrackers Swiss Large Cap UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>STU.PA</t>
+          <t>XSMC.SW</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>iShares MSCI World Information Technology Sector Advanced UCITS ETF USD (Dist)</t>
+          <t>UBS Core MSCI World UCITS ETF hEUR acc</t>
         </is>
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>WITS.AS</t>
+          <t>WRDE.MI</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>HSBC MSCI Pacific ex Japan UCITS ETF USD</t>
+          <t>UBS Core MSCI USA UCITS ETF EUR Hedged acc</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>HMXJ.MI</t>
+          <t>USEUWH.MI</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>UBS BBG Commodity CMCI SF UCITS ETF USD acc</t>
+          <t>UBS MSCI World Selection UCITS ETF USD acc</t>
         </is>
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>BCCMA.SW</t>
+          <t>WDESG.MI</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>iShares FTSE 250 UCITS ETF</t>
+          <t>Xtrackers MSCI UK ESG UCITS ETF 1D</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>MIDD.SW</t>
+          <t>XASX.L</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>UBS Core MSCI EMU UCITS ETF hCHF acc</t>
+          <t>iShares Edge MSCI Europe Quality Factor UCITS ETF</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>EMUCHF.SW</t>
+          <t>IEQU.MI</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>iShares MSCI USA Screened UCITS ETF EUR Hedged (Acc)</t>
+          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>SAUA.MI</t>
+          <t>STN.PA</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Financials UCITS ETF 1C</t>
+          <t>Xtrackers Portfolio UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>XDWF.MI</t>
+          <t>XQUI.MI</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>State Street SPDR Bloomberg 1-3 Month T-Bill UCITS ETF USD Unhedged (Acc)</t>
+          <t>State Street SPDR MSCI Europe Financials UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>TBIL.SW</t>
+          <t>STZ.PA</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>JPMorgan USD Ultra-Short Income UCITS ETF USD (Acc)</t>
+          <t>iShares S&amp;P 500 Consumer Discretionary Sector UCITS ETF (Acc)</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>JPSA.MI</t>
+          <t>IUCD.SW</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>Invesco MDAX UCITS ETF A</t>
+          <t>Vanguard FTSE 250 UCITS ETF (GBP) Accumulating</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>MDAX.MI</t>
+          <t>VMIG.MI</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>HSBC FTSE EPRA NAREIT Developed UCITS ETF USD (Acc)</t>
+          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>HPRA.L</t>
+          <t>BTEC.SW</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>JPMorgan EUR Corporate Bond Research Enhanced Index (ESG) UCITS ETF</t>
+          <t>State Street SPDR S&amp;P 500 Quality Aristocrats UCITS ETF USD Unhedged (Acc)</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>JREB.MI</t>
+          <t>QUS5.SW</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI USA Health Care UCITS ETF 1D</t>
+          <t>iShares MSCI Poland UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B472" t="inlineStr">
-        <is>
-          <t>XUHC.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="473">
-      <c r="A473" t="inlineStr">
-        <is>
-          <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
-        </is>
-      </c>
-      <c r="B473" t="inlineStr">
-        <is>
-          <t>VAPU.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="474">
-      <c r="A474" t="inlineStr">
-        <is>
-          <t>iShares Core MSCI EMU UCITS ETF USD Hedged (Acc)</t>
-        </is>
-      </c>
-      <c r="B474" t="inlineStr">
-        <is>
-          <t>CEUU.AS</t>
-        </is>
-      </c>
-    </row>
-    <row r="475">
-      <c r="A475" t="inlineStr">
-        <is>
-          <t>State Street SPDR MSCI World UCITS ETF EUR Hedged (Acc)</t>
-        </is>
-      </c>
-      <c r="B475" t="inlineStr">
-        <is>
-          <t>SWRE.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="476">
-      <c r="A476" t="inlineStr">
-        <is>
-          <t>Xtrackers Swiss Large Cap UCITS ETF 1C</t>
-        </is>
-      </c>
-      <c r="B476" t="inlineStr">
-        <is>
-          <t>XSMC.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="477">
-      <c r="A477" t="inlineStr">
-        <is>
-          <t>UBS Core MSCI World UCITS ETF hEUR acc</t>
-        </is>
-      </c>
-      <c r="B477" t="inlineStr">
-        <is>
-          <t>WRDE.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="478">
-      <c r="A478" t="inlineStr">
-        <is>
-          <t>UBS Core MSCI USA UCITS ETF EUR Hedged acc</t>
-        </is>
-      </c>
-      <c r="B478" t="inlineStr">
-        <is>
-          <t>USEUWH.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="479">
-      <c r="A479" t="inlineStr">
-        <is>
-          <t>UBS MSCI World Selection UCITS ETF USD acc</t>
-        </is>
-      </c>
-      <c r="B479" t="inlineStr">
-        <is>
-          <t>WDESG.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="480">
-      <c r="A480" t="inlineStr">
-        <is>
-          <t>Xtrackers MSCI UK ESG UCITS ETF 1D</t>
-        </is>
-      </c>
-      <c r="B480" t="inlineStr">
-        <is>
-          <t>XASX.L</t>
-        </is>
-      </c>
-    </row>
-    <row r="481">
-      <c r="A481" t="inlineStr">
-        <is>
-          <t>iShares Edge MSCI Europe Quality Factor UCITS ETF</t>
-        </is>
-      </c>
-      <c r="B481" t="inlineStr">
-        <is>
-          <t>IEQU.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="482">
-      <c r="A482" t="inlineStr">
-        <is>
-          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
-        </is>
-      </c>
-      <c r="B482" t="inlineStr">
-        <is>
-          <t>STN.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="483">
-      <c r="A483" t="inlineStr">
-        <is>
-          <t>Xtrackers Portfolio UCITS ETF 1C</t>
-        </is>
-      </c>
-      <c r="B483" t="inlineStr">
-        <is>
-          <t>XQUI.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="484">
-      <c r="A484" t="inlineStr">
-        <is>
-          <t>State Street SPDR MSCI Europe Financials UCITS ETF EUR</t>
-        </is>
-      </c>
-      <c r="B484" t="inlineStr">
-        <is>
-          <t>STZ.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="485">
-      <c r="A485" t="inlineStr">
-        <is>
-          <t>iShares S&amp;P 500 Consumer Discretionary Sector UCITS ETF (Acc)</t>
-        </is>
-      </c>
-      <c r="B485" t="inlineStr">
-        <is>
-          <t>IUCD.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="486">
-      <c r="A486" t="inlineStr">
-        <is>
-          <t>Vanguard FTSE 250 UCITS ETF (GBP) Accumulating</t>
-        </is>
-      </c>
-      <c r="B486" t="inlineStr">
-        <is>
-          <t>VMIG.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="487">
-      <c r="A487" t="inlineStr">
-        <is>
-          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
-        </is>
-      </c>
-      <c r="B487" t="inlineStr">
-        <is>
-          <t>BTEC.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="488">
-      <c r="A488" t="inlineStr">
-        <is>
-          <t>State Street SPDR S&amp;P 500 Quality Aristocrats UCITS ETF USD Unhedged (Acc)</t>
-        </is>
-      </c>
-      <c r="B488" t="inlineStr">
-        <is>
-          <t>QUS5.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="489">
-      <c r="A489" t="inlineStr">
-        <is>
-          <t>iShares MSCI Poland UCITS ETF USD (Acc)</t>
-        </is>
-      </c>
-      <c r="B489" t="inlineStr">
         <is>
           <t>SPOL.SW</t>
         </is>

</xml_diff>

<commit_message>
feat(etf): add 100 more justETF sample ETFs (extra_count 450 -> 550)
Grow the active universe by ~100 more list-order justETF extras. Seed
regenerates from 471 to 571 tickers (15 core + justETF extras + AUM top-100,
deduped). Historical backfill for the new tickers runs via the cold-start
workflow at the same 2016-01-01 -> today range.
</commit_message>
<xml_diff>
--- a/data/ticker/etf/ticker_active.xlsx
+++ b/data/ticker/etf/ticker_active.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B472"/>
+  <dimension ref="A1:B572"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5231,850 +5231,2050 @@
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>HSBC MSCI Emerging Markets UCITS ETF USD (Acc)</t>
+          <t>Bitwise Physical Litecoin ETP</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>HEMA.PA</t>
+          <t>ELTC.AS</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>iShares EUR Cash UCITS ETF EUR (Acc)</t>
+          <t>Bitwise Physical Solana ETP</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>YCSH.AS</t>
+          <t>ESOLGBP.SW</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Nordic UCITS ETF 1D</t>
+          <t>Bitwise Physical XRP ETP</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>XDN0.SW</t>
+          <t>GXRP.PA</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>JPMorgan US Research Enhanced Index Equity Active UCITS ETF EUR Hedged (acc)</t>
+          <t>Bitwise Solana Staking ETP</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>JUHE.MI</t>
+          <t>BSOL.PA</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2028 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+          <t>CF Crypto Momentum ETP</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>B28A.PA</t>
+          <t>CFMOM.SW</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>Invesco S&amp;P 500 Equal Weight UCITS ETF Acc</t>
+          <t>CT QR Series European Equity Active UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>SPEQ.MI</t>
+          <t>QREU.MI</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>Xtrackers S&amp;P 500 Equal Weight Scored &amp; Screened UCITS ETF 2C - EUR Hedged</t>
+          <t>CT QR Series European Equity Active UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>XEWE.MI</t>
+          <t>QRED.L</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>UBS Core MSCI World UCITS ETF hCHF acc</t>
+          <t>CT QR Series Global Equity Active UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>WORLD.SW</t>
+          <t>QRGE.SW</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>Schroder Global Equity Active UCITS ETF</t>
+          <t>CT QR Series Global Equity Active UCITS ETF USD Dist</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>SAGE.MI</t>
+          <t>QRGD.L</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
+          <t>CT QR Series US Equity Active UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>SXLE.AS</t>
+          <t>QRUS.MI</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>iShares STOXX Europe 600 Utilities UCITS ETF (DE)</t>
+          <t>CT QR Series US Equity Active UCITS ETF USD Dist</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>SX6PEX.SW</t>
+          <t>QRUD.L</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>iShares European Property Yield UCITS ETF</t>
+          <t>Cardano Impact for UNHCR ETP</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>IPRP.AS</t>
+          <t>CASL.SW</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>Invesco CoinShares Global Blockchain UCITS ETF Acc</t>
+          <t>CoinShares Physical Bitcoin</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>BCHN.MI</t>
+          <t>BITC.AS</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>Global X Copper Miners UCITS ETF USD Accumulating</t>
+          <t>CoinShares Physical Litecoin</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>COPX.MI</t>
+          <t>LITE.SW</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>UBS S&amp;P 500 Scored &amp; Screened UCITS ETF hEUR acc</t>
+          <t>CoinShares Physical Staked Cardano</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>5ESGE.MI</t>
+          <t>CSDA.PA</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>iShares MSCI Korea UCITS ETF (Dist)</t>
+          <t>CoinShares Physical Staked Ethereum</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>IKRA.AS</t>
+          <t>CETH.AS</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Minimum Volatility UCITS ETF 1C</t>
+          <t>CoinShares Physical Staked Polkadot</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>XDEB.MI</t>
+          <t>CDOT.SW</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>JPMorgan Global Research Enhanced Index Equity (ESG) UCITS ETF EUR Hedged (acc)</t>
+          <t>CoinShares Physical Staked Solana</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>JRGE.MI</t>
+          <t>SLNC.PA</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>UBS MSCI AC Asia ex Japan SF UCITS ETF USD acc</t>
+          <t>CoinShares Physical Top10 Crypto Market ETP</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>AJEUAS.MI</t>
+          <t>CTEN.PA</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>Invesco S&amp;P 500 Equal Weight Swap UCITS ETF Acc</t>
+          <t>CoinShares Physical XRP</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>RSPS.MI</t>
+          <t>XRPL.PA</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>L&amp;G Battery Value-Chain UCITS ETF</t>
+          <t>DDA Bitcoin Macro ETP</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>BATT.AS</t>
+          <t>BMAC.PA</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>iShares MSCI Europe Quality Dividend Advanced UCITS ETF EUR (Dist)</t>
+          <t>DDA Physical Bitcoin ETP</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>QDVX.SW</t>
+          <t>XBTI.AS</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>iShares MSCI Europe Health Care Sector UCITS ETF EUR (Acc)</t>
+          <t>Defiance AI &amp; Power Infrastructure UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>ESIH.L</t>
+          <t>AIPO.MI</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>HSBC Multi-Factor Worldwide Equity UCITS ETF USD</t>
+          <t>Deka DAX ex Financials 30 UCITS ETF</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>HWWA.L</t>
+          <t>0W81.L</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Japan UCITS ETF 4C - EUR Hedged</t>
+          <t>Deka MSCI Europe MC UCITS ETF</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>XMK9.MI</t>
+          <t>0MQ3.L</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>iShares EUR Floating Rate Bond Advanced UCITS ETF EUR (Dist)</t>
+          <t>Deka MSCI USA MC UCITS ETF</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>EFRN.SW</t>
+          <t>0MPZ.L</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2027 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+          <t>Dimensional Global Core Equity UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>IB27.PA</t>
+          <t>DDGC.L</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>PIMCO Euro Short Maturity UCITS ETF Acc</t>
+          <t>Dimensional Global Targeted Value UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>PJSR.MI</t>
+          <t>DDGT.L</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Emerging Markets Swap UCITS ETF 1C</t>
+          <t>Dimensional Global ex US Core Equity Market UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>XMEM.MI</t>
+          <t>DPXM.L</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>Vanguard ESG Global All Cap UCITS ETF (USD) Accumulating</t>
+          <t>Dimensional US Core Equity Market UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>V3AA.AS</t>
+          <t>DPUM.L</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Japan UCITS ETF JPY Unhedged</t>
+          <t>EUWAX Gold II</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>JPJY.PA</t>
+          <t>BEWGF</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Utilities UCITS ETF 1C</t>
+          <t>Eurizon YIS MSCI Japan Universal UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>XDWU.MI</t>
+          <t>YIJU.MI</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI USA Communication Services UCITS ETF 1D</t>
+          <t>Eurizon YIS MSCI Japan Universal UCITS ETF EUR Hedged (Acc)</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>XUCM.L</t>
+          <t>YIJUH.MI</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
+          <t>Eurizon YIS MSCI North America Universal UCITS ETF EUR Hedged (Acc)</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>EXCD.AS</t>
+          <t>YIAUH.MI</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI Europe Minimum Volatility UCITS ETF</t>
+          <t>Eurizon YIS MSCI North America Universal UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>MVEU.MI</t>
+          <t>YINA2.MI</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>iShares AI Infrastructure UCITS ETF USD (Acc)</t>
+          <t>Eurizon YIS MSCI USA Selection UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>AINF.AS</t>
+          <t>YIUS2.MI</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>Vanguard LifeStrategy 60% Equity UCITS ETF Accumulating</t>
+          <t>Eurizon YIS MSCI USA Universal UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>V60A.AS</t>
+          <t>YIUU2.MI</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Consumer Staples UCITS ETF 1C</t>
+          <t>Fair Oaks AAA CLO Fund UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>XDWS.MI</t>
+          <t>EAAA.MI</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>iShares USD High Yield Corporate Bond ESG SRI UCITS ETF USD (Acc)</t>
+          <t>Fair Oaks AAA CLO Fund UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>DHYE.AS</t>
+          <t>FAAA.L</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>iShares Russell 1000 Growth UCITS ETF USD (Acc)</t>
+          <t>Fidelity ESG USD EM Bond UCITS ETF ACC-GBP (hedged)</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>R1GR.AS</t>
+          <t>FEMP.L</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Europe Utilities UCITS ETF EUR</t>
+          <t>Fidelity ESG USD EM Bond UCITS ETF INC-USD</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>STU.PA</t>
+          <t>FSEM.MI</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>iShares MSCI World Information Technology Sector Advanced UCITS ETF USD (Dist)</t>
+          <t>Fidelity EUR Corporate Bond Research Enhanced PAB UCITS ETF EUR (Dist)</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>WITS.AS</t>
+          <t>FEIG.MI</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>HSBC MSCI Pacific ex Japan UCITS ETF USD</t>
+          <t>Fidelity EUR Corporate Bond Research Enhanced PAB UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>HMXJ.MI</t>
+          <t>FEIA.MI</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>UBS BBG Commodity CMCI SF UCITS ETF USD acc</t>
+          <t>Fidelity EUR Corporate Bond Research Enhanced PAB UCITS ETF GBP Hedged (Acc)</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>BCCMA.SW</t>
+          <t>FEIP.L</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>iShares FTSE 250 UCITS ETF</t>
+          <t>Fidelity EUR Corporate Bond Research Enhanced UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>MIDD.SW</t>
+          <t>FBIE.MI</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>UBS Core MSCI EMU UCITS ETF hCHF acc</t>
+          <t>Fidelity EUR HY Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>EMUCHF.SW</t>
+          <t>FYEP.L</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>iShares MSCI USA Screened UCITS ETF EUR Hedged (Acc)</t>
+          <t>Fidelity EUR HY Corp Bond Research Enhanced PAB UCITS ETF INC-Euro</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>SAUA.MI</t>
+          <t>FYEI.MI</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Financials UCITS ETF 1C</t>
+          <t>Fidelity Emerging Markets Equity Research Enhanced UCITS ETF ACC-USD</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>XDWF.MI</t>
+          <t>FEMR.MI</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>State Street SPDR Bloomberg 1-3 Month T-Bill UCITS ETF USD Unhedged (Acc)</t>
+          <t>Fidelity Emerging Markets Quality Income UCITS ETF ACC-USD</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>TBIL.SW</t>
+          <t>FEMI.MI</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>JPMorgan USD Ultra-Short Income UCITS ETF USD (Acc)</t>
+          <t>Fidelity Emerging Markets Quality Income UCITS ETF INC-USD</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>JPSA.MI</t>
+          <t>FEME.MI</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>Invesco MDAX UCITS ETF A</t>
+          <t>Fidelity Europe Equity Research Enhanced UCITS ETF ACC-Euro</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>MDAX.MI</t>
+          <t>FEUR.MI</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>HSBC FTSE EPRA NAREIT Developed UCITS ETF USD (Acc)</t>
+          <t>Fidelity Europe Quality Income UCITS ETF ACC-Euro</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>HPRA.L</t>
+          <t>FEQD.MI</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>JPMorgan EUR Corporate Bond Research Enhanced Index (ESG) UCITS ETF</t>
+          <t>Fidelity Europe Quality Income UCITS ETF ACC-GBP (hedged)</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>JREB.MI</t>
+          <t>FEQP.L</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI USA Health Care UCITS ETF 1D</t>
+          <t>Fidelity Europe Quality Income UCITS ETF INC-Euro</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>XUHC.SW</t>
+          <t>FEUI.MI</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
+          <t>Fidelity Global Corp Bond Research Enhanced PAB UCITS ETF ACC-Euro (hedged)</t>
         </is>
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>VAPU.SW</t>
+          <t>FSME.MI</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>iShares Core MSCI EMU UCITS ETF USD Hedged (Acc)</t>
+          <t>Fidelity Global Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
         </is>
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>CEUU.AS</t>
+          <t>FSMP.L</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI World UCITS ETF EUR Hedged (Acc)</t>
+          <t>Fidelity Global Corp Bond Research Enhanced PAB UCITS ETF INC-USD</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>SWRE.MI</t>
+          <t>FSMF.MI</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>Xtrackers Swiss Large Cap UCITS ETF 1C</t>
+          <t>Fidelity Global Corp Bond Research Enhanced PAB UCITS ETF INC-USD (hedged)</t>
         </is>
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>XSMC.SW</t>
+          <t>FSMU.SW</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>UBS Core MSCI World UCITS ETF hEUR acc</t>
+          <t>Fidelity Global Equity Research Enhanced PAB UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>WRDE.MI</t>
+          <t>FRPG.L</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>UBS Core MSCI USA UCITS ETF EUR Hedged acc</t>
+          <t>Fidelity Global Equity Research Enhanced UCITS ETF ACC-USD</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>USEUWH.MI</t>
+          <t>FGLR.MI</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>UBS MSCI World Selection UCITS ETF USD acc</t>
+          <t>Fidelity Global HY Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
         </is>
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>WDESG.MI</t>
+          <t>FHYG.L</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI UK ESG UCITS ETF 1D</t>
+          <t>Fidelity Global HY Corp Bond Research Enhanced PAB UCITS ETF INC-Euro (hedged)</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>XASX.L</t>
+          <t>FFGE.MI</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI Europe Quality Factor UCITS ETF</t>
+          <t>Fidelity Global HY Corp Bond Research Enhanced PAB UCITS ETF INC-USD</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>IEQU.MI</t>
+          <t>FGHY.MI</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
+          <t>Fidelity Global HY Corp Bond Research Enhanced PAB UCITS ETF INC-USD (hedged)</t>
         </is>
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>STN.PA</t>
+          <t>FGHU.SW</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>Xtrackers Portfolio UCITS ETF 1C</t>
+          <t>Fidelity Japan Equity Research Enhanced UCITS ETF ACC-JPY</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>XQUI.MI</t>
+          <t>FJPR.MI</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Europe Financials UCITS ETF EUR</t>
+          <t>Fidelity Japan Equity Research Enhanced UCITS ETF INC-JPY</t>
         </is>
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>STZ.PA</t>
+          <t>FJPI.SW</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>iShares S&amp;P 500 Consumer Discretionary Sector UCITS ETF (Acc)</t>
+          <t>Fidelity Pacific ex-Japan Equity Research Enhanced UCITS ETF ACC-USD</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>IUCD.SW</t>
+          <t>FPXR.MI</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>Vanguard FTSE 250 UCITS ETF (GBP) Accumulating</t>
+          <t>Fidelity Physical Bitcoin ETP</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>VMIG.MI</t>
+          <t>FBTC.MI</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
+          <t>Fidelity US Equity Research Enhanced UCITS ETF ACC-USD</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>BTEC.SW</t>
+          <t>FUSR.MI</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>State Street SPDR S&amp;P 500 Quality Aristocrats UCITS ETF USD Unhedged (Acc)</t>
+          <t>Fidelity US Equity Research Enhanced UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>QUS5.SW</t>
+          <t>FUSE.MI</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
+          <t>Fidelity US Fundamental Large Cap Core UCITS ETF ACC-USD</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>FFLC.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>Fidelity US Fundamental Small-Mid Cap UCITS ETF ACC-USD</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>FFSM.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>Fidelity US Quality Income UCITS ETF ACC-Euro (hedged)</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>FUSU.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>Fidelity US Quality Income UCITS ETF ACC-GBP (hedged)</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>FUSP.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>Fidelity US Quality Income UCITS ETF ACC-USD</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>FUSA.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>Fidelity US Quality Income UCITS ETF INC-USD</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>FUSD.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>Fidelity USD Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>FUIP.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>Fidelity USD Corp Bond Research Enhanced PAB UCITS ETF INC-Euro (hedged)</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>FUIE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>Fidelity USD Corp Bond Research Enhanced PAB UCITS ETF INC-USD</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>FUIG.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>Fidelity USD Corporate Bond Research Enhanced UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>FBIU.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>Fidelity USD Corporate Bond Research Enhanced UCITS ETF EUR Hedged Acc</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>FBIH.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Fidelity USD HY Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>FYUP.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>Fidelity USD HY Corp Bond Research Enhanced PAB UCITS ETF INC-USD</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>FYUI.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>First Trust Bloomberg Artificial Intelligence UCITS ETF Class A Accumulation</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>FTAI.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>First Trust Bloomberg Scarce Resources UCITS ETF Class A Accumulation</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>SCAR.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>First Trust Capital Strength UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>FTCS.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>First Trust FactorFX UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>FTFX.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>First Trust FactorFX UCITS ETF EUR Hedged Acc</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>FXEU.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>First Trust FactorFX UCITS ETF GBP Hedged Acc</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>FXGB.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>First Trust Global Capital Strength ESG Leaders UCITS ETF Class A Accumulation</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>FCSG.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>First Trust Global Equity Income UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>FGBL.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>First Trust Global Equity Income UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>GINC.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>First Trust Indxx Future Economy Metals UCITS ETF Class A Accumulation</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>MINR.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>First Trust Indxx Innovative Transaction &amp; Process UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>BLOK.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>First Trust NYSE Arca Biotechnology UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>FBT.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>First Trust Rising Dividend Achievers UCITS ETF Class A Accumulation</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>RDVY.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>First Trust SMID Rising Dividend Achievers UCITS ETF Class A Accumulation</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>SDVY.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>First Trust SMID Rising Dividend Achievers UCITS ETF Class B Distribution</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>SDVI.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>First Trust US Equity Income UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>UNCA.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>First Trust US Equity Income UCITS ETF Dist</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>UINC.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>HSBC MSCI Emerging Markets UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>HEMA.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>iShares EUR Cash UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>YCSH.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI Nordic UCITS ETF 1D</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>XDN0.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>JPMorgan US Research Enhanced Index Equity Active UCITS ETF EUR Hedged (acc)</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>JUHE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>iShares iBonds Dec 2028 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>B28A.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Invesco S&amp;P 500 Equal Weight UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>SPEQ.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Xtrackers S&amp;P 500 Equal Weight Scored &amp; Screened UCITS ETF 2C - EUR Hedged</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>XEWE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>UBS Core MSCI World UCITS ETF hCHF acc</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>WORLD.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>Schroder Global Equity Active UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>SAGE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>SXLE.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>iShares STOXX Europe 600 Utilities UCITS ETF (DE)</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>SX6PEX.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>iShares European Property Yield UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>IPRP.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>Invesco CoinShares Global Blockchain UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>BCHN.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Global X Copper Miners UCITS ETF USD Accumulating</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>COPX.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>UBS S&amp;P 500 Scored &amp; Screened UCITS ETF hEUR acc</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>5ESGE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>iShares MSCI Korea UCITS ETF (Dist)</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>IKRA.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Minimum Volatility UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>XDEB.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>JPMorgan Global Research Enhanced Index Equity (ESG) UCITS ETF EUR Hedged (acc)</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>JRGE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>UBS MSCI AC Asia ex Japan SF UCITS ETF USD acc</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>AJEUAS.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>Invesco S&amp;P 500 Equal Weight Swap UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>RSPS.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>L&amp;G Battery Value-Chain UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>BATT.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>iShares MSCI Europe Quality Dividend Advanced UCITS ETF EUR (Dist)</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>QDVX.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>iShares MSCI Europe Health Care Sector UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>ESIH.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>HSBC Multi-Factor Worldwide Equity UCITS ETF USD</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>HWWA.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI Japan UCITS ETF 4C - EUR Hedged</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>XMK9.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>iShares EUR Floating Rate Bond Advanced UCITS ETF EUR (Dist)</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>EFRN.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>iShares iBonds Dec 2027 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>IB27.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>PIMCO Euro Short Maturity UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>PJSR.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI Emerging Markets Swap UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>XMEM.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>Vanguard ESG Global All Cap UCITS ETF (USD) Accumulating</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>V3AA.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI Japan UCITS ETF JPY Unhedged</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>JPJY.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Utilities UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>XDWU.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI USA Communication Services UCITS ETF 1D</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>XUCM.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>EXCD.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>iShares Edge MSCI Europe Minimum Volatility UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>MVEU.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>iShares AI Infrastructure UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>AINF.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>Vanguard LifeStrategy 60% Equity UCITS ETF Accumulating</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>V60A.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Consumer Staples UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>XDWS.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>iShares USD High Yield Corporate Bond ESG SRI UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>DHYE.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>iShares Russell 1000 Growth UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>R1GR.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI Europe Utilities UCITS ETF EUR</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>STU.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>iShares MSCI World Information Technology Sector Advanced UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>WITS.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>HSBC MSCI Pacific ex Japan UCITS ETF USD</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>HMXJ.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>UBS BBG Commodity CMCI SF UCITS ETF USD acc</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>BCCMA.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>iShares FTSE 250 UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>MIDD.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>UBS Core MSCI EMU UCITS ETF hCHF acc</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>EMUCHF.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>iShares MSCI USA Screened UCITS ETF EUR Hedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>SAUA.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Financials UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>XDWF.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>State Street SPDR Bloomberg 1-3 Month T-Bill UCITS ETF USD Unhedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>TBIL.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>JPMorgan USD Ultra-Short Income UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>JPSA.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>Invesco MDAX UCITS ETF A</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>MDAX.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>HSBC FTSE EPRA NAREIT Developed UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>HPRA.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>JPMorgan EUR Corporate Bond Research Enhanced Index (ESG) UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>JREB.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI USA Health Care UCITS ETF 1D</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>XUHC.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>VAPU.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>iShares Core MSCI EMU UCITS ETF USD Hedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>CEUU.AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI World UCITS ETF EUR Hedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>SWRE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>Xtrackers Swiss Large Cap UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>XSMC.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>UBS Core MSCI World UCITS ETF hEUR acc</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>WRDE.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>UBS Core MSCI USA UCITS ETF EUR Hedged acc</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>USEUWH.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>UBS MSCI World Selection UCITS ETF USD acc</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>WDESG.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI UK ESG UCITS ETF 1D</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>XASX.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>iShares Edge MSCI Europe Quality Factor UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>IEQU.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>STN.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>Xtrackers Portfolio UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>XQUI.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI Europe Financials UCITS ETF EUR</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>STZ.PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>iShares S&amp;P 500 Consumer Discretionary Sector UCITS ETF (Acc)</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>IUCD.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>Vanguard FTSE 250 UCITS ETF (GBP) Accumulating</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>VMIG.MI</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>BTEC.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>State Street SPDR S&amp;P 500 Quality Aristocrats UCITS ETF USD Unhedged (Acc)</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>QUS5.SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
           <t>iShares MSCI Poland UCITS ETF USD (Acc)</t>
         </is>
       </c>
-      <c r="B472" t="inlineStr">
+      <c r="B572" t="inlineStr">
         <is>
           <t>SPOL.SW</t>
         </is>

</xml_diff>

<commit_message>
fix(etf): prune 12 dead tickers from the 571-ticker run (universe -> 559)
The extra_count=550 cold-start downloaded 559/571 (98%), 746,493 rows, range
2016-01-04 -> 2026-07-13. 12 symbols returned no Yahoo data (thin .L/.SW/.MI
listings and OTC symbols); fold them into KNOWN_DEAD.

Regenerated seed is 559 tickers and matches the committed historical parquet
symbols exactly, so no re-backfill is needed.
</commit_message>
<xml_diff>
--- a/data/ticker/etf/ticker_active.xlsx
+++ b/data/ticker/etf/ticker_active.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B572"/>
+  <dimension ref="A1:B560"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5243,2038 +5243,1894 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>Bitwise Physical Solana ETP</t>
+          <t>Bitwise Physical XRP ETP</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>ESOLGBP.SW</t>
+          <t>GXRP.PA</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>Bitwise Physical XRP ETP</t>
+          <t>Bitwise Solana Staking ETP</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>GXRP.PA</t>
+          <t>BSOL.PA</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>Bitwise Solana Staking ETP</t>
+          <t>CT QR Series European Equity Active UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>BSOL.PA</t>
+          <t>QREU.MI</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>CF Crypto Momentum ETP</t>
+          <t>CT QR Series European Equity Active UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>CFMOM.SW</t>
+          <t>QRED.L</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>CT QR Series European Equity Active UCITS ETF EUR Acc</t>
+          <t>CT QR Series Global Equity Active UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>QREU.MI</t>
+          <t>QRGE.SW</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>CT QR Series European Equity Active UCITS ETF EUR Dist</t>
+          <t>CT QR Series Global Equity Active UCITS ETF USD Dist</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>QRED.L</t>
+          <t>QRGD.L</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>CT QR Series Global Equity Active UCITS ETF USD Acc</t>
+          <t>CT QR Series US Equity Active UCITS ETF USD Acc</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>QRGE.SW</t>
+          <t>QRUS.MI</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>CT QR Series Global Equity Active UCITS ETF USD Dist</t>
+          <t>CT QR Series US Equity Active UCITS ETF USD Dist</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>QRGD.L</t>
+          <t>QRUD.L</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>CT QR Series US Equity Active UCITS ETF USD Acc</t>
+          <t>CoinShares Physical Bitcoin</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>QRUS.MI</t>
+          <t>BITC.AS</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>CT QR Series US Equity Active UCITS ETF USD Dist</t>
+          <t>CoinShares Physical Litecoin</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>QRUD.L</t>
+          <t>LITE.SW</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>Cardano Impact for UNHCR ETP</t>
+          <t>CoinShares Physical Staked Cardano</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>CASL.SW</t>
+          <t>CSDA.PA</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>CoinShares Physical Bitcoin</t>
+          <t>CoinShares Physical Staked Ethereum</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>BITC.AS</t>
+          <t>CETH.AS</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>CoinShares Physical Litecoin</t>
+          <t>CoinShares Physical Staked Polkadot</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>LITE.SW</t>
+          <t>CDOT.SW</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>CoinShares Physical Staked Cardano</t>
+          <t>CoinShares Physical Staked Solana</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>CSDA.PA</t>
+          <t>SLNC.PA</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>CoinShares Physical Staked Ethereum</t>
+          <t>CoinShares Physical Top10 Crypto Market ETP</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>CETH.AS</t>
+          <t>CTEN.PA</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>CoinShares Physical Staked Polkadot</t>
+          <t>CoinShares Physical XRP</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>CDOT.SW</t>
+          <t>XRPL.PA</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>CoinShares Physical Staked Solana</t>
+          <t>Defiance AI &amp; Power Infrastructure UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>SLNC.PA</t>
+          <t>AIPO.MI</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>CoinShares Physical Top10 Crypto Market ETP</t>
+          <t>Dimensional Global Core Equity UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>CTEN.PA</t>
+          <t>DDGC.L</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>CoinShares Physical XRP</t>
+          <t>Dimensional Global Targeted Value UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>XRPL.PA</t>
+          <t>DDGT.L</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>DDA Bitcoin Macro ETP</t>
+          <t>Dimensional Global ex US Core Equity Market UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>BMAC.PA</t>
+          <t>DPXM.L</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>DDA Physical Bitcoin ETP</t>
+          <t>Dimensional US Core Equity Market UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>XBTI.AS</t>
+          <t>DPUM.L</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>Defiance AI &amp; Power Infrastructure UCITS ETF Acc</t>
+          <t>Eurizon YIS MSCI Japan Universal UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>AIPO.MI</t>
+          <t>YIJU.MI</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>Deka DAX ex Financials 30 UCITS ETF</t>
+          <t>Eurizon YIS MSCI Japan Universal UCITS ETF EUR Hedged (Acc)</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>0W81.L</t>
+          <t>YIJUH.MI</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>Deka MSCI Europe MC UCITS ETF</t>
+          <t>Eurizon YIS MSCI North America Universal UCITS ETF EUR Hedged (Acc)</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>0MQ3.L</t>
+          <t>YIAUH.MI</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>Deka MSCI USA MC UCITS ETF</t>
+          <t>Eurizon YIS MSCI North America Universal UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>0MPZ.L</t>
+          <t>YINA2.MI</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>Dimensional Global Core Equity UCITS ETF USD (Acc)</t>
+          <t>Eurizon YIS MSCI USA Selection UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>DDGC.L</t>
+          <t>YIUS2.MI</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>Dimensional Global Targeted Value UCITS ETF USD (Acc)</t>
+          <t>Eurizon YIS MSCI USA Universal UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>DDGT.L</t>
+          <t>YIUU2.MI</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>Dimensional Global ex US Core Equity Market UCITS ETF USD (Acc)</t>
+          <t>Fair Oaks AAA CLO Fund UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>DPXM.L</t>
+          <t>EAAA.MI</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>Dimensional US Core Equity Market UCITS ETF USD (Acc)</t>
+          <t>Fair Oaks AAA CLO Fund UCITS ETF EUR Dist</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>DPUM.L</t>
+          <t>FAAA.L</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>EUWAX Gold II</t>
+          <t>Fidelity ESG USD EM Bond UCITS ETF ACC-GBP (hedged)</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>BEWGF</t>
+          <t>FEMP.L</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>Eurizon YIS MSCI Japan Universal UCITS ETF EUR (Acc)</t>
+          <t>Fidelity ESG USD EM Bond UCITS ETF INC-USD</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>YIJU.MI</t>
+          <t>FSEM.MI</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>Eurizon YIS MSCI Japan Universal UCITS ETF EUR Hedged (Acc)</t>
+          <t>Fidelity EUR Corporate Bond Research Enhanced PAB UCITS ETF EUR Acc</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>YIJUH.MI</t>
+          <t>FEIA.MI</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>Eurizon YIS MSCI North America Universal UCITS ETF EUR Hedged (Acc)</t>
+          <t>Fidelity EUR Corporate Bond Research Enhanced PAB UCITS ETF GBP Hedged (Acc)</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>YIAUH.MI</t>
+          <t>FEIP.L</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>Eurizon YIS MSCI North America Universal UCITS ETF USD (Acc)</t>
+          <t>Fidelity EUR Corporate Bond Research Enhanced UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>YINA2.MI</t>
+          <t>FBIE.MI</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>Eurizon YIS MSCI USA Selection UCITS ETF USD (Acc)</t>
+          <t>Fidelity EUR HY Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>YIUS2.MI</t>
+          <t>FYEP.L</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>Eurizon YIS MSCI USA Universal UCITS ETF USD (Acc)</t>
+          <t>Fidelity EUR HY Corp Bond Research Enhanced PAB UCITS ETF INC-Euro</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>YIUU2.MI</t>
+          <t>FYEI.MI</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>Fair Oaks AAA CLO Fund UCITS ETF EUR Acc</t>
+          <t>Fidelity Emerging Markets Equity Research Enhanced UCITS ETF ACC-USD</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>EAAA.MI</t>
+          <t>FEMR.MI</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>Fair Oaks AAA CLO Fund UCITS ETF EUR Dist</t>
+          <t>Fidelity Emerging Markets Quality Income UCITS ETF ACC-USD</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>FAAA.L</t>
+          <t>FEMI.MI</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>Fidelity ESG USD EM Bond UCITS ETF ACC-GBP (hedged)</t>
+          <t>Fidelity Emerging Markets Quality Income UCITS ETF INC-USD</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>FEMP.L</t>
+          <t>FEME.MI</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>Fidelity ESG USD EM Bond UCITS ETF INC-USD</t>
+          <t>Fidelity Europe Equity Research Enhanced UCITS ETF ACC-Euro</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>FSEM.MI</t>
+          <t>FEUR.MI</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>Fidelity EUR Corporate Bond Research Enhanced PAB UCITS ETF EUR (Dist)</t>
+          <t>Fidelity Europe Quality Income UCITS ETF ACC-Euro</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>FEIG.MI</t>
+          <t>FEQD.MI</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>Fidelity EUR Corporate Bond Research Enhanced PAB UCITS ETF EUR Acc</t>
+          <t>Fidelity Europe Quality Income UCITS ETF ACC-GBP (hedged)</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>FEIA.MI</t>
+          <t>FEQP.L</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>Fidelity EUR Corporate Bond Research Enhanced PAB UCITS ETF GBP Hedged (Acc)</t>
+          <t>Fidelity Europe Quality Income UCITS ETF INC-Euro</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>FEIP.L</t>
+          <t>FEUI.MI</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>Fidelity EUR Corporate Bond Research Enhanced UCITS ETF Acc</t>
+          <t>Fidelity Global Corp Bond Research Enhanced PAB UCITS ETF ACC-Euro (hedged)</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>FBIE.MI</t>
+          <t>FSME.MI</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>Fidelity EUR HY Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
+          <t>Fidelity Global Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>FYEP.L</t>
+          <t>FSMP.L</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>Fidelity EUR HY Corp Bond Research Enhanced PAB UCITS ETF INC-Euro</t>
+          <t>Fidelity Global Corp Bond Research Enhanced PAB UCITS ETF INC-USD</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>FYEI.MI</t>
+          <t>FSMF.MI</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>Fidelity Emerging Markets Equity Research Enhanced UCITS ETF ACC-USD</t>
+          <t>Fidelity Global Corp Bond Research Enhanced PAB UCITS ETF INC-USD (hedged)</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>FEMR.MI</t>
+          <t>FSMU.SW</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>Fidelity Emerging Markets Quality Income UCITS ETF ACC-USD</t>
+          <t>Fidelity Global Equity Research Enhanced PAB UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>FEMI.MI</t>
+          <t>FRPG.L</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>Fidelity Emerging Markets Quality Income UCITS ETF INC-USD</t>
+          <t>Fidelity Global Equity Research Enhanced UCITS ETF ACC-USD</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>FEME.MI</t>
+          <t>FGLR.MI</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>Fidelity Europe Equity Research Enhanced UCITS ETF ACC-Euro</t>
+          <t>Fidelity Global HY Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>FEUR.MI</t>
+          <t>FHYG.L</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>Fidelity Europe Quality Income UCITS ETF ACC-Euro</t>
+          <t>Fidelity Global HY Corp Bond Research Enhanced PAB UCITS ETF INC-Euro (hedged)</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>FEQD.MI</t>
+          <t>FFGE.MI</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>Fidelity Europe Quality Income UCITS ETF ACC-GBP (hedged)</t>
+          <t>Fidelity Global HY Corp Bond Research Enhanced PAB UCITS ETF INC-USD</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>FEQP.L</t>
+          <t>FGHY.MI</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>Fidelity Europe Quality Income UCITS ETF INC-Euro</t>
+          <t>Fidelity Global HY Corp Bond Research Enhanced PAB UCITS ETF INC-USD (hedged)</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>FEUI.MI</t>
+          <t>FGHU.SW</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>Fidelity Global Corp Bond Research Enhanced PAB UCITS ETF ACC-Euro (hedged)</t>
+          <t>Fidelity Japan Equity Research Enhanced UCITS ETF ACC-JPY</t>
         </is>
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>FSME.MI</t>
+          <t>FJPR.MI</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>Fidelity Global Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
+          <t>Fidelity Japan Equity Research Enhanced UCITS ETF INC-JPY</t>
         </is>
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>FSMP.L</t>
+          <t>FJPI.SW</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>Fidelity Global Corp Bond Research Enhanced PAB UCITS ETF INC-USD</t>
+          <t>Fidelity Pacific ex-Japan Equity Research Enhanced UCITS ETF ACC-USD</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>FSMF.MI</t>
+          <t>FPXR.MI</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>Fidelity Global Corp Bond Research Enhanced PAB UCITS ETF INC-USD (hedged)</t>
+          <t>Fidelity Physical Bitcoin ETP</t>
         </is>
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>FSMU.SW</t>
+          <t>FBTC.MI</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>Fidelity Global Equity Research Enhanced PAB UCITS ETF USD (Acc)</t>
+          <t>Fidelity US Equity Research Enhanced UCITS ETF ACC-USD</t>
         </is>
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>FRPG.L</t>
+          <t>FUSR.MI</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>Fidelity Global Equity Research Enhanced UCITS ETF ACC-USD</t>
+          <t>Fidelity US Equity Research Enhanced UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>FGLR.MI</t>
+          <t>FUSE.MI</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>Fidelity Global HY Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
+          <t>Fidelity US Fundamental Large Cap Core UCITS ETF ACC-USD</t>
         </is>
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>FHYG.L</t>
+          <t>FFLC.MI</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>Fidelity Global HY Corp Bond Research Enhanced PAB UCITS ETF INC-Euro (hedged)</t>
+          <t>Fidelity US Fundamental Small-Mid Cap UCITS ETF ACC-USD</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>FFGE.MI</t>
+          <t>FFSM.MI</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>Fidelity Global HY Corp Bond Research Enhanced PAB UCITS ETF INC-USD</t>
+          <t>Fidelity US Quality Income UCITS ETF ACC-Euro (hedged)</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>FGHY.MI</t>
+          <t>FUSU.MI</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>Fidelity Global HY Corp Bond Research Enhanced PAB UCITS ETF INC-USD (hedged)</t>
+          <t>Fidelity US Quality Income UCITS ETF ACC-GBP (hedged)</t>
         </is>
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>FGHU.SW</t>
+          <t>FUSP.L</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>Fidelity Japan Equity Research Enhanced UCITS ETF ACC-JPY</t>
+          <t>Fidelity US Quality Income UCITS ETF ACC-USD</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>FJPR.MI</t>
+          <t>FUSA.MI</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>Fidelity Japan Equity Research Enhanced UCITS ETF INC-JPY</t>
+          <t>Fidelity US Quality Income UCITS ETF INC-USD</t>
         </is>
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>FJPI.SW</t>
+          <t>FUSD.MI</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>Fidelity Pacific ex-Japan Equity Research Enhanced UCITS ETF ACC-USD</t>
+          <t>Fidelity USD Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>FPXR.MI</t>
+          <t>FUIP.L</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>Fidelity Physical Bitcoin ETP</t>
+          <t>Fidelity USD Corporate Bond Research Enhanced UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>FBTC.MI</t>
+          <t>FBIU.MI</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>Fidelity US Equity Research Enhanced UCITS ETF ACC-USD</t>
+          <t>Fidelity USD Corporate Bond Research Enhanced UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>FUSR.MI</t>
+          <t>FBIH.MI</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>Fidelity US Equity Research Enhanced UCITS ETF EUR Hedged Acc</t>
+          <t>Fidelity USD HY Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>FUSE.MI</t>
+          <t>FYUP.L</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>Fidelity US Fundamental Large Cap Core UCITS ETF ACC-USD</t>
+          <t>Fidelity USD HY Corp Bond Research Enhanced PAB UCITS ETF INC-USD</t>
         </is>
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>FFLC.MI</t>
+          <t>FYUI.SW</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>Fidelity US Fundamental Small-Mid Cap UCITS ETF ACC-USD</t>
+          <t>First Trust Bloomberg Artificial Intelligence UCITS ETF Class A Accumulation</t>
         </is>
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>FFSM.MI</t>
+          <t>FTAI.MI</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>Fidelity US Quality Income UCITS ETF ACC-Euro (hedged)</t>
+          <t>First Trust Bloomberg Scarce Resources UCITS ETF Class A Accumulation</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>FUSU.MI</t>
+          <t>SCAR.MI</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>Fidelity US Quality Income UCITS ETF ACC-GBP (hedged)</t>
+          <t>First Trust Capital Strength UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>FUSP.L</t>
+          <t>FTCS.L</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>Fidelity US Quality Income UCITS ETF ACC-USD</t>
+          <t>First Trust FactorFX UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>FUSA.MI</t>
+          <t>FTFX.L</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>Fidelity US Quality Income UCITS ETF INC-USD</t>
+          <t>First Trust FactorFX UCITS ETF EUR Hedged Acc</t>
         </is>
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>FUSD.MI</t>
+          <t>FXEU.AS</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>Fidelity USD Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
+          <t>First Trust FactorFX UCITS ETF GBP Hedged Acc</t>
         </is>
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>FUIP.L</t>
+          <t>FXGB.L</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>Fidelity USD Corp Bond Research Enhanced PAB UCITS ETF INC-Euro (hedged)</t>
+          <t>First Trust Global Capital Strength ESG Leaders UCITS ETF Class A Accumulation</t>
         </is>
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>FUIE.MI</t>
+          <t>FCSG.AS</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>Fidelity USD Corp Bond Research Enhanced PAB UCITS ETF INC-USD</t>
+          <t>First Trust Global Equity Income UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>FUIG.MI</t>
+          <t>FGBL.PA</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>Fidelity USD Corporate Bond Research Enhanced UCITS ETF Acc</t>
+          <t>First Trust Global Equity Income UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>FBIU.MI</t>
+          <t>GINC.AS</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>Fidelity USD Corporate Bond Research Enhanced UCITS ETF EUR Hedged Acc</t>
+          <t>First Trust Indxx Future Economy Metals UCITS ETF Class A Accumulation</t>
         </is>
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>FBIH.MI</t>
+          <t>MINR.MI</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>Fidelity USD HY Corp Bond Research Enhanced PAB UCITS ETF ACC-GBP (hedged)</t>
+          <t>First Trust Indxx Innovative Transaction &amp; Process UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>FYUP.L</t>
+          <t>BLOK.MI</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>Fidelity USD HY Corp Bond Research Enhanced PAB UCITS ETF INC-USD</t>
+          <t>First Trust NYSE Arca Biotechnology UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>FYUI.SW</t>
+          <t>FBT.MI</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>First Trust Bloomberg Artificial Intelligence UCITS ETF Class A Accumulation</t>
+          <t>First Trust Rising Dividend Achievers UCITS ETF Class A Accumulation</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>FTAI.MI</t>
+          <t>RDVY.AS</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>First Trust Bloomberg Scarce Resources UCITS ETF Class A Accumulation</t>
+          <t>First Trust SMID Rising Dividend Achievers UCITS ETF Class A Accumulation</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>SCAR.MI</t>
+          <t>SDVY.MI</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>First Trust Capital Strength UCITS ETF Acc</t>
+          <t>First Trust SMID Rising Dividend Achievers UCITS ETF Class B Distribution</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>FTCS.L</t>
+          <t>SDVI.L</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>First Trust FactorFX UCITS ETF Acc</t>
+          <t>First Trust US Equity Income UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>FTFX.L</t>
+          <t>UNCA.MI</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>First Trust FactorFX UCITS ETF EUR Hedged Acc</t>
+          <t>First Trust US Equity Income UCITS ETF Dist</t>
         </is>
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>FXEU.AS</t>
+          <t>UINC.L</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>First Trust FactorFX UCITS ETF GBP Hedged Acc</t>
+          <t>HSBC MSCI Emerging Markets UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>FXGB.L</t>
+          <t>HEMA.PA</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
         <is>
-          <t>First Trust Global Capital Strength ESG Leaders UCITS ETF Class A Accumulation</t>
+          <t>iShares EUR Cash UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>FCSG.AS</t>
+          <t>YCSH.AS</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>First Trust Global Equity Income UCITS ETF Acc</t>
+          <t>Xtrackers MSCI Nordic UCITS ETF 1D</t>
         </is>
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>FGBL.PA</t>
+          <t>XDN0.SW</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>First Trust Global Equity Income UCITS ETF Dist</t>
+          <t>JPMorgan US Research Enhanced Index Equity Active UCITS ETF EUR Hedged (acc)</t>
         </is>
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>GINC.AS</t>
+          <t>JUHE.MI</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>First Trust Indxx Future Economy Metals UCITS ETF Class A Accumulation</t>
+          <t>iShares iBonds Dec 2028 Term EUR Corporate UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>MINR.MI</t>
+          <t>B28A.PA</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>First Trust Indxx Innovative Transaction &amp; Process UCITS ETF Acc</t>
+          <t>Invesco S&amp;P 500 Equal Weight UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>BLOK.MI</t>
+          <t>SPEQ.MI</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
         <is>
-          <t>First Trust NYSE Arca Biotechnology UCITS ETF Acc</t>
+          <t>Xtrackers S&amp;P 500 Equal Weight Scored &amp; Screened UCITS ETF 2C - EUR Hedged</t>
         </is>
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>FBT.MI</t>
+          <t>XEWE.MI</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
         <is>
-          <t>First Trust Rising Dividend Achievers UCITS ETF Class A Accumulation</t>
+          <t>UBS Core MSCI World UCITS ETF hCHF acc</t>
         </is>
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>RDVY.AS</t>
+          <t>WORLD.SW</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t>First Trust SMID Rising Dividend Achievers UCITS ETF Class A Accumulation</t>
+          <t>Schroder Global Equity Active UCITS ETF</t>
         </is>
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>SDVY.MI</t>
+          <t>SAGE.MI</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
         <is>
-          <t>First Trust SMID Rising Dividend Achievers UCITS ETF Class B Distribution</t>
+          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
         </is>
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>SDVI.L</t>
+          <t>SXLE.AS</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>First Trust US Equity Income UCITS ETF Acc</t>
+          <t>iShares STOXX Europe 600 Utilities UCITS ETF (DE)</t>
         </is>
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>UNCA.MI</t>
+          <t>SX6PEX.SW</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>First Trust US Equity Income UCITS ETF Dist</t>
+          <t>iShares European Property Yield UCITS ETF</t>
         </is>
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>UINC.L</t>
+          <t>IPRP.AS</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>HSBC MSCI Emerging Markets UCITS ETF USD (Acc)</t>
+          <t>Invesco CoinShares Global Blockchain UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>HEMA.PA</t>
+          <t>BCHN.MI</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>iShares EUR Cash UCITS ETF EUR (Acc)</t>
+          <t>Global X Copper Miners UCITS ETF USD Accumulating</t>
         </is>
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>YCSH.AS</t>
+          <t>COPX.MI</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Nordic UCITS ETF 1D</t>
+          <t>UBS S&amp;P 500 Scored &amp; Screened UCITS ETF hEUR acc</t>
         </is>
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>XDN0.SW</t>
+          <t>5ESGE.MI</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>JPMorgan US Research Enhanced Index Equity Active UCITS ETF EUR Hedged (acc)</t>
+          <t>iShares MSCI Korea UCITS ETF (Dist)</t>
         </is>
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>JUHE.MI</t>
+          <t>IKRA.AS</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2028 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+          <t>Xtrackers MSCI World Minimum Volatility UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>B28A.PA</t>
+          <t>XDEB.MI</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
-          <t>Invesco S&amp;P 500 Equal Weight UCITS ETF Acc</t>
+          <t>JPMorgan Global Research Enhanced Index Equity (ESG) UCITS ETF EUR Hedged (acc)</t>
         </is>
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>SPEQ.MI</t>
+          <t>JRGE.MI</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" t="inlineStr">
         <is>
-          <t>Xtrackers S&amp;P 500 Equal Weight Scored &amp; Screened UCITS ETF 2C - EUR Hedged</t>
+          <t>UBS MSCI AC Asia ex Japan SF UCITS ETF USD acc</t>
         </is>
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>XEWE.MI</t>
+          <t>AJEUAS.MI</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>UBS Core MSCI World UCITS ETF hCHF acc</t>
+          <t>Invesco S&amp;P 500 Equal Weight Swap UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>WORLD.SW</t>
+          <t>RSPS.MI</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>Schroder Global Equity Active UCITS ETF</t>
+          <t>L&amp;G Battery Value-Chain UCITS ETF</t>
         </is>
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>SAGE.MI</t>
+          <t>BATT.AS</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
         <is>
-          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
+          <t>iShares MSCI Europe Quality Dividend Advanced UCITS ETF EUR (Dist)</t>
         </is>
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>SXLE.AS</t>
+          <t>QDVX.SW</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>iShares STOXX Europe 600 Utilities UCITS ETF (DE)</t>
+          <t>iShares MSCI Europe Health Care Sector UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>SX6PEX.SW</t>
+          <t>ESIH.L</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>iShares European Property Yield UCITS ETF</t>
+          <t>HSBC Multi-Factor Worldwide Equity UCITS ETF USD</t>
         </is>
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>IPRP.AS</t>
+          <t>HWWA.L</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>Invesco CoinShares Global Blockchain UCITS ETF Acc</t>
+          <t>Xtrackers MSCI Japan UCITS ETF 4C - EUR Hedged</t>
         </is>
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>BCHN.MI</t>
+          <t>XMK9.MI</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>Global X Copper Miners UCITS ETF USD Accumulating</t>
+          <t>iShares EUR Floating Rate Bond Advanced UCITS ETF EUR (Dist)</t>
         </is>
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>COPX.MI</t>
+          <t>EFRN.SW</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>UBS S&amp;P 500 Scored &amp; Screened UCITS ETF hEUR acc</t>
+          <t>iShares iBonds Dec 2027 Term EUR Corporate UCITS ETF EUR (Acc)</t>
         </is>
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>5ESGE.MI</t>
+          <t>IB27.PA</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>iShares MSCI Korea UCITS ETF (Dist)</t>
+          <t>PIMCO Euro Short Maturity UCITS ETF Acc</t>
         </is>
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>IKRA.AS</t>
+          <t>PJSR.MI</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Minimum Volatility UCITS ETF 1C</t>
+          <t>Xtrackers MSCI Emerging Markets Swap UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>XDEB.MI</t>
+          <t>XMEM.MI</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>JPMorgan Global Research Enhanced Index Equity (ESG) UCITS ETF EUR Hedged (acc)</t>
+          <t>Vanguard ESG Global All Cap UCITS ETF (USD) Accumulating</t>
         </is>
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>JRGE.MI</t>
+          <t>V3AA.AS</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>UBS MSCI AC Asia ex Japan SF UCITS ETF USD acc</t>
+          <t>State Street SPDR MSCI Japan UCITS ETF JPY Unhedged</t>
         </is>
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>AJEUAS.MI</t>
+          <t>JPJY.PA</t>
         </is>
       </c>
     </row>
     <row r="521">
       <c r="A521" t="inlineStr">
         <is>
-          <t>Invesco S&amp;P 500 Equal Weight Swap UCITS ETF Acc</t>
+          <t>Xtrackers MSCI World Utilities UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>RSPS.MI</t>
+          <t>XDWU.MI</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" t="inlineStr">
         <is>
-          <t>L&amp;G Battery Value-Chain UCITS ETF</t>
+          <t>Xtrackers MSCI USA Communication Services UCITS ETF 1D</t>
         </is>
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>BATT.AS</t>
+          <t>XUCM.L</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>iShares MSCI Europe Quality Dividend Advanced UCITS ETF EUR (Dist)</t>
+          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>QDVX.SW</t>
+          <t>EXCD.AS</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
         <is>
-          <t>iShares MSCI Europe Health Care Sector UCITS ETF EUR (Acc)</t>
+          <t>iShares Edge MSCI Europe Minimum Volatility UCITS ETF</t>
         </is>
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>ESIH.L</t>
+          <t>MVEU.MI</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" t="inlineStr">
         <is>
-          <t>HSBC Multi-Factor Worldwide Equity UCITS ETF USD</t>
+          <t>iShares AI Infrastructure UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>HWWA.L</t>
+          <t>AINF.AS</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Japan UCITS ETF 4C - EUR Hedged</t>
+          <t>Vanguard LifeStrategy 60% Equity UCITS ETF Accumulating</t>
         </is>
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>XMK9.MI</t>
+          <t>V60A.AS</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" t="inlineStr">
         <is>
-          <t>iShares EUR Floating Rate Bond Advanced UCITS ETF EUR (Dist)</t>
+          <t>Xtrackers MSCI World Consumer Staples UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>EFRN.SW</t>
+          <t>XDWS.MI</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2027 Term EUR Corporate UCITS ETF EUR (Acc)</t>
+          <t>iShares USD High Yield Corporate Bond ESG SRI UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>IB27.PA</t>
+          <t>DHYE.AS</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" t="inlineStr">
         <is>
-          <t>PIMCO Euro Short Maturity UCITS ETF Acc</t>
+          <t>iShares Russell 1000 Growth UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>PJSR.MI</t>
+          <t>R1GR.AS</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Emerging Markets Swap UCITS ETF 1C</t>
+          <t>State Street SPDR MSCI Europe Utilities UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>XMEM.MI</t>
+          <t>STU.PA</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" t="inlineStr">
         <is>
-          <t>Vanguard ESG Global All Cap UCITS ETF (USD) Accumulating</t>
+          <t>iShares MSCI World Information Technology Sector Advanced UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>V3AA.AS</t>
+          <t>WITS.AS</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Japan UCITS ETF JPY Unhedged</t>
+          <t>HSBC MSCI Pacific ex Japan UCITS ETF USD</t>
         </is>
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>JPJY.PA</t>
+          <t>HMXJ.MI</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Utilities UCITS ETF 1C</t>
+          <t>UBS BBG Commodity CMCI SF UCITS ETF USD acc</t>
         </is>
       </c>
       <c r="B533" t="inlineStr">
         <is>
-          <t>XDWU.MI</t>
+          <t>BCCMA.SW</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI USA Communication Services UCITS ETF 1D</t>
+          <t>iShares FTSE 250 UCITS ETF</t>
         </is>
       </c>
       <c r="B534" t="inlineStr">
         <is>
-          <t>XUCM.L</t>
+          <t>MIDD.SW</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" t="inlineStr">
         <is>
-          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
+          <t>UBS Core MSCI EMU UCITS ETF hCHF acc</t>
         </is>
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>EXCD.AS</t>
+          <t>EMUCHF.SW</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI Europe Minimum Volatility UCITS ETF</t>
+          <t>iShares MSCI USA Screened UCITS ETF EUR Hedged (Acc)</t>
         </is>
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>MVEU.MI</t>
+          <t>SAUA.MI</t>
         </is>
       </c>
     </row>
     <row r="537">
       <c r="A537" t="inlineStr">
         <is>
-          <t>iShares AI Infrastructure UCITS ETF USD (Acc)</t>
+          <t>Xtrackers MSCI World Financials UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>AINF.AS</t>
+          <t>XDWF.MI</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" t="inlineStr">
         <is>
-          <t>Vanguard LifeStrategy 60% Equity UCITS ETF Accumulating</t>
+          <t>State Street SPDR Bloomberg 1-3 Month T-Bill UCITS ETF USD Unhedged (Acc)</t>
         </is>
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>V60A.AS</t>
+          <t>TBIL.SW</t>
         </is>
       </c>
     </row>
     <row r="539">
       <c r="A539" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Consumer Staples UCITS ETF 1C</t>
+          <t>JPMorgan USD Ultra-Short Income UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>XDWS.MI</t>
+          <t>JPSA.MI</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
         <is>
-          <t>iShares USD High Yield Corporate Bond ESG SRI UCITS ETF USD (Acc)</t>
+          <t>Invesco MDAX UCITS ETF A</t>
         </is>
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>DHYE.AS</t>
+          <t>MDAX.MI</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
         <is>
-          <t>iShares Russell 1000 Growth UCITS ETF USD (Acc)</t>
+          <t>HSBC FTSE EPRA NAREIT Developed UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>R1GR.AS</t>
+          <t>HPRA.L</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Europe Utilities UCITS ETF EUR</t>
+          <t>JPMorgan EUR Corporate Bond Research Enhanced Index (ESG) UCITS ETF</t>
         </is>
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>STU.PA</t>
+          <t>JREB.MI</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="A543" t="inlineStr">
         <is>
-          <t>iShares MSCI World Information Technology Sector Advanced UCITS ETF USD (Dist)</t>
+          <t>Xtrackers MSCI USA Health Care UCITS ETF 1D</t>
         </is>
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>WITS.AS</t>
+          <t>XUHC.SW</t>
         </is>
       </c>
     </row>
     <row r="544">
       <c r="A544" t="inlineStr">
         <is>
-          <t>HSBC MSCI Pacific ex Japan UCITS ETF USD</t>
+          <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
         </is>
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>HMXJ.MI</t>
+          <t>VAPU.SW</t>
         </is>
       </c>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
         <is>
-          <t>UBS BBG Commodity CMCI SF UCITS ETF USD acc</t>
+          <t>iShares Core MSCI EMU UCITS ETF USD Hedged (Acc)</t>
         </is>
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>BCCMA.SW</t>
+          <t>CEUU.AS</t>
         </is>
       </c>
     </row>
     <row r="546">
       <c r="A546" t="inlineStr">
         <is>
-          <t>iShares FTSE 250 UCITS ETF</t>
+          <t>State Street SPDR MSCI World UCITS ETF EUR Hedged (Acc)</t>
         </is>
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>MIDD.SW</t>
+          <t>SWRE.MI</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">
         <is>
-          <t>UBS Core MSCI EMU UCITS ETF hCHF acc</t>
+          <t>Xtrackers Swiss Large Cap UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B547" t="inlineStr">
         <is>
-          <t>EMUCHF.SW</t>
+          <t>XSMC.SW</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" t="inlineStr">
         <is>
-          <t>iShares MSCI USA Screened UCITS ETF EUR Hedged (Acc)</t>
+          <t>UBS Core MSCI World UCITS ETF hEUR acc</t>
         </is>
       </c>
       <c r="B548" t="inlineStr">
         <is>
-          <t>SAUA.MI</t>
+          <t>WRDE.MI</t>
         </is>
       </c>
     </row>
     <row r="549">
       <c r="A549" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Financials UCITS ETF 1C</t>
+          <t>UBS Core MSCI USA UCITS ETF EUR Hedged acc</t>
         </is>
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>XDWF.MI</t>
+          <t>USEUWH.MI</t>
         </is>
       </c>
     </row>
     <row r="550">
       <c r="A550" t="inlineStr">
         <is>
-          <t>State Street SPDR Bloomberg 1-3 Month T-Bill UCITS ETF USD Unhedged (Acc)</t>
+          <t>UBS MSCI World Selection UCITS ETF USD acc</t>
         </is>
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>TBIL.SW</t>
+          <t>WDESG.MI</t>
         </is>
       </c>
     </row>
     <row r="551">
       <c r="A551" t="inlineStr">
         <is>
-          <t>JPMorgan USD Ultra-Short Income UCITS ETF USD (Acc)</t>
+          <t>Xtrackers MSCI UK ESG UCITS ETF 1D</t>
         </is>
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>JPSA.MI</t>
+          <t>XASX.L</t>
         </is>
       </c>
     </row>
     <row r="552">
       <c r="A552" t="inlineStr">
         <is>
-          <t>Invesco MDAX UCITS ETF A</t>
+          <t>iShares Edge MSCI Europe Quality Factor UCITS ETF</t>
         </is>
       </c>
       <c r="B552" t="inlineStr">
         <is>
-          <t>MDAX.MI</t>
+          <t>IEQU.MI</t>
         </is>
       </c>
     </row>
     <row r="553">
       <c r="A553" t="inlineStr">
         <is>
-          <t>HSBC FTSE EPRA NAREIT Developed UCITS ETF USD (Acc)</t>
+          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>HPRA.L</t>
+          <t>STN.PA</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" t="inlineStr">
         <is>
-          <t>JPMorgan EUR Corporate Bond Research Enhanced Index (ESG) UCITS ETF</t>
+          <t>Xtrackers Portfolio UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>JREB.MI</t>
+          <t>XQUI.MI</t>
         </is>
       </c>
     </row>
     <row r="555">
       <c r="A555" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI USA Health Care UCITS ETF 1D</t>
+          <t>State Street SPDR MSCI Europe Financials UCITS ETF EUR</t>
         </is>
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>XUHC.SW</t>
+          <t>STZ.PA</t>
         </is>
       </c>
     </row>
     <row r="556">
       <c r="A556" t="inlineStr">
         <is>
-          <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
+          <t>iShares S&amp;P 500 Consumer Discretionary Sector UCITS ETF (Acc)</t>
         </is>
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>VAPU.SW</t>
+          <t>IUCD.SW</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" t="inlineStr">
         <is>
-          <t>iShares Core MSCI EMU UCITS ETF USD Hedged (Acc)</t>
+          <t>Vanguard FTSE 250 UCITS ETF (GBP) Accumulating</t>
         </is>
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>CEUU.AS</t>
+          <t>VMIG.MI</t>
         </is>
       </c>
     </row>
     <row r="558">
       <c r="A558" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI World UCITS ETF EUR Hedged (Acc)</t>
+          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
         </is>
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t>SWRE.MI</t>
+          <t>BTEC.SW</t>
         </is>
       </c>
     </row>
     <row r="559">
       <c r="A559" t="inlineStr">
         <is>
-          <t>Xtrackers Swiss Large Cap UCITS ETF 1C</t>
+          <t>State Street SPDR S&amp;P 500 Quality Aristocrats UCITS ETF USD Unhedged (Acc)</t>
         </is>
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>XSMC.SW</t>
+          <t>QUS5.SW</t>
         </is>
       </c>
     </row>
     <row r="560">
       <c r="A560" t="inlineStr">
         <is>
-          <t>UBS Core MSCI World UCITS ETF hEUR acc</t>
+          <t>iShares MSCI Poland UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B560" t="inlineStr">
-        <is>
-          <t>WRDE.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="561">
-      <c r="A561" t="inlineStr">
-        <is>
-          <t>UBS Core MSCI USA UCITS ETF EUR Hedged acc</t>
-        </is>
-      </c>
-      <c r="B561" t="inlineStr">
-        <is>
-          <t>USEUWH.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="562">
-      <c r="A562" t="inlineStr">
-        <is>
-          <t>UBS MSCI World Selection UCITS ETF USD acc</t>
-        </is>
-      </c>
-      <c r="B562" t="inlineStr">
-        <is>
-          <t>WDESG.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="563">
-      <c r="A563" t="inlineStr">
-        <is>
-          <t>Xtrackers MSCI UK ESG UCITS ETF 1D</t>
-        </is>
-      </c>
-      <c r="B563" t="inlineStr">
-        <is>
-          <t>XASX.L</t>
-        </is>
-      </c>
-    </row>
-    <row r="564">
-      <c r="A564" t="inlineStr">
-        <is>
-          <t>iShares Edge MSCI Europe Quality Factor UCITS ETF</t>
-        </is>
-      </c>
-      <c r="B564" t="inlineStr">
-        <is>
-          <t>IEQU.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="565">
-      <c r="A565" t="inlineStr">
-        <is>
-          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
-        </is>
-      </c>
-      <c r="B565" t="inlineStr">
-        <is>
-          <t>STN.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="566">
-      <c r="A566" t="inlineStr">
-        <is>
-          <t>Xtrackers Portfolio UCITS ETF 1C</t>
-        </is>
-      </c>
-      <c r="B566" t="inlineStr">
-        <is>
-          <t>XQUI.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="567">
-      <c r="A567" t="inlineStr">
-        <is>
-          <t>State Street SPDR MSCI Europe Financials UCITS ETF EUR</t>
-        </is>
-      </c>
-      <c r="B567" t="inlineStr">
-        <is>
-          <t>STZ.PA</t>
-        </is>
-      </c>
-    </row>
-    <row r="568">
-      <c r="A568" t="inlineStr">
-        <is>
-          <t>iShares S&amp;P 500 Consumer Discretionary Sector UCITS ETF (Acc)</t>
-        </is>
-      </c>
-      <c r="B568" t="inlineStr">
-        <is>
-          <t>IUCD.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="569">
-      <c r="A569" t="inlineStr">
-        <is>
-          <t>Vanguard FTSE 250 UCITS ETF (GBP) Accumulating</t>
-        </is>
-      </c>
-      <c r="B569" t="inlineStr">
-        <is>
-          <t>VMIG.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="570">
-      <c r="A570" t="inlineStr">
-        <is>
-          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
-        </is>
-      </c>
-      <c r="B570" t="inlineStr">
-        <is>
-          <t>BTEC.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="571">
-      <c r="A571" t="inlineStr">
-        <is>
-          <t>State Street SPDR S&amp;P 500 Quality Aristocrats UCITS ETF USD Unhedged (Acc)</t>
-        </is>
-      </c>
-      <c r="B571" t="inlineStr">
-        <is>
-          <t>QUS5.SW</t>
-        </is>
-      </c>
-    </row>
-    <row r="572">
-      <c r="A572" t="inlineStr">
-        <is>
-          <t>iShares MSCI Poland UCITS ETF USD (Acc)</t>
-        </is>
-      </c>
-      <c r="B572" t="inlineStr">
         <is>
           <t>SPOL.SW</t>
         </is>

</xml_diff>